<commit_message>
docs: avancement du rapport et des diagrammes UML
Ajout de la journée du 12.05 au journal de travail.
</commit_message>
<xml_diff>
--- a/doc/GAMEZ_Journal.xlsx
+++ b/doc/GAMEZ_Journal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/thibaudfrederic_gamez_studentfr_ch/Documents/TPI/tpi2026-codementor/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABB02B47-4CF3-4A0F-8D30-4B356D7B79EE}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58766AB4-7609-4881-B248-B038BF3DA048}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,42 +36,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="20">
   <si>
     <t>Insérer les lignes au-dessus de celle-ci !</t>
-  </si>
-  <si>
-    <r>
-      <t>Projet :</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">[Titre du projet]      </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">                      </t>
-    </r>
-  </si>
-  <si>
-    <t>[Nom Prénom du candidat]</t>
   </si>
   <si>
     <t>Date</t>
@@ -104,6 +71,69 @@
   <si>
     <t>Total général &gt;</t>
   </si>
+  <si>
+    <r>
+      <t>Projet :</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>CodeMentor</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">                      </t>
+    </r>
+  </si>
+  <si>
+    <t>Gamez Thibaud</t>
+  </si>
+  <si>
+    <t>Lecture cahier des charges et préparation</t>
+  </si>
+  <si>
+    <t>Planning</t>
+  </si>
+  <si>
+    <t>Documentation des technos et cahier des charges</t>
+  </si>
+  <si>
+    <t>Préparation de la réunion et réunion</t>
+  </si>
+  <si>
+    <t>Rédaction du PV et envoie</t>
+  </si>
+  <si>
+    <t>Création du diagramme usecase</t>
+  </si>
+  <si>
+    <t>Travail sur le diagramme de séquence système</t>
+  </si>
+  <si>
+    <t>Début du TPI, j'ai pris plus de temps que prévu pour le planning et la documentation</t>
+  </si>
+  <si>
+    <t>diagramme ER de base de données</t>
+  </si>
+  <si>
+    <t>Second jour, j'ai pu rattraper un peu le retard en avancant plus vite que prévu sur le diagramme ER et le usecase</t>
+  </si>
 </sst>
 </file>
 
@@ -113,7 +143,7 @@
     <numFmt numFmtId="164" formatCode="dd/mm/yy;@"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -173,6 +203,11 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -399,7 +434,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -448,6 +483,13 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -484,6 +526,10 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
@@ -496,81 +542,51 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="22">
     <dxf>
       <font>
         <strike val="0"/>
@@ -824,6 +840,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1185,178 +1205,217 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
+      <c r="A1" s="28" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
     </row>
     <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="34" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="35"/>
+      <c r="A2" s="35" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="35"/>
+      <c r="C2" s="36"/>
       <c r="D2" s="4">
         <v>151446</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="29" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="30"/>
+      <c r="D4" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="31"/>
+      <c r="B5" s="31"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="28" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="29"/>
-      <c r="D4" s="5" t="s">
+    </row>
+    <row r="6" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="37">
+        <v>46153</v>
+      </c>
+      <c r="B6" s="33" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="34"/>
+      <c r="D6" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="16"/>
+      <c r="B7" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="20"/>
+      <c r="D7" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="16"/>
+      <c r="B8" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="20"/>
+      <c r="D8" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="16"/>
+      <c r="B9" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="20"/>
+      <c r="D9" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="16"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="8"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="16"/>
+      <c r="B11" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="30"/>
-      <c r="B5" s="30"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="6" t="s">
+      <c r="C11" s="3" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="26"/>
-      <c r="B6" s="32"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="7"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="14"/>
-      <c r="B7" s="17"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="8"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="14"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="8"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="14"/>
-      <c r="B9" s="17"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="8"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="14"/>
-      <c r="B10" s="17"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="8"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="14"/>
-      <c r="B11" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>7</v>
       </c>
       <c r="D11" s="9">
         <f>SUM(D6:D10)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="14"/>
-      <c r="B12" s="19"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="21"/>
+      <c r="A12" s="16"/>
+      <c r="B12" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="22"/>
+      <c r="D12" s="23"/>
     </row>
     <row r="13" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="13"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="7"/>
+      <c r="A13" s="15">
+        <v>46154</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="18"/>
+      <c r="D13" s="7">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="14"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="8"/>
+      <c r="A14" s="16"/>
+      <c r="B14" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="20"/>
+      <c r="D14" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="14"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="8"/>
+      <c r="A15" s="16"/>
+      <c r="B15" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="14"/>
-      <c r="B16" s="17"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="8"/>
+      <c r="A16" s="16"/>
+      <c r="B16" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="20"/>
+      <c r="D16" s="8">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="14"/>
-      <c r="B17" s="17"/>
-      <c r="C17" s="18"/>
+      <c r="A17" s="16"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="20"/>
       <c r="D17" s="8"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="14"/>
+      <c r="A18" s="16"/>
       <c r="B18" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D18" s="9">
         <f>SUM(D13:D17)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="14"/>
-      <c r="B19" s="19"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="21"/>
+      <c r="A19" s="16"/>
+      <c r="B19" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="22"/>
+      <c r="D19" s="23"/>
     </row>
     <row r="20" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="13"/>
-      <c r="B20" s="15"/>
-      <c r="C20" s="16"/>
+      <c r="A20" s="15"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="18"/>
       <c r="D20" s="7"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="14"/>
-      <c r="B21" s="17"/>
-      <c r="C21" s="18"/>
+      <c r="A21" s="16"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="20"/>
       <c r="D21" s="8"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="14"/>
-      <c r="B22" s="17"/>
-      <c r="C22" s="18"/>
+      <c r="A22" s="16"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="20"/>
       <c r="D22" s="8"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="14"/>
-      <c r="B23" s="17"/>
-      <c r="C23" s="18"/>
+      <c r="A23" s="16"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="20"/>
       <c r="D23" s="8"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="14"/>
-      <c r="B24" s="17"/>
-      <c r="C24" s="18"/>
+      <c r="A24" s="16"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="20"/>
       <c r="D24" s="8"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="14"/>
+      <c r="A25" s="16"/>
       <c r="B25" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D25" s="9">
         <f>SUM(D20:D24)</f>
@@ -1364,48 +1423,48 @@
       </c>
     </row>
     <row r="26" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="14"/>
-      <c r="B26" s="19"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="21"/>
+      <c r="A26" s="16"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="23"/>
     </row>
     <row r="27" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="13"/>
-      <c r="B27" s="15"/>
-      <c r="C27" s="16"/>
+      <c r="A27" s="15"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="18"/>
       <c r="D27" s="7"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="14"/>
-      <c r="B28" s="17"/>
-      <c r="C28" s="18"/>
+      <c r="A28" s="16"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="20"/>
       <c r="D28" s="8"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="14"/>
-      <c r="B29" s="17"/>
-      <c r="C29" s="18"/>
+      <c r="A29" s="16"/>
+      <c r="B29" s="19"/>
+      <c r="C29" s="20"/>
       <c r="D29" s="8"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="14"/>
-      <c r="B30" s="17"/>
-      <c r="C30" s="18"/>
+      <c r="A30" s="16"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="20"/>
       <c r="D30" s="8"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="14"/>
-      <c r="B31" s="17"/>
-      <c r="C31" s="18"/>
+      <c r="A31" s="16"/>
+      <c r="B31" s="19"/>
+      <c r="C31" s="20"/>
       <c r="D31" s="8"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="14"/>
+      <c r="A32" s="16"/>
       <c r="B32" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D32" s="9">
         <f>SUM(D27:D31)</f>
@@ -1413,48 +1472,48 @@
       </c>
     </row>
     <row r="33" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="25"/>
-      <c r="B33" s="22"/>
-      <c r="C33" s="23"/>
-      <c r="D33" s="24"/>
+      <c r="A33" s="24"/>
+      <c r="B33" s="25"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="27"/>
     </row>
     <row r="34" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="13"/>
-      <c r="B34" s="15"/>
-      <c r="C34" s="16"/>
+      <c r="A34" s="15"/>
+      <c r="B34" s="17"/>
+      <c r="C34" s="18"/>
       <c r="D34" s="7"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="14"/>
-      <c r="B35" s="17"/>
-      <c r="C35" s="18"/>
+      <c r="A35" s="16"/>
+      <c r="B35" s="19"/>
+      <c r="C35" s="20"/>
       <c r="D35" s="8"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="14"/>
-      <c r="B36" s="17"/>
-      <c r="C36" s="18"/>
+      <c r="A36" s="16"/>
+      <c r="B36" s="19"/>
+      <c r="C36" s="20"/>
       <c r="D36" s="8"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="14"/>
-      <c r="B37" s="17"/>
-      <c r="C37" s="18"/>
+      <c r="A37" s="16"/>
+      <c r="B37" s="19"/>
+      <c r="C37" s="20"/>
       <c r="D37" s="8"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="14"/>
-      <c r="B38" s="17"/>
-      <c r="C38" s="18"/>
+      <c r="A38" s="16"/>
+      <c r="B38" s="19"/>
+      <c r="C38" s="20"/>
       <c r="D38" s="8"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="14"/>
+      <c r="A39" s="16"/>
       <c r="B39" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D39" s="9">
         <f>SUM(D34:D38)</f>
@@ -1462,48 +1521,48 @@
       </c>
     </row>
     <row r="40" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="25"/>
-      <c r="B40" s="22"/>
-      <c r="C40" s="23"/>
-      <c r="D40" s="24"/>
+      <c r="A40" s="24"/>
+      <c r="B40" s="25"/>
+      <c r="C40" s="26"/>
+      <c r="D40" s="27"/>
     </row>
     <row r="41" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="13"/>
-      <c r="B41" s="15"/>
-      <c r="C41" s="16"/>
+      <c r="A41" s="15"/>
+      <c r="B41" s="17"/>
+      <c r="C41" s="18"/>
       <c r="D41" s="7"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="14"/>
-      <c r="B42" s="17"/>
-      <c r="C42" s="18"/>
+      <c r="A42" s="16"/>
+      <c r="B42" s="19"/>
+      <c r="C42" s="20"/>
       <c r="D42" s="8"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="14"/>
-      <c r="B43" s="17"/>
-      <c r="C43" s="18"/>
+      <c r="A43" s="16"/>
+      <c r="B43" s="19"/>
+      <c r="C43" s="20"/>
       <c r="D43" s="8"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="14"/>
-      <c r="B44" s="17"/>
-      <c r="C44" s="18"/>
+      <c r="A44" s="16"/>
+      <c r="B44" s="19"/>
+      <c r="C44" s="20"/>
       <c r="D44" s="8"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="14"/>
-      <c r="B45" s="17"/>
-      <c r="C45" s="18"/>
+      <c r="A45" s="16"/>
+      <c r="B45" s="19"/>
+      <c r="C45" s="20"/>
       <c r="D45" s="8"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="14"/>
+      <c r="A46" s="16"/>
       <c r="B46" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D46" s="9">
         <f>SUM(D41:D45)</f>
@@ -1511,48 +1570,48 @@
       </c>
     </row>
     <row r="47" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="25"/>
-      <c r="B47" s="22"/>
-      <c r="C47" s="23"/>
-      <c r="D47" s="24"/>
+      <c r="A47" s="24"/>
+      <c r="B47" s="25"/>
+      <c r="C47" s="26"/>
+      <c r="D47" s="27"/>
     </row>
     <row r="48" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="13"/>
-      <c r="B48" s="15"/>
-      <c r="C48" s="16"/>
+      <c r="A48" s="15"/>
+      <c r="B48" s="17"/>
+      <c r="C48" s="18"/>
       <c r="D48" s="7"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="14"/>
-      <c r="B49" s="17"/>
-      <c r="C49" s="18"/>
+      <c r="A49" s="16"/>
+      <c r="B49" s="19"/>
+      <c r="C49" s="20"/>
       <c r="D49" s="8"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A50" s="14"/>
-      <c r="B50" s="17"/>
-      <c r="C50" s="18"/>
+      <c r="A50" s="16"/>
+      <c r="B50" s="19"/>
+      <c r="C50" s="20"/>
       <c r="D50" s="8"/>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A51" s="14"/>
-      <c r="B51" s="17"/>
-      <c r="C51" s="18"/>
+      <c r="A51" s="16"/>
+      <c r="B51" s="19"/>
+      <c r="C51" s="20"/>
       <c r="D51" s="8"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="14"/>
-      <c r="B52" s="17"/>
-      <c r="C52" s="18"/>
+      <c r="A52" s="16"/>
+      <c r="B52" s="19"/>
+      <c r="C52" s="20"/>
       <c r="D52" s="8"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="14"/>
+      <c r="A53" s="16"/>
       <c r="B53" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D53" s="9">
         <f>SUM(D48:D52)</f>
@@ -1560,48 +1619,48 @@
       </c>
     </row>
     <row r="54" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="25"/>
-      <c r="B54" s="22"/>
-      <c r="C54" s="23"/>
-      <c r="D54" s="24"/>
+      <c r="A54" s="24"/>
+      <c r="B54" s="25"/>
+      <c r="C54" s="26"/>
+      <c r="D54" s="27"/>
     </row>
     <row r="55" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="13"/>
-      <c r="B55" s="15"/>
-      <c r="C55" s="16"/>
+      <c r="A55" s="15"/>
+      <c r="B55" s="17"/>
+      <c r="C55" s="18"/>
       <c r="D55" s="7"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="14"/>
-      <c r="B56" s="17"/>
-      <c r="C56" s="18"/>
+      <c r="A56" s="16"/>
+      <c r="B56" s="19"/>
+      <c r="C56" s="20"/>
       <c r="D56" s="8"/>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" s="14"/>
-      <c r="B57" s="17"/>
-      <c r="C57" s="18"/>
+      <c r="A57" s="16"/>
+      <c r="B57" s="19"/>
+      <c r="C57" s="20"/>
       <c r="D57" s="8"/>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" s="14"/>
-      <c r="B58" s="17"/>
-      <c r="C58" s="18"/>
+      <c r="A58" s="16"/>
+      <c r="B58" s="19"/>
+      <c r="C58" s="20"/>
       <c r="D58" s="8"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A59" s="14"/>
-      <c r="B59" s="17"/>
-      <c r="C59" s="18"/>
+      <c r="A59" s="16"/>
+      <c r="B59" s="19"/>
+      <c r="C59" s="20"/>
       <c r="D59" s="8"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" s="14"/>
+      <c r="A60" s="16"/>
       <c r="B60" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D60" s="9">
         <f>SUM(D55:D59)</f>
@@ -1609,48 +1668,48 @@
       </c>
     </row>
     <row r="61" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="25"/>
-      <c r="B61" s="22"/>
-      <c r="C61" s="23"/>
-      <c r="D61" s="24"/>
+      <c r="A61" s="24"/>
+      <c r="B61" s="25"/>
+      <c r="C61" s="26"/>
+      <c r="D61" s="27"/>
     </row>
     <row r="62" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="13"/>
-      <c r="B62" s="15"/>
-      <c r="C62" s="16"/>
+      <c r="A62" s="15"/>
+      <c r="B62" s="17"/>
+      <c r="C62" s="18"/>
       <c r="D62" s="7"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="14"/>
-      <c r="B63" s="17"/>
-      <c r="C63" s="18"/>
+      <c r="A63" s="16"/>
+      <c r="B63" s="19"/>
+      <c r="C63" s="20"/>
       <c r="D63" s="8"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="14"/>
-      <c r="B64" s="17"/>
-      <c r="C64" s="18"/>
+      <c r="A64" s="16"/>
+      <c r="B64" s="19"/>
+      <c r="C64" s="20"/>
       <c r="D64" s="8"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" s="14"/>
-      <c r="B65" s="17"/>
-      <c r="C65" s="18"/>
+      <c r="A65" s="16"/>
+      <c r="B65" s="19"/>
+      <c r="C65" s="20"/>
       <c r="D65" s="8"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" s="14"/>
-      <c r="B66" s="17"/>
-      <c r="C66" s="18"/>
+      <c r="A66" s="16"/>
+      <c r="B66" s="19"/>
+      <c r="C66" s="20"/>
       <c r="D66" s="8"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="14"/>
+      <c r="A67" s="16"/>
       <c r="B67" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D67" s="9">
         <f>SUM(D62:D66)</f>
@@ -1658,48 +1717,48 @@
       </c>
     </row>
     <row r="68" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="14"/>
-      <c r="B68" s="19"/>
-      <c r="C68" s="20"/>
-      <c r="D68" s="21"/>
+      <c r="A68" s="16"/>
+      <c r="B68" s="21"/>
+      <c r="C68" s="22"/>
+      <c r="D68" s="23"/>
     </row>
     <row r="69" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="13"/>
-      <c r="B69" s="15"/>
-      <c r="C69" s="16"/>
+      <c r="A69" s="15"/>
+      <c r="B69" s="17"/>
+      <c r="C69" s="18"/>
       <c r="D69" s="7"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="14"/>
-      <c r="B70" s="17"/>
-      <c r="C70" s="18"/>
+      <c r="A70" s="16"/>
+      <c r="B70" s="19"/>
+      <c r="C70" s="20"/>
       <c r="D70" s="8"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" s="14"/>
-      <c r="B71" s="17"/>
-      <c r="C71" s="18"/>
+      <c r="A71" s="16"/>
+      <c r="B71" s="19"/>
+      <c r="C71" s="20"/>
       <c r="D71" s="8"/>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="14"/>
-      <c r="B72" s="17"/>
-      <c r="C72" s="18"/>
+      <c r="A72" s="16"/>
+      <c r="B72" s="19"/>
+      <c r="C72" s="20"/>
       <c r="D72" s="8"/>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" s="14"/>
-      <c r="B73" s="17"/>
-      <c r="C73" s="18"/>
+      <c r="A73" s="16"/>
+      <c r="B73" s="19"/>
+      <c r="C73" s="20"/>
       <c r="D73" s="8"/>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="14"/>
+      <c r="A74" s="16"/>
       <c r="B74" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D74" s="9">
         <f>SUM(D69:D73)</f>
@@ -1707,48 +1766,48 @@
       </c>
     </row>
     <row r="75" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="25"/>
-      <c r="B75" s="22"/>
-      <c r="C75" s="23"/>
-      <c r="D75" s="24"/>
+      <c r="A75" s="24"/>
+      <c r="B75" s="25"/>
+      <c r="C75" s="26"/>
+      <c r="D75" s="27"/>
     </row>
     <row r="76" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="13"/>
-      <c r="B76" s="15"/>
-      <c r="C76" s="16"/>
+      <c r="A76" s="15"/>
+      <c r="B76" s="17"/>
+      <c r="C76" s="18"/>
       <c r="D76" s="7"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="14"/>
-      <c r="B77" s="17"/>
-      <c r="C77" s="18"/>
+      <c r="A77" s="16"/>
+      <c r="B77" s="19"/>
+      <c r="C77" s="20"/>
       <c r="D77" s="8"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="14"/>
-      <c r="B78" s="17"/>
-      <c r="C78" s="18"/>
+      <c r="A78" s="16"/>
+      <c r="B78" s="19"/>
+      <c r="C78" s="20"/>
       <c r="D78" s="8"/>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="14"/>
-      <c r="B79" s="17"/>
-      <c r="C79" s="18"/>
+      <c r="A79" s="16"/>
+      <c r="B79" s="19"/>
+      <c r="C79" s="20"/>
       <c r="D79" s="8"/>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" s="14"/>
-      <c r="B80" s="17"/>
-      <c r="C80" s="18"/>
+      <c r="A80" s="16"/>
+      <c r="B80" s="19"/>
+      <c r="C80" s="20"/>
       <c r="D80" s="8"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A81" s="14"/>
+      <c r="A81" s="16"/>
       <c r="B81" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D81" s="9">
         <f>SUM(D76:D80)</f>
@@ -1756,37 +1815,101 @@
       </c>
     </row>
     <row r="82" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="25"/>
-      <c r="B82" s="22"/>
-      <c r="C82" s="23"/>
-      <c r="D82" s="24"/>
+      <c r="A82" s="24"/>
+      <c r="B82" s="25"/>
+      <c r="C82" s="26"/>
+      <c r="D82" s="27"/>
     </row>
     <row r="83" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="11"/>
       <c r="B83" s="10"/>
       <c r="C83" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D83" s="12">
         <f>D11+D18+D25+D32+D39+D46+D53+D60+D67+D74+D81</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A84" s="14" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="36" t="s">
-        <v>0</v>
-      </c>
-      <c r="B84" s="36"/>
-      <c r="C84" s="36"/>
-      <c r="D84" s="36"/>
+      <c r="B84" s="14"/>
+      <c r="C84" s="14"/>
+      <c r="D84" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="82">
+  <mergeCells count="81">
+    <mergeCell ref="A20:A26"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="A76:A82"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="B78:C78"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B82:D82"/>
+    <mergeCell ref="A48:A54"/>
+    <mergeCell ref="A69:A75"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="B75:D75"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="A55:A61"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="A41:A47"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="A62:A68"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B68:D68"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="A6:A12"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B4:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:A5"/>
     <mergeCell ref="A84:D84"/>
     <mergeCell ref="A13:A19"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B19:D19"/>
@@ -1798,87 +1921,14 @@
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="A34:A40"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B4:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A6:A12"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B12:D12"/>
     <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="A62:A68"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B68:D68"/>
-    <mergeCell ref="A41:A47"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="A48:A54"/>
-    <mergeCell ref="A69:A75"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="B75:D75"/>
-    <mergeCell ref="A76:A82"/>
-    <mergeCell ref="B76:C76"/>
-    <mergeCell ref="B77:C77"/>
-    <mergeCell ref="B78:C78"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="B80:C80"/>
-    <mergeCell ref="B82:D82"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="A55:A61"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="B59:C59"/>
-    <mergeCell ref="B61:D61"/>
-    <mergeCell ref="A20:A26"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B26:D26"/>
   </mergeCells>
-  <conditionalFormatting sqref="D6:D11">
-    <cfRule type="containsText" dxfId="23" priority="23" operator="containsText" text="Terminé">
+  <conditionalFormatting sqref="D6:D11 D13:D14 D16:D18">
+    <cfRule type="containsText" dxfId="21" priority="23" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="22" priority="24" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="20" priority="24" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D6)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D13:D18">
-    <cfRule type="containsText" dxfId="21" priority="21" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D13)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="22" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D13)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D20:D25">

</xml_diff>

<commit_message>
docs: finalise les diagrammes UML d'analyse, le script SQL et la maquette Stitch
Mise à jour du journal et du planning.
</commit_message>
<xml_diff>
--- a/doc/GAMEZ_Journal.xlsx
+++ b/doc/GAMEZ_Journal.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/thibaudfrederic_gamez_studentfr_ch/Documents/TPI/tpi2026-codementor/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58766AB4-7609-4881-B248-B038BF3DA048}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17C8924E-38E3-4D59-80F1-DC51E62CC784}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="8" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Journal!$A$5:$HI$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$D$83</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Journal!$B:$D,Journal!$1:$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$D$84</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="27">
   <si>
     <t>Insérer les lignes au-dessus de celle-ci !</t>
   </si>
@@ -133,6 +133,27 @@
   </si>
   <si>
     <t>Second jour, j'ai pu rattraper un peu le retard en avancant plus vite que prévu sur le diagramme ER et le usecase</t>
+  </si>
+  <si>
+    <t>Finalisation diagrammes de séquence système (DSS2 et DSS3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Création des 3 diagrammes d'activité (Ajouter, Consulter résultats, Supprimer un projet) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réparation du diagramme des cas d'utilisation </t>
+  </si>
+  <si>
+    <t>Decouverte d'un bug dans le diagramme des cas d'utilisation</t>
+  </si>
+  <si>
+    <t>Maquette Stitch</t>
+  </si>
+  <si>
+    <t>Création du diagramme de base de donnée</t>
+  </si>
+  <si>
+    <t>J'ai bien avancé, j'ai découvert que mon usecase était cassé et j'ai du le refaire sinon la conception commence bien</t>
   </si>
 </sst>
 </file>
@@ -209,7 +230,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -228,6 +249,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="18">
     <border>
@@ -434,7 +467,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -580,35 +613,33 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="22">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="20">
     <dxf>
       <font>
         <strike val="0"/>
@@ -1194,8 +1225,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D84"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D85"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5703125" style="1"/>
     <col min="2" max="3" width="31.7109375" style="1" customWidth="1"/>
@@ -1380,65 +1411,91 @@
       <c r="D19" s="23"/>
     </row>
     <row r="20" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="15"/>
-      <c r="B20" s="17"/>
+      <c r="A20" s="15">
+        <v>46157</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>20</v>
+      </c>
       <c r="C20" s="18"/>
-      <c r="D20" s="7"/>
+      <c r="D20" s="7">
+        <v>2</v>
+      </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="16"/>
-      <c r="B21" s="19"/>
+      <c r="B21" s="38" t="s">
+        <v>21</v>
+      </c>
       <c r="C21" s="20"/>
-      <c r="D21" s="8"/>
+      <c r="D21" s="8">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="16"/>
-      <c r="B22" s="19"/>
-      <c r="C22" s="20"/>
+      <c r="B22" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" s="40"/>
       <c r="D22" s="8"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="16"/>
-      <c r="B23" s="19"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="8"/>
+      <c r="B23" s="41" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" s="42"/>
+      <c r="D23" s="8">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="16"/>
-      <c r="B24" s="19"/>
+      <c r="B24" s="19" t="s">
+        <v>24</v>
+      </c>
       <c r="C24" s="20"/>
-      <c r="D24" s="8"/>
+      <c r="D24" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="16"/>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C25" s="20"/>
+      <c r="D25" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" s="16"/>
+      <c r="B26" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C26" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D25" s="9">
-        <f>SUM(D20:D24)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="16"/>
-      <c r="B26" s="21"/>
-      <c r="C26" s="22"/>
-      <c r="D26" s="23"/>
-    </row>
-    <row r="27" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="15"/>
-      <c r="B27" s="17"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="7"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="16"/>
-      <c r="B28" s="19"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="8"/>
+      <c r="D26" s="9">
+        <f>SUM(D20:D25)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="16"/>
+      <c r="B27" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" s="22"/>
+      <c r="D27" s="23"/>
+    </row>
+    <row r="28" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="15"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="7"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="16"/>
@@ -1460,34 +1517,34 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="16"/>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="19"/>
+      <c r="C32" s="20"/>
+      <c r="D32" s="8"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" s="16"/>
+      <c r="B33" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C33" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D32" s="9">
-        <f>SUM(D27:D31)</f>
+      <c r="D33" s="9">
+        <f>SUM(D28:D32)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="24"/>
-      <c r="B33" s="25"/>
-      <c r="C33" s="26"/>
-      <c r="D33" s="27"/>
-    </row>
-    <row r="34" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="15"/>
-      <c r="B34" s="17"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="7"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="16"/>
-      <c r="B35" s="19"/>
-      <c r="C35" s="20"/>
-      <c r="D35" s="8"/>
+    <row r="34" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="24"/>
+      <c r="B34" s="25"/>
+      <c r="C34" s="26"/>
+      <c r="D34" s="27"/>
+    </row>
+    <row r="35" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="15"/>
+      <c r="B35" s="17"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="7"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="16"/>
@@ -1509,34 +1566,34 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="16"/>
-      <c r="B39" s="2" t="s">
+      <c r="B39" s="19"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="8"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" s="16"/>
+      <c r="B40" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C40" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D39" s="9">
-        <f>SUM(D34:D38)</f>
+      <c r="D40" s="9">
+        <f>SUM(D35:D39)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="24"/>
-      <c r="B40" s="25"/>
-      <c r="C40" s="26"/>
-      <c r="D40" s="27"/>
-    </row>
-    <row r="41" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="15"/>
-      <c r="B41" s="17"/>
-      <c r="C41" s="18"/>
-      <c r="D41" s="7"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="16"/>
-      <c r="B42" s="19"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="8"/>
+    <row r="41" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="24"/>
+      <c r="B41" s="25"/>
+      <c r="C41" s="26"/>
+      <c r="D41" s="27"/>
+    </row>
+    <row r="42" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="15"/>
+      <c r="B42" s="17"/>
+      <c r="C42" s="18"/>
+      <c r="D42" s="7"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="16"/>
@@ -1558,34 +1615,34 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="16"/>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="19"/>
+      <c r="C46" s="20"/>
+      <c r="D46" s="8"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" s="16"/>
+      <c r="B47" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="C47" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D46" s="9">
-        <f>SUM(D41:D45)</f>
+      <c r="D47" s="9">
+        <f>SUM(D42:D46)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="24"/>
-      <c r="B47" s="25"/>
-      <c r="C47" s="26"/>
-      <c r="D47" s="27"/>
-    </row>
-    <row r="48" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="15"/>
-      <c r="B48" s="17"/>
-      <c r="C48" s="18"/>
-      <c r="D48" s="7"/>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="16"/>
-      <c r="B49" s="19"/>
-      <c r="C49" s="20"/>
-      <c r="D49" s="8"/>
+    <row r="48" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="24"/>
+      <c r="B48" s="25"/>
+      <c r="C48" s="26"/>
+      <c r="D48" s="27"/>
+    </row>
+    <row r="49" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="15"/>
+      <c r="B49" s="17"/>
+      <c r="C49" s="18"/>
+      <c r="D49" s="7"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" s="16"/>
@@ -1607,34 +1664,34 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" s="16"/>
-      <c r="B53" s="2" t="s">
+      <c r="B53" s="19"/>
+      <c r="C53" s="20"/>
+      <c r="D53" s="8"/>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" s="16"/>
+      <c r="B54" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C53" s="3" t="s">
+      <c r="C54" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D53" s="9">
-        <f>SUM(D48:D52)</f>
+      <c r="D54" s="9">
+        <f>SUM(D49:D53)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="24"/>
-      <c r="B54" s="25"/>
-      <c r="C54" s="26"/>
-      <c r="D54" s="27"/>
-    </row>
-    <row r="55" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="15"/>
-      <c r="B55" s="17"/>
-      <c r="C55" s="18"/>
-      <c r="D55" s="7"/>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="16"/>
-      <c r="B56" s="19"/>
-      <c r="C56" s="20"/>
-      <c r="D56" s="8"/>
+    <row r="55" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="24"/>
+      <c r="B55" s="25"/>
+      <c r="C55" s="26"/>
+      <c r="D55" s="27"/>
+    </row>
+    <row r="56" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="15"/>
+      <c r="B56" s="17"/>
+      <c r="C56" s="18"/>
+      <c r="D56" s="7"/>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" s="16"/>
@@ -1656,34 +1713,34 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" s="16"/>
-      <c r="B60" s="2" t="s">
+      <c r="B60" s="19"/>
+      <c r="C60" s="20"/>
+      <c r="D60" s="8"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" s="16"/>
+      <c r="B61" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C60" s="3" t="s">
+      <c r="C61" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D60" s="9">
-        <f>SUM(D55:D59)</f>
+      <c r="D61" s="9">
+        <f>SUM(D56:D60)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="24"/>
-      <c r="B61" s="25"/>
-      <c r="C61" s="26"/>
-      <c r="D61" s="27"/>
-    </row>
-    <row r="62" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="15"/>
-      <c r="B62" s="17"/>
-      <c r="C62" s="18"/>
-      <c r="D62" s="7"/>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="16"/>
-      <c r="B63" s="19"/>
-      <c r="C63" s="20"/>
-      <c r="D63" s="8"/>
+    <row r="62" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="24"/>
+      <c r="B62" s="25"/>
+      <c r="C62" s="26"/>
+      <c r="D62" s="27"/>
+    </row>
+    <row r="63" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="15"/>
+      <c r="B63" s="17"/>
+      <c r="C63" s="18"/>
+      <c r="D63" s="7"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" s="16"/>
@@ -1705,34 +1762,34 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" s="16"/>
-      <c r="B67" s="2" t="s">
+      <c r="B67" s="19"/>
+      <c r="C67" s="20"/>
+      <c r="D67" s="8"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" s="16"/>
+      <c r="B68" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C67" s="3" t="s">
+      <c r="C68" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D67" s="9">
-        <f>SUM(D62:D66)</f>
+      <c r="D68" s="9">
+        <f>SUM(D63:D67)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="16"/>
-      <c r="B68" s="21"/>
-      <c r="C68" s="22"/>
-      <c r="D68" s="23"/>
-    </row>
-    <row r="69" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="15"/>
-      <c r="B69" s="17"/>
-      <c r="C69" s="18"/>
-      <c r="D69" s="7"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="16"/>
-      <c r="B70" s="19"/>
-      <c r="C70" s="20"/>
-      <c r="D70" s="8"/>
+    <row r="69" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="16"/>
+      <c r="B69" s="21"/>
+      <c r="C69" s="22"/>
+      <c r="D69" s="23"/>
+    </row>
+    <row r="70" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="15"/>
+      <c r="B70" s="17"/>
+      <c r="C70" s="18"/>
+      <c r="D70" s="7"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" s="16"/>
@@ -1754,34 +1811,34 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" s="16"/>
-      <c r="B74" s="2" t="s">
+      <c r="B74" s="19"/>
+      <c r="C74" s="20"/>
+      <c r="D74" s="8"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" s="16"/>
+      <c r="B75" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C74" s="3" t="s">
+      <c r="C75" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D74" s="9">
-        <f>SUM(D69:D73)</f>
+      <c r="D75" s="9">
+        <f>SUM(D70:D74)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="24"/>
-      <c r="B75" s="25"/>
-      <c r="C75" s="26"/>
-      <c r="D75" s="27"/>
-    </row>
-    <row r="76" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="15"/>
-      <c r="B76" s="17"/>
-      <c r="C76" s="18"/>
-      <c r="D76" s="7"/>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="16"/>
-      <c r="B77" s="19"/>
-      <c r="C77" s="20"/>
-      <c r="D77" s="8"/>
+    <row r="76" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A76" s="24"/>
+      <c r="B76" s="25"/>
+      <c r="C76" s="26"/>
+      <c r="D76" s="27"/>
+    </row>
+    <row r="77" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="15"/>
+      <c r="B77" s="17"/>
+      <c r="C77" s="18"/>
+      <c r="D77" s="7"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A78" s="16"/>
@@ -1803,98 +1860,105 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A81" s="16"/>
-      <c r="B81" s="2" t="s">
+      <c r="B81" s="19"/>
+      <c r="C81" s="20"/>
+      <c r="D81" s="8"/>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" s="16"/>
+      <c r="B82" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C81" s="3" t="s">
+      <c r="C82" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D81" s="9">
-        <f>SUM(D76:D80)</f>
+      <c r="D82" s="9">
+        <f>SUM(D77:D81)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="24"/>
-      <c r="B82" s="25"/>
-      <c r="C82" s="26"/>
-      <c r="D82" s="27"/>
-    </row>
-    <row r="83" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="11"/>
-      <c r="B83" s="10"/>
-      <c r="C83" s="3" t="s">
+    <row r="83" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="24"/>
+      <c r="B83" s="25"/>
+      <c r="C83" s="26"/>
+      <c r="D83" s="27"/>
+    </row>
+    <row r="84" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A84" s="11"/>
+      <c r="B84" s="10"/>
+      <c r="C84" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D83" s="12">
-        <f>D11+D18+D25+D32+D39+D46+D53+D60+D67+D74+D81</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="14" t="s">
+      <c r="D84" s="12">
+        <f>D11+D18+D26+D33+D40+D47+D54+D61+D68+D75+D82</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A85" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B84" s="14"/>
-      <c r="C84" s="14"/>
-      <c r="D84" s="14"/>
+      <c r="B85" s="14"/>
+      <c r="C85" s="14"/>
+      <c r="D85" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="81">
-    <mergeCell ref="A20:A26"/>
+  <mergeCells count="82">
+    <mergeCell ref="A20:A27"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B27:D27"/>
     <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="B56:C56"/>
     <mergeCell ref="B57:C57"/>
     <mergeCell ref="B58:C58"/>
     <mergeCell ref="B59:C59"/>
-    <mergeCell ref="B61:D61"/>
-    <mergeCell ref="A76:A82"/>
-    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="B62:D62"/>
+    <mergeCell ref="A77:A83"/>
     <mergeCell ref="B77:C77"/>
     <mergeCell ref="B78:C78"/>
     <mergeCell ref="B79:C79"/>
     <mergeCell ref="B80:C80"/>
-    <mergeCell ref="B82:D82"/>
-    <mergeCell ref="A48:A54"/>
-    <mergeCell ref="A69:A75"/>
-    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B83:D83"/>
+    <mergeCell ref="A49:A55"/>
+    <mergeCell ref="A70:A76"/>
     <mergeCell ref="B70:C70"/>
     <mergeCell ref="B71:C71"/>
     <mergeCell ref="B72:C72"/>
     <mergeCell ref="B73:C73"/>
-    <mergeCell ref="B75:D75"/>
-    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="B76:D76"/>
     <mergeCell ref="B49:C49"/>
     <mergeCell ref="B50:C50"/>
     <mergeCell ref="B51:C51"/>
     <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="A55:A61"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="A41:A47"/>
-    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="A56:A62"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="A42:A48"/>
     <mergeCell ref="B42:C42"/>
     <mergeCell ref="B43:C43"/>
     <mergeCell ref="B44:C44"/>
     <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="A62:A68"/>
-    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="A63:A69"/>
     <mergeCell ref="B63:C63"/>
     <mergeCell ref="B64:C64"/>
     <mergeCell ref="B65:C65"/>
     <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B68:D68"/>
-    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="B69:D69"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B41:D41"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B10:C10"/>
@@ -1906,109 +1970,101 @@
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A84:D84"/>
+    <mergeCell ref="A85:D85"/>
     <mergeCell ref="A13:A19"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A27:A33"/>
-    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="A28:A34"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="A34:A40"/>
-    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="A35:A41"/>
+    <mergeCell ref="B35:C35"/>
   </mergeCells>
-  <conditionalFormatting sqref="D6:D11 D13:D14 D16:D18">
-    <cfRule type="containsText" dxfId="21" priority="23" operator="containsText" text="Terminé">
+  <conditionalFormatting sqref="D6:D11 D13:D14 D16:D18 D20:D23 D25:D26">
+    <cfRule type="containsText" dxfId="19" priority="23" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="24" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="18" priority="24" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D6)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D20:D25">
-    <cfRule type="containsText" dxfId="19" priority="3" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D20)))</formula>
+  <conditionalFormatting sqref="D28:D33">
+    <cfRule type="containsText" dxfId="17" priority="19" operator="containsText" text="Terminé">
+      <formula>NOT(ISERROR(SEARCH("Terminé",D28)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="4" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D20)))</formula>
+    <cfRule type="containsText" dxfId="16" priority="20" operator="containsText" text="En cours">
+      <formula>NOT(ISERROR(SEARCH("En cours",D28)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D27:D32">
-    <cfRule type="containsText" dxfId="17" priority="19" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D27)))</formula>
+  <conditionalFormatting sqref="D35:D40">
+    <cfRule type="containsText" dxfId="15" priority="17" operator="containsText" text="Terminé">
+      <formula>NOT(ISERROR(SEARCH("Terminé",D35)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="20" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D27)))</formula>
+    <cfRule type="containsText" dxfId="14" priority="18" operator="containsText" text="En cours">
+      <formula>NOT(ISERROR(SEARCH("En cours",D35)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D34:D39">
-    <cfRule type="containsText" dxfId="15" priority="17" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D34)))</formula>
+  <conditionalFormatting sqref="D42:D47">
+    <cfRule type="containsText" dxfId="13" priority="9" operator="containsText" text="Terminé">
+      <formula>NOT(ISERROR(SEARCH("Terminé",D42)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="18" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D34)))</formula>
+    <cfRule type="containsText" dxfId="12" priority="10" operator="containsText" text="En cours">
+      <formula>NOT(ISERROR(SEARCH("En cours",D42)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D41:D46">
-    <cfRule type="containsText" dxfId="13" priority="9" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D41)))</formula>
+  <conditionalFormatting sqref="D49:D54">
+    <cfRule type="containsText" dxfId="11" priority="7" operator="containsText" text="Terminé">
+      <formula>NOT(ISERROR(SEARCH("Terminé",D49)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="10" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D41)))</formula>
+    <cfRule type="containsText" dxfId="10" priority="8" operator="containsText" text="En cours">
+      <formula>NOT(ISERROR(SEARCH("En cours",D49)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D48:D53">
-    <cfRule type="containsText" dxfId="11" priority="7" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D48)))</formula>
+  <conditionalFormatting sqref="D56:D61">
+    <cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="Terminé">
+      <formula>NOT(ISERROR(SEARCH("Terminé",D56)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="8" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D48)))</formula>
+    <cfRule type="containsText" dxfId="8" priority="6" operator="containsText" text="En cours">
+      <formula>NOT(ISERROR(SEARCH("En cours",D56)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D55:D60">
-    <cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D55)))</formula>
+  <conditionalFormatting sqref="D63:D68">
+    <cfRule type="containsText" dxfId="7" priority="15" operator="containsText" text="Terminé">
+      <formula>NOT(ISERROR(SEARCH("Terminé",D63)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="6" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D55)))</formula>
+    <cfRule type="containsText" dxfId="6" priority="16" operator="containsText" text="En cours">
+      <formula>NOT(ISERROR(SEARCH("En cours",D63)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D62:D67">
-    <cfRule type="containsText" dxfId="7" priority="15" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D62)))</formula>
+  <conditionalFormatting sqref="D70:D75">
+    <cfRule type="containsText" dxfId="5" priority="13" operator="containsText" text="Terminé">
+      <formula>NOT(ISERROR(SEARCH("Terminé",D70)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="16" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D62)))</formula>
+    <cfRule type="containsText" dxfId="4" priority="14" operator="containsText" text="En cours">
+      <formula>NOT(ISERROR(SEARCH("En cours",D70)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D69:D74">
-    <cfRule type="containsText" dxfId="5" priority="13" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D69)))</formula>
+  <conditionalFormatting sqref="D77:D82">
+    <cfRule type="containsText" dxfId="3" priority="11" operator="containsText" text="Terminé">
+      <formula>NOT(ISERROR(SEARCH("Terminé",D77)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="14" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D69)))</formula>
+    <cfRule type="containsText" dxfId="2" priority="12" operator="containsText" text="En cours">
+      <formula>NOT(ISERROR(SEARCH("En cours",D77)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D76:D81">
-    <cfRule type="containsText" dxfId="3" priority="11" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D76)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="12" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D76)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D83">
+  <conditionalFormatting sqref="D84">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D83)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D84)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D83)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D84)))</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
@@ -2020,8 +2076,8 @@
     <oddFooter>&amp;L&amp;8&amp;F&amp;R&amp;8Page &amp;P/&amp;N</oddFooter>
   </headerFooter>
   <rowBreaks count="2" manualBreakCount="2">
-    <brk id="47" max="16383" man="1"/>
-    <brk id="83" max="3" man="1"/>
+    <brk id="48" max="16383" man="1"/>
+    <brk id="84" max="3" man="1"/>
   </rowBreaks>
   <legacyDrawingHF r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(server): début de l'implémentation du backend
Avancement du rapport et des diagrammes.
</commit_message>
<xml_diff>
--- a/doc/GAMEZ_Journal.xlsx
+++ b/doc/GAMEZ_Journal.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/thibaudfrederic_gamez_studentfr_ch/Documents/TPI/tpi2026-codementor/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17C8924E-38E3-4D59-80F1-DC51E62CC784}"/>
+  <xr:revisionPtr revIDLastSave="96" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{694ADE40-25B2-4FCC-9C82-5D63D7EE3CA7}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2640" yWindow="2640" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="8" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Journal!$A$5:$HI$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$D$86</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Journal!$B:$D,Journal!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$D$84</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="35">
   <si>
     <t>Insérer les lignes au-dessus de celle-ci !</t>
   </si>
@@ -154,6 +154,30 @@
   </si>
   <si>
     <t>J'ai bien avancé, j'ai découvert que mon usecase était cassé et j'ai du le refaire sinon la conception commence bien</t>
+  </si>
+  <si>
+    <t>Diagramme de classe frontend</t>
+  </si>
+  <si>
+    <t>Diagramme de classe backend</t>
+  </si>
+  <si>
+    <t>Conception des endpoints API REST</t>
+  </si>
+  <si>
+    <t>Conception des tests</t>
+  </si>
+  <si>
+    <t>Structure MVC de base</t>
+  </si>
+  <si>
+    <t>Création base de donnée</t>
+  </si>
+  <si>
+    <t>Documentation conception</t>
+  </si>
+  <si>
+    <t>Cette journée s'est bien passé, j'ai pu commencer l'implementation du backend en faisant la structure de base et la base de donnée. Je suis confiant</t>
   </si>
 </sst>
 </file>
@@ -467,7 +491,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -519,120 +543,128 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1225,8 +1257,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D85"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D87"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5703125" style="1"/>
     <col min="2" max="3" width="31.7109375" style="1" customWidth="1"/>
@@ -1236,93 +1268,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
     </row>
     <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="36"/>
+      <c r="B2" s="42"/>
+      <c r="C2" s="43"/>
       <c r="D2" s="4">
         <v>151446</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="30"/>
+      <c r="C4" s="37"/>
       <c r="D4" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="31"/>
-      <c r="B5" s="31"/>
-      <c r="C5" s="32"/>
+      <c r="A5" s="38"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="39"/>
       <c r="D5" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="37">
+      <c r="A6" s="34">
         <v>46153</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="34"/>
+      <c r="C6" s="41"/>
       <c r="D6" s="7">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="16"/>
-      <c r="B7" s="19" t="s">
+      <c r="A7" s="17"/>
+      <c r="B7" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="20"/>
+      <c r="C7" s="21"/>
       <c r="D7" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="16"/>
-      <c r="B8" s="19" t="s">
+      <c r="A8" s="17"/>
+      <c r="B8" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="20"/>
+      <c r="C8" s="21"/>
       <c r="D8" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="16"/>
-      <c r="B9" s="19" t="s">
+      <c r="A9" s="17"/>
+      <c r="B9" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="20"/>
+      <c r="C9" s="21"/>
       <c r="D9" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="16"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="20"/>
+      <c r="A10" s="17"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="21"/>
       <c r="D10" s="8"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="16"/>
+      <c r="A11" s="17"/>
       <c r="B11" s="2" t="s">
         <v>6</v>
       </c>
@@ -1335,37 +1367,37 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="16"/>
-      <c r="B12" s="21" t="s">
+      <c r="A12" s="17"/>
+      <c r="B12" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="22"/>
-      <c r="D12" s="23"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="27"/>
     </row>
     <row r="13" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="15">
+      <c r="A13" s="16">
         <v>46154</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="18"/>
+      <c r="C13" s="19"/>
       <c r="D13" s="7">
         <v>0.5</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="16"/>
-      <c r="B14" s="19" t="s">
+      <c r="A14" s="17"/>
+      <c r="B14" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="20"/>
+      <c r="C14" s="21"/>
       <c r="D14" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="16"/>
+      <c r="A15" s="17"/>
       <c r="B15" s="13" t="s">
         <v>18</v>
       </c>
@@ -1374,23 +1406,23 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="16"/>
-      <c r="B16" s="19" t="s">
+      <c r="A16" s="17"/>
+      <c r="B16" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="20"/>
+      <c r="C16" s="21"/>
       <c r="D16" s="8">
         <v>1.5</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="16"/>
-      <c r="B17" s="19"/>
-      <c r="C17" s="20"/>
+      <c r="A17" s="17"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="21"/>
       <c r="D17" s="8"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="16"/>
+      <c r="A18" s="17"/>
       <c r="B18" s="2" t="s">
         <v>6</v>
       </c>
@@ -1403,75 +1435,75 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="16"/>
-      <c r="B19" s="21" t="s">
+      <c r="A19" s="17"/>
+      <c r="B19" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="22"/>
-      <c r="D19" s="23"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="27"/>
     </row>
     <row r="20" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="15">
+      <c r="A20" s="16">
         <v>46157</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="18"/>
+      <c r="C20" s="19"/>
       <c r="D20" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="16"/>
-      <c r="B21" s="38" t="s">
+      <c r="A21" s="17"/>
+      <c r="B21" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="20"/>
+      <c r="C21" s="21"/>
       <c r="D21" s="8">
         <v>2.5</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="16"/>
-      <c r="B22" s="39" t="s">
+      <c r="A22" s="17"/>
+      <c r="B22" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="40"/>
+      <c r="C22" s="23"/>
       <c r="D22" s="8"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="16"/>
-      <c r="B23" s="41" t="s">
+      <c r="A23" s="17"/>
+      <c r="B23" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="42"/>
+      <c r="C23" s="29"/>
       <c r="D23" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="16"/>
-      <c r="B24" s="19" t="s">
+      <c r="A24" s="17"/>
+      <c r="B24" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="20"/>
+      <c r="C24" s="21"/>
       <c r="D24" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="16"/>
-      <c r="B25" s="19" t="s">
+      <c r="A25" s="17"/>
+      <c r="B25" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="C25" s="20"/>
+      <c r="C25" s="21"/>
       <c r="D25" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="16"/>
+      <c r="A26" s="17"/>
       <c r="B26" s="2" t="s">
         <v>6</v>
       </c>
@@ -1484,426 +1516,544 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="16"/>
-      <c r="B27" s="21" t="s">
+      <c r="A27" s="17"/>
+      <c r="B27" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="22"/>
-      <c r="D27" s="23"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="27"/>
     </row>
     <row r="28" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="15"/>
-      <c r="B28" s="17"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="7"/>
+      <c r="A28" s="16">
+        <v>46160</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" s="19"/>
+      <c r="D28" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="16"/>
-      <c r="B29" s="19"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="8"/>
+      <c r="A29" s="17"/>
+      <c r="B29" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C29" s="21"/>
+      <c r="D29" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="16"/>
-      <c r="B30" s="19"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="8"/>
+      <c r="A30" s="17"/>
+      <c r="B30" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="C30" s="21"/>
+      <c r="D30" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="16"/>
-      <c r="B31" s="19"/>
-      <c r="C31" s="20"/>
-      <c r="D31" s="8"/>
+      <c r="A31" s="17"/>
+      <c r="B31" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="C31" s="21"/>
+      <c r="D31" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="16"/>
-      <c r="B32" s="19"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="8"/>
+      <c r="A32" s="17"/>
+      <c r="B32" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C32" s="15"/>
+      <c r="D32" s="8">
+        <v>2</v>
+      </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="16"/>
-      <c r="B33" s="2" t="s">
+      <c r="A33" s="17"/>
+      <c r="B33" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" s="15"/>
+      <c r="D33" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" s="17"/>
+      <c r="B34" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C34" s="21"/>
+      <c r="D34" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" s="17"/>
+      <c r="B35" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C35" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D33" s="9">
-        <f>SUM(D28:D32)</f>
+      <c r="D35" s="9">
+        <f>SUM(D28:D34)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="33"/>
+      <c r="B36" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="C36" s="31"/>
+      <c r="D36" s="32"/>
+    </row>
+    <row r="37" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="16"/>
+      <c r="B37" s="18"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="7"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" s="17"/>
+      <c r="B38" s="24"/>
+      <c r="C38" s="21"/>
+      <c r="D38" s="8"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" s="17"/>
+      <c r="B39" s="24"/>
+      <c r="C39" s="21"/>
+      <c r="D39" s="8"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" s="17"/>
+      <c r="B40" s="24"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="8"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" s="17"/>
+      <c r="B41" s="24"/>
+      <c r="C41" s="21"/>
+      <c r="D41" s="8"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" s="17"/>
+      <c r="B42" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D42" s="9">
+        <f>SUM(D37:D41)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="24"/>
-      <c r="B34" s="25"/>
-      <c r="C34" s="26"/>
-      <c r="D34" s="27"/>
-    </row>
-    <row r="35" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="15"/>
-      <c r="B35" s="17"/>
-      <c r="C35" s="18"/>
-      <c r="D35" s="7"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="16"/>
-      <c r="B36" s="19"/>
-      <c r="C36" s="20"/>
-      <c r="D36" s="8"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="16"/>
-      <c r="B37" s="19"/>
-      <c r="C37" s="20"/>
-      <c r="D37" s="8"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="16"/>
-      <c r="B38" s="19"/>
-      <c r="C38" s="20"/>
-      <c r="D38" s="8"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="16"/>
-      <c r="B39" s="19"/>
-      <c r="C39" s="20"/>
-      <c r="D39" s="8"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="16"/>
-      <c r="B40" s="2" t="s">
+    <row r="43" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="33"/>
+      <c r="B43" s="30"/>
+      <c r="C43" s="31"/>
+      <c r="D43" s="32"/>
+    </row>
+    <row r="44" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="16"/>
+      <c r="B44" s="18"/>
+      <c r="C44" s="19"/>
+      <c r="D44" s="7"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" s="17"/>
+      <c r="B45" s="24"/>
+      <c r="C45" s="21"/>
+      <c r="D45" s="8"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" s="17"/>
+      <c r="B46" s="24"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="8"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" s="17"/>
+      <c r="B47" s="24"/>
+      <c r="C47" s="21"/>
+      <c r="D47" s="8"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" s="17"/>
+      <c r="B48" s="24"/>
+      <c r="C48" s="21"/>
+      <c r="D48" s="8"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" s="17"/>
+      <c r="B49" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C49" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D40" s="9">
-        <f>SUM(D35:D39)</f>
+      <c r="D49" s="9">
+        <f>SUM(D44:D48)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="24"/>
-      <c r="B41" s="25"/>
-      <c r="C41" s="26"/>
-      <c r="D41" s="27"/>
-    </row>
-    <row r="42" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="15"/>
-      <c r="B42" s="17"/>
-      <c r="C42" s="18"/>
-      <c r="D42" s="7"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="16"/>
-      <c r="B43" s="19"/>
-      <c r="C43" s="20"/>
-      <c r="D43" s="8"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="16"/>
-      <c r="B44" s="19"/>
-      <c r="C44" s="20"/>
-      <c r="D44" s="8"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="16"/>
-      <c r="B45" s="19"/>
-      <c r="C45" s="20"/>
-      <c r="D45" s="8"/>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="16"/>
-      <c r="B46" s="19"/>
-      <c r="C46" s="20"/>
-      <c r="D46" s="8"/>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="16"/>
-      <c r="B47" s="2" t="s">
+    <row r="50" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="33"/>
+      <c r="B50" s="30"/>
+      <c r="C50" s="31"/>
+      <c r="D50" s="32"/>
+    </row>
+    <row r="51" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="16"/>
+      <c r="B51" s="18"/>
+      <c r="C51" s="19"/>
+      <c r="D51" s="7"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" s="17"/>
+      <c r="B52" s="24"/>
+      <c r="C52" s="21"/>
+      <c r="D52" s="8"/>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" s="17"/>
+      <c r="B53" s="24"/>
+      <c r="C53" s="21"/>
+      <c r="D53" s="8"/>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" s="17"/>
+      <c r="B54" s="24"/>
+      <c r="C54" s="21"/>
+      <c r="D54" s="8"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" s="17"/>
+      <c r="B55" s="24"/>
+      <c r="C55" s="21"/>
+      <c r="D55" s="8"/>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" s="17"/>
+      <c r="B56" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C47" s="3" t="s">
+      <c r="C56" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D47" s="9">
-        <f>SUM(D42:D46)</f>
+      <c r="D56" s="9">
+        <f>SUM(D51:D55)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="24"/>
-      <c r="B48" s="25"/>
-      <c r="C48" s="26"/>
-      <c r="D48" s="27"/>
-    </row>
-    <row r="49" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="15"/>
-      <c r="B49" s="17"/>
-      <c r="C49" s="18"/>
-      <c r="D49" s="7"/>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A50" s="16"/>
-      <c r="B50" s="19"/>
-      <c r="C50" s="20"/>
-      <c r="D50" s="8"/>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A51" s="16"/>
-      <c r="B51" s="19"/>
-      <c r="C51" s="20"/>
-      <c r="D51" s="8"/>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="16"/>
-      <c r="B52" s="19"/>
-      <c r="C52" s="20"/>
-      <c r="D52" s="8"/>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="16"/>
-      <c r="B53" s="19"/>
-      <c r="C53" s="20"/>
-      <c r="D53" s="8"/>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="16"/>
-      <c r="B54" s="2" t="s">
+    <row r="57" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="33"/>
+      <c r="B57" s="30"/>
+      <c r="C57" s="31"/>
+      <c r="D57" s="32"/>
+    </row>
+    <row r="58" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="16"/>
+      <c r="B58" s="18"/>
+      <c r="C58" s="19"/>
+      <c r="D58" s="7"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" s="17"/>
+      <c r="B59" s="24"/>
+      <c r="C59" s="21"/>
+      <c r="D59" s="8"/>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" s="17"/>
+      <c r="B60" s="24"/>
+      <c r="C60" s="21"/>
+      <c r="D60" s="8"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" s="17"/>
+      <c r="B61" s="24"/>
+      <c r="C61" s="21"/>
+      <c r="D61" s="8"/>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" s="17"/>
+      <c r="B62" s="24"/>
+      <c r="C62" s="21"/>
+      <c r="D62" s="8"/>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" s="17"/>
+      <c r="B63" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="C63" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D54" s="9">
-        <f>SUM(D49:D53)</f>
+      <c r="D63" s="9">
+        <f>SUM(D58:D62)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="24"/>
-      <c r="B55" s="25"/>
-      <c r="C55" s="26"/>
-      <c r="D55" s="27"/>
-    </row>
-    <row r="56" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="15"/>
-      <c r="B56" s="17"/>
-      <c r="C56" s="18"/>
-      <c r="D56" s="7"/>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" s="16"/>
-      <c r="B57" s="19"/>
-      <c r="C57" s="20"/>
-      <c r="D57" s="8"/>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" s="16"/>
-      <c r="B58" s="19"/>
-      <c r="C58" s="20"/>
-      <c r="D58" s="8"/>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A59" s="16"/>
-      <c r="B59" s="19"/>
-      <c r="C59" s="20"/>
-      <c r="D59" s="8"/>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" s="16"/>
-      <c r="B60" s="19"/>
-      <c r="C60" s="20"/>
-      <c r="D60" s="8"/>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" s="16"/>
-      <c r="B61" s="2" t="s">
+    <row r="64" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="33"/>
+      <c r="B64" s="30"/>
+      <c r="C64" s="31"/>
+      <c r="D64" s="32"/>
+    </row>
+    <row r="65" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="16"/>
+      <c r="B65" s="18"/>
+      <c r="C65" s="19"/>
+      <c r="D65" s="7"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" s="17"/>
+      <c r="B66" s="24"/>
+      <c r="C66" s="21"/>
+      <c r="D66" s="8"/>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" s="17"/>
+      <c r="B67" s="24"/>
+      <c r="C67" s="21"/>
+      <c r="D67" s="8"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" s="17"/>
+      <c r="B68" s="24"/>
+      <c r="C68" s="21"/>
+      <c r="D68" s="8"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A69" s="17"/>
+      <c r="B69" s="24"/>
+      <c r="C69" s="21"/>
+      <c r="D69" s="8"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" s="17"/>
+      <c r="B70" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C61" s="3" t="s">
+      <c r="C70" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D61" s="9">
-        <f>SUM(D56:D60)</f>
+      <c r="D70" s="9">
+        <f>SUM(D65:D69)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="24"/>
-      <c r="B62" s="25"/>
-      <c r="C62" s="26"/>
-      <c r="D62" s="27"/>
-    </row>
-    <row r="63" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="15"/>
-      <c r="B63" s="17"/>
-      <c r="C63" s="18"/>
-      <c r="D63" s="7"/>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="16"/>
-      <c r="B64" s="19"/>
-      <c r="C64" s="20"/>
-      <c r="D64" s="8"/>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" s="16"/>
-      <c r="B65" s="19"/>
-      <c r="C65" s="20"/>
-      <c r="D65" s="8"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" s="16"/>
-      <c r="B66" s="19"/>
-      <c r="C66" s="20"/>
-      <c r="D66" s="8"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="16"/>
-      <c r="B67" s="19"/>
-      <c r="C67" s="20"/>
-      <c r="D67" s="8"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="16"/>
-      <c r="B68" s="2" t="s">
+    <row r="71" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="17"/>
+      <c r="B71" s="25"/>
+      <c r="C71" s="26"/>
+      <c r="D71" s="27"/>
+    </row>
+    <row r="72" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="16"/>
+      <c r="B72" s="18"/>
+      <c r="C72" s="19"/>
+      <c r="D72" s="7"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A73" s="17"/>
+      <c r="B73" s="24"/>
+      <c r="C73" s="21"/>
+      <c r="D73" s="8"/>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" s="17"/>
+      <c r="B74" s="24"/>
+      <c r="C74" s="21"/>
+      <c r="D74" s="8"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" s="17"/>
+      <c r="B75" s="24"/>
+      <c r="C75" s="21"/>
+      <c r="D75" s="8"/>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" s="17"/>
+      <c r="B76" s="24"/>
+      <c r="C76" s="21"/>
+      <c r="D76" s="8"/>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" s="17"/>
+      <c r="B77" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C68" s="3" t="s">
+      <c r="C77" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D68" s="9">
-        <f>SUM(D63:D67)</f>
+      <c r="D77" s="9">
+        <f>SUM(D72:D76)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="16"/>
-      <c r="B69" s="21"/>
-      <c r="C69" s="22"/>
-      <c r="D69" s="23"/>
-    </row>
-    <row r="70" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="15"/>
-      <c r="B70" s="17"/>
-      <c r="C70" s="18"/>
-      <c r="D70" s="7"/>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" s="16"/>
-      <c r="B71" s="19"/>
-      <c r="C71" s="20"/>
-      <c r="D71" s="8"/>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="16"/>
-      <c r="B72" s="19"/>
-      <c r="C72" s="20"/>
-      <c r="D72" s="8"/>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" s="16"/>
-      <c r="B73" s="19"/>
-      <c r="C73" s="20"/>
-      <c r="D73" s="8"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="16"/>
-      <c r="B74" s="19"/>
-      <c r="C74" s="20"/>
-      <c r="D74" s="8"/>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="16"/>
-      <c r="B75" s="2" t="s">
+    <row r="78" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="33"/>
+      <c r="B78" s="30"/>
+      <c r="C78" s="31"/>
+      <c r="D78" s="32"/>
+    </row>
+    <row r="79" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A79" s="16"/>
+      <c r="B79" s="18"/>
+      <c r="C79" s="19"/>
+      <c r="D79" s="7"/>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" s="17"/>
+      <c r="B80" s="24"/>
+      <c r="C80" s="21"/>
+      <c r="D80" s="8"/>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A81" s="17"/>
+      <c r="B81" s="24"/>
+      <c r="C81" s="21"/>
+      <c r="D81" s="8"/>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" s="17"/>
+      <c r="B82" s="24"/>
+      <c r="C82" s="21"/>
+      <c r="D82" s="8"/>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" s="17"/>
+      <c r="B83" s="24"/>
+      <c r="C83" s="21"/>
+      <c r="D83" s="8"/>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A84" s="17"/>
+      <c r="B84" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C75" s="3" t="s">
+      <c r="C84" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D75" s="9">
-        <f>SUM(D70:D74)</f>
+      <c r="D84" s="9">
+        <f>SUM(D79:D83)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="24"/>
-      <c r="B76" s="25"/>
-      <c r="C76" s="26"/>
-      <c r="D76" s="27"/>
-    </row>
-    <row r="77" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="15"/>
-      <c r="B77" s="17"/>
-      <c r="C77" s="18"/>
-      <c r="D77" s="7"/>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="16"/>
-      <c r="B78" s="19"/>
-      <c r="C78" s="20"/>
-      <c r="D78" s="8"/>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="16"/>
-      <c r="B79" s="19"/>
-      <c r="C79" s="20"/>
-      <c r="D79" s="8"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" s="16"/>
-      <c r="B80" s="19"/>
-      <c r="C80" s="20"/>
-      <c r="D80" s="8"/>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A81" s="16"/>
-      <c r="B81" s="19"/>
-      <c r="C81" s="20"/>
-      <c r="D81" s="8"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" s="16"/>
-      <c r="B82" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C82" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D82" s="9">
-        <f>SUM(D77:D81)</f>
+    <row r="85" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A85" s="33"/>
+      <c r="B85" s="30"/>
+      <c r="C85" s="31"/>
+      <c r="D85" s="32"/>
+    </row>
+    <row r="86" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A86" s="11"/>
+      <c r="B86" s="10"/>
+      <c r="C86" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D86" s="12">
+        <f>D11+D18+D26+D35+D42+D49+D56+D63+D70+D77+D84</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A87" s="44" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="83" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="24"/>
-      <c r="B83" s="25"/>
-      <c r="C83" s="26"/>
-      <c r="D83" s="27"/>
-    </row>
-    <row r="84" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="11"/>
-      <c r="B84" s="10"/>
-      <c r="C84" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D84" s="12">
-        <f>D11+D18+D26+D33+D40+D47+D54+D61+D68+D75+D82</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A85" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B85" s="14"/>
-      <c r="C85" s="14"/>
-      <c r="D85" s="14"/>
+      <c r="B87" s="44"/>
+      <c r="C87" s="44"/>
+      <c r="D87" s="44"/>
     </row>
   </sheetData>
   <mergeCells count="82">
+    <mergeCell ref="A87:D87"/>
+    <mergeCell ref="A13:A19"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="A28:A36"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="A37:A43"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B4:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="A6:A12"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="A65:A71"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="B68:C68"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B71:D71"/>
+    <mergeCell ref="A44:A50"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="A51:A57"/>
+    <mergeCell ref="A72:A78"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="B78:D78"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="A58:A64"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="A79:A85"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B85:D85"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B64:D64"/>
     <mergeCell ref="A20:A27"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B21:C21"/>
@@ -1912,80 +2062,6 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="B59:C59"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="B62:D62"/>
-    <mergeCell ref="A77:A83"/>
-    <mergeCell ref="B77:C77"/>
-    <mergeCell ref="B78:C78"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="B80:C80"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B83:D83"/>
-    <mergeCell ref="A49:A55"/>
-    <mergeCell ref="A70:A76"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="B76:D76"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="A56:A62"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="A42:A48"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B48:D48"/>
-    <mergeCell ref="A63:A69"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="B69:D69"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A6:A12"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B4:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A85:D85"/>
-    <mergeCell ref="A13:A19"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A28:A34"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="A35:A41"/>
-    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <conditionalFormatting sqref="D6:D11 D13:D14 D16:D18 D20:D23 D25:D26">
     <cfRule type="containsText" dxfId="19" priority="23" operator="containsText" text="Terminé">
@@ -1995,7 +2071,7 @@
       <formula>NOT(ISERROR(SEARCH("En cours",D6)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D28:D33">
+  <conditionalFormatting sqref="D28:D35">
     <cfRule type="containsText" dxfId="17" priority="19" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D28)))</formula>
     </cfRule>
@@ -2003,68 +2079,68 @@
       <formula>NOT(ISERROR(SEARCH("En cours",D28)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D35:D40">
+  <conditionalFormatting sqref="D37:D42">
     <cfRule type="containsText" dxfId="15" priority="17" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D35)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D37)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="14" priority="18" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D35)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D37)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D42:D47">
+  <conditionalFormatting sqref="D44:D49">
     <cfRule type="containsText" dxfId="13" priority="9" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D42)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D44)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="12" priority="10" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D42)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D44)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D49:D54">
+  <conditionalFormatting sqref="D51:D56">
     <cfRule type="containsText" dxfId="11" priority="7" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D49)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D51)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="10" priority="8" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D49)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D51)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D56:D61">
+  <conditionalFormatting sqref="D58:D63">
     <cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D56)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D58)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="8" priority="6" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D56)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D58)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D63:D68">
+  <conditionalFormatting sqref="D65:D70">
     <cfRule type="containsText" dxfId="7" priority="15" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D63)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D65)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="16" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D63)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D65)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D70:D75">
+  <conditionalFormatting sqref="D72:D77">
     <cfRule type="containsText" dxfId="5" priority="13" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D70)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D72)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="14" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D70)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D72)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D77:D82">
+  <conditionalFormatting sqref="D79:D84">
     <cfRule type="containsText" dxfId="3" priority="11" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D77)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D79)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="2" priority="12" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D77)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D79)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D84">
+  <conditionalFormatting sqref="D86">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D84)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D86)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D84)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D86)))</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
@@ -2076,8 +2152,8 @@
     <oddFooter>&amp;L&amp;8&amp;F&amp;R&amp;8Page &amp;P/&amp;N</oddFooter>
   </headerFooter>
   <rowBreaks count="2" manualBreakCount="2">
-    <brk id="48" max="16383" man="1"/>
-    <brk id="84" max="3" man="1"/>
+    <brk id="50" max="16383" man="1"/>
+    <brk id="86" max="3" man="1"/>
   </rowBreaks>
   <legacyDrawingHF r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: mise à jour du rapport, du planning et du journal
</commit_message>
<xml_diff>
--- a/doc/GAMEZ_Journal.xlsx
+++ b/doc/GAMEZ_Journal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/thibaudfrederic_gamez_studentfr_ch/Documents/TPI/tpi2026-codementor/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="96" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{694ADE40-25B2-4FCC-9C82-5D63D7EE3CA7}"/>
+  <xr:revisionPtr revIDLastSave="117" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7955D887-A663-4A9A-AE44-7D9F99C04AFD}"/>
   <bookViews>
     <workbookView xWindow="2640" yWindow="2640" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="40">
   <si>
     <t>Insérer les lignes au-dessus de celle-ci !</t>
   </si>
@@ -178,6 +178,21 @@
   </si>
   <si>
     <t>Cette journée s'est bien passé, j'ai pu commencer l'implementation du backend en faisant la structure de base et la base de donnée. Je suis confiant</t>
+  </si>
+  <si>
+    <t>La table "suggested_fix" complique les choses et n'est pas très utile</t>
+  </si>
+  <si>
+    <t>Supression et changement des schémas et de la structure du code</t>
+  </si>
+  <si>
+    <t>Ajout des tâches todolist</t>
+  </si>
+  <si>
+    <t>Documentation</t>
+  </si>
+  <si>
+    <t>J'ai pris du retard sur l'implémentation mais je pense pas que ca poseras problème</t>
   </si>
 </sst>
 </file>
@@ -254,7 +269,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -285,6 +300,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="18">
     <border>
@@ -491,7 +512,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -623,6 +644,14 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -665,6 +694,20 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1268,51 +1311,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
     </row>
     <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="43"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="45"/>
       <c r="D2" s="4">
         <v>151446</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="37"/>
+      <c r="C4" s="39"/>
       <c r="D4" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="38"/>
-      <c r="B5" s="38"/>
-      <c r="C5" s="39"/>
+      <c r="A5" s="40"/>
+      <c r="B5" s="40"/>
+      <c r="C5" s="41"/>
       <c r="D5" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="34">
+      <c r="A6" s="36">
         <v>46153</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="41"/>
+      <c r="C6" s="43"/>
       <c r="D6" s="7">
         <v>3</v>
       </c>
@@ -1339,10 +1382,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="17"/>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="21"/>
+      <c r="C9" s="35"/>
       <c r="D9" s="8">
         <v>1</v>
       </c>
@@ -1617,28 +1660,46 @@
       <c r="D36" s="32"/>
     </row>
     <row r="37" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="16"/>
-      <c r="B37" s="18"/>
-      <c r="C37" s="19"/>
-      <c r="D37" s="7"/>
+      <c r="A37" s="16">
+        <v>46161</v>
+      </c>
+      <c r="B37" s="47" t="s">
+        <v>35</v>
+      </c>
+      <c r="C37" s="48"/>
+      <c r="D37" s="7">
+        <v>0</v>
+      </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="17"/>
-      <c r="B38" s="24"/>
-      <c r="C38" s="21"/>
-      <c r="D38" s="8"/>
+      <c r="B38" s="49" t="s">
+        <v>36</v>
+      </c>
+      <c r="C38" s="50"/>
+      <c r="D38" s="8">
+        <v>2</v>
+      </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="17"/>
-      <c r="B39" s="24"/>
+      <c r="B39" s="24" t="s">
+        <v>37</v>
+      </c>
       <c r="C39" s="21"/>
-      <c r="D39" s="8"/>
+      <c r="D39" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="17"/>
-      <c r="B40" s="24"/>
+      <c r="B40" s="24" t="s">
+        <v>38</v>
+      </c>
       <c r="C40" s="21"/>
-      <c r="D40" s="8"/>
+      <c r="D40" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="17"/>
@@ -1656,12 +1717,14 @@
       </c>
       <c r="D42" s="9">
         <f>SUM(D37:D41)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="33"/>
-      <c r="B43" s="30"/>
+      <c r="B43" s="30" t="s">
+        <v>39</v>
+      </c>
       <c r="C43" s="31"/>
       <c r="D43" s="32"/>
     </row>
@@ -1967,19 +2030,19 @@
       </c>
       <c r="D86" s="12">
         <f>D11+D18+D26+D35+D42+D49+D56+D63+D70+D77+D84</f>
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A87" s="44" t="s">
+      <c r="A87" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B87" s="44"/>
-      <c r="C87" s="44"/>
-      <c r="D87" s="44"/>
+      <c r="B87" s="46"/>
+      <c r="C87" s="46"/>
+      <c r="D87" s="46"/>
     </row>
   </sheetData>
-  <mergeCells count="82">
+  <mergeCells count="81">
     <mergeCell ref="A87:D87"/>
     <mergeCell ref="A13:A19"/>
     <mergeCell ref="B13:C13"/>
@@ -1995,23 +2058,22 @@
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="A37:A43"/>
-    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="A6:A12"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B8:C8"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="B4:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A6:A12"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B38:C38"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="B41:C41"/>
     <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
     <mergeCell ref="A65:A71"/>
     <mergeCell ref="B65:C65"/>
     <mergeCell ref="B66:C66"/>

</xml_diff>

<commit_message>
docs: avancement du rapport, du planning et du journal
</commit_message>
<xml_diff>
--- a/doc/GAMEZ_Journal.xlsx
+++ b/doc/GAMEZ_Journal.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/thibaudfrederic_gamez_studentfr_ch/Documents/TPI/tpi2026-codementor/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="117" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7955D887-A663-4A9A-AE44-7D9F99C04AFD}"/>
+  <xr:revisionPtr revIDLastSave="123" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{083039BA-7EF5-4E0E-A345-71FC00E7F862}"/>
   <bookViews>
-    <workbookView xWindow="2640" yWindow="2640" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="8" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Journal!$A$5:$HI$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">Journal!$B:$D,Journal!$1:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$D$86</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">Journal!$B:$D,Journal!$1:$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="43">
   <si>
     <t>Insérer les lignes au-dessus de celle-ci !</t>
   </si>
@@ -193,6 +193,15 @@
   </si>
   <si>
     <t>J'ai pris du retard sur l'implémentation mais je pense pas que ca poseras problème</t>
+  </si>
+  <si>
+    <t>Finalisation doc analyse</t>
+  </si>
+  <si>
+    <t>Finalisation doc conception</t>
+  </si>
+  <si>
+    <t>J'ai fais que de la documentation, toujours en retard du coup mais vais pouvoir le rattraper demain</t>
   </si>
 </sst>
 </file>
@@ -572,6 +581,12 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -694,12 +709,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1301,7 +1310,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D87"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5703125" style="1"/>
     <col min="2" max="3" width="31.7109375" style="1" customWidth="1"/>
@@ -1311,93 +1320,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
     </row>
     <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="45"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="47"/>
       <c r="D2" s="4">
         <v>151446</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="38" t="s">
+      <c r="B4" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="39"/>
+      <c r="C4" s="41"/>
       <c r="D4" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="40"/>
-      <c r="B5" s="40"/>
-      <c r="C5" s="41"/>
+      <c r="A5" s="42"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="43"/>
       <c r="D5" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="36">
+      <c r="A6" s="38">
         <v>46153</v>
       </c>
-      <c r="B6" s="42" t="s">
+      <c r="B6" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="43"/>
+      <c r="C6" s="45"/>
       <c r="D6" s="7">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="17"/>
-      <c r="B7" s="24" t="s">
+      <c r="A7" s="19"/>
+      <c r="B7" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="21"/>
+      <c r="C7" s="23"/>
       <c r="D7" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="17"/>
-      <c r="B8" s="24" t="s">
+      <c r="A8" s="19"/>
+      <c r="B8" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="21"/>
+      <c r="C8" s="23"/>
       <c r="D8" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="17"/>
-      <c r="B9" s="34" t="s">
+      <c r="A9" s="19"/>
+      <c r="B9" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="35"/>
+      <c r="C9" s="37"/>
       <c r="D9" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="17"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="21"/>
+      <c r="A10" s="19"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="23"/>
       <c r="D10" s="8"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="17"/>
+      <c r="A11" s="19"/>
       <c r="B11" s="2" t="s">
         <v>6</v>
       </c>
@@ -1410,37 +1419,37 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="17"/>
-      <c r="B12" s="25" t="s">
+      <c r="A12" s="19"/>
+      <c r="B12" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="26"/>
-      <c r="D12" s="27"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="29"/>
     </row>
     <row r="13" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="16">
+      <c r="A13" s="18">
         <v>46154</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="19"/>
+      <c r="C13" s="21"/>
       <c r="D13" s="7">
         <v>0.5</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="17"/>
-      <c r="B14" s="24" t="s">
+      <c r="A14" s="19"/>
+      <c r="B14" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="21"/>
+      <c r="C14" s="23"/>
       <c r="D14" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="17"/>
+      <c r="A15" s="19"/>
       <c r="B15" s="13" t="s">
         <v>18</v>
       </c>
@@ -1449,23 +1458,23 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="17"/>
-      <c r="B16" s="24" t="s">
+      <c r="A16" s="19"/>
+      <c r="B16" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="21"/>
+      <c r="C16" s="23"/>
       <c r="D16" s="8">
         <v>1.5</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="17"/>
-      <c r="B17" s="24"/>
-      <c r="C17" s="21"/>
+      <c r="A17" s="19"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="23"/>
       <c r="D17" s="8"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="17"/>
+      <c r="A18" s="19"/>
       <c r="B18" s="2" t="s">
         <v>6</v>
       </c>
@@ -1478,75 +1487,75 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="17"/>
-      <c r="B19" s="25" t="s">
+      <c r="A19" s="19"/>
+      <c r="B19" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="26"/>
-      <c r="D19" s="27"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="29"/>
     </row>
     <row r="20" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="16">
+      <c r="A20" s="18">
         <v>46157</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="19"/>
+      <c r="C20" s="21"/>
       <c r="D20" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="17"/>
-      <c r="B21" s="20" t="s">
+      <c r="A21" s="19"/>
+      <c r="B21" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="21"/>
+      <c r="C21" s="23"/>
       <c r="D21" s="8">
         <v>2.5</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="17"/>
-      <c r="B22" s="22" t="s">
+      <c r="A22" s="19"/>
+      <c r="B22" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="23"/>
+      <c r="C22" s="25"/>
       <c r="D22" s="8"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="17"/>
-      <c r="B23" s="28" t="s">
+      <c r="A23" s="19"/>
+      <c r="B23" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="29"/>
+      <c r="C23" s="31"/>
       <c r="D23" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="17"/>
-      <c r="B24" s="24" t="s">
+      <c r="A24" s="19"/>
+      <c r="B24" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="21"/>
+      <c r="C24" s="23"/>
       <c r="D24" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="17"/>
-      <c r="B25" s="24" t="s">
+      <c r="A25" s="19"/>
+      <c r="B25" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="C25" s="21"/>
+      <c r="C25" s="23"/>
       <c r="D25" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="17"/>
+      <c r="A26" s="19"/>
       <c r="B26" s="2" t="s">
         <v>6</v>
       </c>
@@ -1559,57 +1568,57 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="17"/>
-      <c r="B27" s="25" t="s">
+      <c r="A27" s="19"/>
+      <c r="B27" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="26"/>
-      <c r="D27" s="27"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="29"/>
     </row>
     <row r="28" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="16">
+      <c r="A28" s="18">
         <v>46160</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="19"/>
+      <c r="C28" s="21"/>
       <c r="D28" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="17"/>
-      <c r="B29" s="24" t="s">
+      <c r="A29" s="19"/>
+      <c r="B29" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="21"/>
+      <c r="C29" s="23"/>
       <c r="D29" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="17"/>
-      <c r="B30" s="24" t="s">
+      <c r="A30" s="19"/>
+      <c r="B30" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="21"/>
+      <c r="C30" s="23"/>
       <c r="D30" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="17"/>
-      <c r="B31" s="24" t="s">
+      <c r="A31" s="19"/>
+      <c r="B31" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="21"/>
+      <c r="C31" s="23"/>
       <c r="D31" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="17"/>
+      <c r="A32" s="19"/>
       <c r="B32" s="14" t="s">
         <v>31</v>
       </c>
@@ -1619,7 +1628,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="17"/>
+      <c r="A33" s="19"/>
       <c r="B33" s="14" t="s">
         <v>32</v>
       </c>
@@ -1629,17 +1638,17 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="17"/>
-      <c r="B34" s="24" t="s">
+      <c r="A34" s="19"/>
+      <c r="B34" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="21"/>
+      <c r="C34" s="23"/>
       <c r="D34" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="17"/>
+      <c r="A35" s="19"/>
       <c r="B35" s="2" t="s">
         <v>6</v>
       </c>
@@ -1652,27 +1661,27 @@
       </c>
     </row>
     <row r="36" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="33"/>
-      <c r="B36" s="30" t="s">
+      <c r="A36" s="35"/>
+      <c r="B36" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="C36" s="31"/>
-      <c r="D36" s="32"/>
+      <c r="C36" s="33"/>
+      <c r="D36" s="34"/>
     </row>
     <row r="37" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="16">
+      <c r="A37" s="18">
         <v>46161</v>
       </c>
-      <c r="B37" s="47" t="s">
+      <c r="B37" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="C37" s="48"/>
+      <c r="C37" s="17"/>
       <c r="D37" s="7">
         <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="17"/>
+      <c r="A38" s="19"/>
       <c r="B38" s="49" t="s">
         <v>36</v>
       </c>
@@ -1682,33 +1691,33 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="17"/>
-      <c r="B39" s="24" t="s">
+      <c r="A39" s="19"/>
+      <c r="B39" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="C39" s="21"/>
+      <c r="C39" s="23"/>
       <c r="D39" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="17"/>
-      <c r="B40" s="24" t="s">
+      <c r="A40" s="19"/>
+      <c r="B40" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="21"/>
+      <c r="C40" s="23"/>
       <c r="D40" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="17"/>
-      <c r="B41" s="24"/>
-      <c r="C41" s="21"/>
+      <c r="A41" s="19"/>
+      <c r="B41" s="26"/>
+      <c r="C41" s="23"/>
       <c r="D41" s="8"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="17"/>
+      <c r="A42" s="19"/>
       <c r="B42" s="2" t="s">
         <v>6</v>
       </c>
@@ -1721,45 +1730,55 @@
       </c>
     </row>
     <row r="43" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="33"/>
-      <c r="B43" s="30" t="s">
+      <c r="A43" s="35"/>
+      <c r="B43" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="C43" s="31"/>
-      <c r="D43" s="32"/>
+      <c r="C43" s="33"/>
+      <c r="D43" s="34"/>
     </row>
     <row r="44" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="16"/>
-      <c r="B44" s="18"/>
-      <c r="C44" s="19"/>
-      <c r="D44" s="7"/>
+      <c r="A44" s="18">
+        <v>46163</v>
+      </c>
+      <c r="B44" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C44" s="21"/>
+      <c r="D44" s="7">
+        <v>2</v>
+      </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="17"/>
-      <c r="B45" s="24"/>
-      <c r="C45" s="21"/>
-      <c r="D45" s="8"/>
+      <c r="A45" s="19"/>
+      <c r="B45" s="26" t="s">
+        <v>41</v>
+      </c>
+      <c r="C45" s="23"/>
+      <c r="D45" s="8">
+        <v>2</v>
+      </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="17"/>
-      <c r="B46" s="24"/>
-      <c r="C46" s="21"/>
+      <c r="A46" s="19"/>
+      <c r="B46" s="26"/>
+      <c r="C46" s="23"/>
       <c r="D46" s="8"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="17"/>
-      <c r="B47" s="24"/>
-      <c r="C47" s="21"/>
+      <c r="A47" s="19"/>
+      <c r="B47" s="26"/>
+      <c r="C47" s="23"/>
       <c r="D47" s="8"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="17"/>
-      <c r="B48" s="24"/>
-      <c r="C48" s="21"/>
+      <c r="A48" s="19"/>
+      <c r="B48" s="26"/>
+      <c r="C48" s="23"/>
       <c r="D48" s="8"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="17"/>
+      <c r="A49" s="19"/>
       <c r="B49" s="2" t="s">
         <v>6</v>
       </c>
@@ -1768,47 +1787,49 @@
       </c>
       <c r="D49" s="9">
         <f>SUM(D44:D48)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="33"/>
-      <c r="B50" s="30"/>
-      <c r="C50" s="31"/>
-      <c r="D50" s="32"/>
+      <c r="A50" s="35"/>
+      <c r="B50" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="C50" s="33"/>
+      <c r="D50" s="34"/>
     </row>
     <row r="51" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="16"/>
-      <c r="B51" s="18"/>
-      <c r="C51" s="19"/>
+      <c r="A51" s="18"/>
+      <c r="B51" s="20"/>
+      <c r="C51" s="21"/>
       <c r="D51" s="7"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="17"/>
-      <c r="B52" s="24"/>
-      <c r="C52" s="21"/>
+      <c r="A52" s="19"/>
+      <c r="B52" s="26"/>
+      <c r="C52" s="23"/>
       <c r="D52" s="8"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="17"/>
-      <c r="B53" s="24"/>
-      <c r="C53" s="21"/>
+      <c r="A53" s="19"/>
+      <c r="B53" s="26"/>
+      <c r="C53" s="23"/>
       <c r="D53" s="8"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="17"/>
-      <c r="B54" s="24"/>
-      <c r="C54" s="21"/>
+      <c r="A54" s="19"/>
+      <c r="B54" s="26"/>
+      <c r="C54" s="23"/>
       <c r="D54" s="8"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" s="17"/>
-      <c r="B55" s="24"/>
-      <c r="C55" s="21"/>
+      <c r="A55" s="19"/>
+      <c r="B55" s="26"/>
+      <c r="C55" s="23"/>
       <c r="D55" s="8"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="17"/>
+      <c r="A56" s="19"/>
       <c r="B56" s="2" t="s">
         <v>6</v>
       </c>
@@ -1821,43 +1842,43 @@
       </c>
     </row>
     <row r="57" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="33"/>
-      <c r="B57" s="30"/>
-      <c r="C57" s="31"/>
-      <c r="D57" s="32"/>
+      <c r="A57" s="35"/>
+      <c r="B57" s="32"/>
+      <c r="C57" s="33"/>
+      <c r="D57" s="34"/>
     </row>
     <row r="58" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="16"/>
-      <c r="B58" s="18"/>
-      <c r="C58" s="19"/>
+      <c r="A58" s="18"/>
+      <c r="B58" s="20"/>
+      <c r="C58" s="21"/>
       <c r="D58" s="7"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A59" s="17"/>
-      <c r="B59" s="24"/>
-      <c r="C59" s="21"/>
+      <c r="A59" s="19"/>
+      <c r="B59" s="26"/>
+      <c r="C59" s="23"/>
       <c r="D59" s="8"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" s="17"/>
-      <c r="B60" s="24"/>
-      <c r="C60" s="21"/>
+      <c r="A60" s="19"/>
+      <c r="B60" s="26"/>
+      <c r="C60" s="23"/>
       <c r="D60" s="8"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" s="17"/>
-      <c r="B61" s="24"/>
-      <c r="C61" s="21"/>
+      <c r="A61" s="19"/>
+      <c r="B61" s="26"/>
+      <c r="C61" s="23"/>
       <c r="D61" s="8"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="17"/>
-      <c r="B62" s="24"/>
-      <c r="C62" s="21"/>
+      <c r="A62" s="19"/>
+      <c r="B62" s="26"/>
+      <c r="C62" s="23"/>
       <c r="D62" s="8"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="17"/>
+      <c r="A63" s="19"/>
       <c r="B63" s="2" t="s">
         <v>6</v>
       </c>
@@ -1870,43 +1891,43 @@
       </c>
     </row>
     <row r="64" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="33"/>
-      <c r="B64" s="30"/>
-      <c r="C64" s="31"/>
-      <c r="D64" s="32"/>
+      <c r="A64" s="35"/>
+      <c r="B64" s="32"/>
+      <c r="C64" s="33"/>
+      <c r="D64" s="34"/>
     </row>
     <row r="65" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="16"/>
-      <c r="B65" s="18"/>
-      <c r="C65" s="19"/>
+      <c r="A65" s="18"/>
+      <c r="B65" s="20"/>
+      <c r="C65" s="21"/>
       <c r="D65" s="7"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" s="17"/>
-      <c r="B66" s="24"/>
-      <c r="C66" s="21"/>
+      <c r="A66" s="19"/>
+      <c r="B66" s="26"/>
+      <c r="C66" s="23"/>
       <c r="D66" s="8"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="17"/>
-      <c r="B67" s="24"/>
-      <c r="C67" s="21"/>
+      <c r="A67" s="19"/>
+      <c r="B67" s="26"/>
+      <c r="C67" s="23"/>
       <c r="D67" s="8"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="17"/>
-      <c r="B68" s="24"/>
-      <c r="C68" s="21"/>
+      <c r="A68" s="19"/>
+      <c r="B68" s="26"/>
+      <c r="C68" s="23"/>
       <c r="D68" s="8"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="17"/>
-      <c r="B69" s="24"/>
-      <c r="C69" s="21"/>
+      <c r="A69" s="19"/>
+      <c r="B69" s="26"/>
+      <c r="C69" s="23"/>
       <c r="D69" s="8"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="17"/>
+      <c r="A70" s="19"/>
       <c r="B70" s="2" t="s">
         <v>6</v>
       </c>
@@ -1919,43 +1940,43 @@
       </c>
     </row>
     <row r="71" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="17"/>
-      <c r="B71" s="25"/>
-      <c r="C71" s="26"/>
-      <c r="D71" s="27"/>
+      <c r="A71" s="19"/>
+      <c r="B71" s="27"/>
+      <c r="C71" s="28"/>
+      <c r="D71" s="29"/>
     </row>
     <row r="72" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="16"/>
-      <c r="B72" s="18"/>
-      <c r="C72" s="19"/>
+      <c r="A72" s="18"/>
+      <c r="B72" s="20"/>
+      <c r="C72" s="21"/>
       <c r="D72" s="7"/>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" s="17"/>
-      <c r="B73" s="24"/>
-      <c r="C73" s="21"/>
+      <c r="A73" s="19"/>
+      <c r="B73" s="26"/>
+      <c r="C73" s="23"/>
       <c r="D73" s="8"/>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="17"/>
-      <c r="B74" s="24"/>
-      <c r="C74" s="21"/>
+      <c r="A74" s="19"/>
+      <c r="B74" s="26"/>
+      <c r="C74" s="23"/>
       <c r="D74" s="8"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="17"/>
-      <c r="B75" s="24"/>
-      <c r="C75" s="21"/>
+      <c r="A75" s="19"/>
+      <c r="B75" s="26"/>
+      <c r="C75" s="23"/>
       <c r="D75" s="8"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="17"/>
-      <c r="B76" s="24"/>
-      <c r="C76" s="21"/>
+      <c r="A76" s="19"/>
+      <c r="B76" s="26"/>
+      <c r="C76" s="23"/>
       <c r="D76" s="8"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="17"/>
+      <c r="A77" s="19"/>
       <c r="B77" s="2" t="s">
         <v>6</v>
       </c>
@@ -1968,43 +1989,43 @@
       </c>
     </row>
     <row r="78" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="33"/>
-      <c r="B78" s="30"/>
-      <c r="C78" s="31"/>
-      <c r="D78" s="32"/>
+      <c r="A78" s="35"/>
+      <c r="B78" s="32"/>
+      <c r="C78" s="33"/>
+      <c r="D78" s="34"/>
     </row>
     <row r="79" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="16"/>
-      <c r="B79" s="18"/>
-      <c r="C79" s="19"/>
+      <c r="A79" s="18"/>
+      <c r="B79" s="20"/>
+      <c r="C79" s="21"/>
       <c r="D79" s="7"/>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" s="17"/>
-      <c r="B80" s="24"/>
-      <c r="C80" s="21"/>
+      <c r="A80" s="19"/>
+      <c r="B80" s="26"/>
+      <c r="C80" s="23"/>
       <c r="D80" s="8"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A81" s="17"/>
-      <c r="B81" s="24"/>
-      <c r="C81" s="21"/>
+      <c r="A81" s="19"/>
+      <c r="B81" s="26"/>
+      <c r="C81" s="23"/>
       <c r="D81" s="8"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" s="17"/>
-      <c r="B82" s="24"/>
-      <c r="C82" s="21"/>
+      <c r="A82" s="19"/>
+      <c r="B82" s="26"/>
+      <c r="C82" s="23"/>
       <c r="D82" s="8"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" s="17"/>
-      <c r="B83" s="24"/>
-      <c r="C83" s="21"/>
+      <c r="A83" s="19"/>
+      <c r="B83" s="26"/>
+      <c r="C83" s="23"/>
       <c r="D83" s="8"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="17"/>
+      <c r="A84" s="19"/>
       <c r="B84" s="2" t="s">
         <v>6</v>
       </c>
@@ -2017,10 +2038,10 @@
       </c>
     </row>
     <row r="85" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="33"/>
-      <c r="B85" s="30"/>
-      <c r="C85" s="31"/>
-      <c r="D85" s="32"/>
+      <c r="A85" s="35"/>
+      <c r="B85" s="32"/>
+      <c r="C85" s="33"/>
+      <c r="D85" s="34"/>
     </row>
     <row r="86" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="11"/>
@@ -2030,16 +2051,16 @@
       </c>
       <c r="D86" s="12">
         <f>D11+D18+D26+D35+D42+D49+D56+D63+D70+D77+D84</f>
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A87" s="46" t="s">
+      <c r="A87" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B87" s="46"/>
-      <c r="C87" s="46"/>
-      <c r="D87" s="46"/>
+      <c r="B87" s="48"/>
+      <c r="C87" s="48"/>
+      <c r="D87" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="81">

</xml_diff>

<commit_message>
feat(server): OAuth GitHub, services projet/GitHub et middleware d'authentification
Mise à jour du rapport, du planning et du journal.
</commit_message>
<xml_diff>
--- a/doc/GAMEZ_Journal.xlsx
+++ b/doc/GAMEZ_Journal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/thibaudfrederic_gamez_studentfr_ch/Documents/TPI/tpi2026-codementor/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="123" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{083039BA-7EF5-4E0E-A345-71FC00E7F862}"/>
+  <xr:revisionPtr revIDLastSave="144" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2BA4BDF-C0F2-4C4A-8205-E3EDB440E1B7}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="8" r:id="rId1"/>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Journal!$A$5:$HI$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Journal!$B:$D,Journal!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$D$86</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$D$88</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="49">
   <si>
     <t>Insérer les lignes au-dessus de celle-ci !</t>
   </si>
@@ -202,6 +202,24 @@
   </si>
   <si>
     <t>J'ai fais que de la documentation, toujours en retard du coup mais vais pouvoir le rattraper demain</t>
+  </si>
+  <si>
+    <t>Réflexion sur les modèles et décision de ne pas en faire</t>
+  </si>
+  <si>
+    <t>Implémentation authentification github</t>
+  </si>
+  <si>
+    <t>Rendez-vous avec Meylan</t>
+  </si>
+  <si>
+    <t>Implémentation du service github</t>
+  </si>
+  <si>
+    <t>Service et endspoints projets</t>
+  </si>
+  <si>
+    <t>Je me suis rendu compte après implémentation des modèles qu'ils étaient en fait inutile, j'ai donc décider de les retiré du code. L'implementation de l'authentification via github fonctionne parfaitement, les endpoints de projet sont fait et la récuperation des fichiers et projets git hub aussi. Je rattrapes mon leger retard</t>
   </si>
 </sst>
 </file>
@@ -587,6 +605,10 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -604,13 +626,101 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
@@ -619,103 +729,11 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1309,7 +1327,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D87"/>
+  <dimension ref="A1:D89"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5703125" style="1"/>
@@ -1320,93 +1338,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
     </row>
     <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="47"/>
+      <c r="B2" s="42"/>
+      <c r="C2" s="43"/>
       <c r="D2" s="4">
         <v>151446</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="41"/>
+      <c r="C4" s="37"/>
       <c r="D4" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="42"/>
-      <c r="B5" s="42"/>
-      <c r="C5" s="43"/>
+      <c r="A5" s="38"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="39"/>
       <c r="D5" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="38">
+      <c r="A6" s="34">
         <v>46153</v>
       </c>
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="45"/>
+      <c r="C6" s="41"/>
       <c r="D6" s="7">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="19"/>
-      <c r="B7" s="26" t="s">
+      <c r="A7" s="20"/>
+      <c r="B7" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="23"/>
+      <c r="C7" s="24"/>
       <c r="D7" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="19"/>
-      <c r="B8" s="26" t="s">
+      <c r="A8" s="20"/>
+      <c r="B8" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="23"/>
+      <c r="C8" s="24"/>
       <c r="D8" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="19"/>
-      <c r="B9" s="36" t="s">
+      <c r="A9" s="20"/>
+      <c r="B9" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="37"/>
+      <c r="C9" s="45"/>
       <c r="D9" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="19"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="23"/>
+      <c r="A10" s="20"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="24"/>
       <c r="D10" s="8"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="19"/>
+      <c r="A11" s="20"/>
       <c r="B11" s="2" t="s">
         <v>6</v>
       </c>
@@ -1419,37 +1437,37 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="19"/>
-      <c r="B12" s="27" t="s">
+      <c r="A12" s="20"/>
+      <c r="B12" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="28"/>
-      <c r="D12" s="29"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="27"/>
     </row>
     <row r="13" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="18">
+      <c r="A13" s="19">
         <v>46154</v>
       </c>
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="21"/>
+      <c r="C13" s="22"/>
       <c r="D13" s="7">
         <v>0.5</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="19"/>
-      <c r="B14" s="26" t="s">
+      <c r="A14" s="20"/>
+      <c r="B14" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="23"/>
+      <c r="C14" s="24"/>
       <c r="D14" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="19"/>
+      <c r="A15" s="20"/>
       <c r="B15" s="13" t="s">
         <v>18</v>
       </c>
@@ -1458,23 +1476,23 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="19"/>
-      <c r="B16" s="26" t="s">
+      <c r="A16" s="20"/>
+      <c r="B16" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="23"/>
+      <c r="C16" s="24"/>
       <c r="D16" s="8">
         <v>1.5</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="19"/>
-      <c r="B17" s="26"/>
-      <c r="C17" s="23"/>
+      <c r="A17" s="20"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="24"/>
       <c r="D17" s="8"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="19"/>
+      <c r="A18" s="20"/>
       <c r="B18" s="2" t="s">
         <v>6</v>
       </c>
@@ -1487,75 +1505,75 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="19"/>
-      <c r="B19" s="27" t="s">
+      <c r="A19" s="20"/>
+      <c r="B19" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="28"/>
-      <c r="D19" s="29"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="27"/>
     </row>
     <row r="20" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="18">
+      <c r="A20" s="19">
         <v>46157</v>
       </c>
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="21"/>
+      <c r="C20" s="22"/>
       <c r="D20" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="19"/>
-      <c r="B21" s="22" t="s">
+      <c r="A21" s="20"/>
+      <c r="B21" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="23"/>
+      <c r="C21" s="24"/>
       <c r="D21" s="8">
         <v>2.5</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="19"/>
-      <c r="B22" s="24" t="s">
+      <c r="A22" s="20"/>
+      <c r="B22" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="25"/>
+      <c r="C22" s="48"/>
       <c r="D22" s="8"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="19"/>
-      <c r="B23" s="30" t="s">
+      <c r="A23" s="20"/>
+      <c r="B23" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="31"/>
+      <c r="C23" s="50"/>
       <c r="D23" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="19"/>
-      <c r="B24" s="26" t="s">
+      <c r="A24" s="20"/>
+      <c r="B24" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="23"/>
+      <c r="C24" s="24"/>
       <c r="D24" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="19"/>
-      <c r="B25" s="26" t="s">
+      <c r="A25" s="20"/>
+      <c r="B25" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="C25" s="23"/>
+      <c r="C25" s="24"/>
       <c r="D25" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="19"/>
+      <c r="A26" s="20"/>
       <c r="B26" s="2" t="s">
         <v>6</v>
       </c>
@@ -1568,57 +1586,57 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="19"/>
-      <c r="B27" s="27" t="s">
+      <c r="A27" s="20"/>
+      <c r="B27" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="28"/>
-      <c r="D27" s="29"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="27"/>
     </row>
     <row r="28" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="18">
+      <c r="A28" s="19">
         <v>46160</v>
       </c>
-      <c r="B28" s="20" t="s">
+      <c r="B28" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="21"/>
+      <c r="C28" s="22"/>
       <c r="D28" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="19"/>
-      <c r="B29" s="26" t="s">
+      <c r="A29" s="20"/>
+      <c r="B29" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="23"/>
+      <c r="C29" s="24"/>
       <c r="D29" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="19"/>
-      <c r="B30" s="26" t="s">
+      <c r="A30" s="20"/>
+      <c r="B30" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="23"/>
+      <c r="C30" s="24"/>
       <c r="D30" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="19"/>
-      <c r="B31" s="26" t="s">
+      <c r="A31" s="20"/>
+      <c r="B31" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="23"/>
+      <c r="C31" s="24"/>
       <c r="D31" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="19"/>
+      <c r="A32" s="20"/>
       <c r="B32" s="14" t="s">
         <v>31</v>
       </c>
@@ -1628,7 +1646,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="19"/>
+      <c r="A33" s="20"/>
       <c r="B33" s="14" t="s">
         <v>32</v>
       </c>
@@ -1638,17 +1656,17 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="19"/>
-      <c r="B34" s="26" t="s">
+      <c r="A34" s="20"/>
+      <c r="B34" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="23"/>
+      <c r="C34" s="24"/>
       <c r="D34" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="19"/>
+      <c r="A35" s="20"/>
       <c r="B35" s="2" t="s">
         <v>6</v>
       </c>
@@ -1661,15 +1679,15 @@
       </c>
     </row>
     <row r="36" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="35"/>
-      <c r="B36" s="32" t="s">
+      <c r="A36" s="28"/>
+      <c r="B36" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="C36" s="33"/>
-      <c r="D36" s="34"/>
+      <c r="C36" s="30"/>
+      <c r="D36" s="31"/>
     </row>
     <row r="37" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="18">
+      <c r="A37" s="19">
         <v>46161</v>
       </c>
       <c r="B37" s="16" t="s">
@@ -1681,43 +1699,43 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="19"/>
-      <c r="B38" s="49" t="s">
+      <c r="A38" s="20"/>
+      <c r="B38" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="C38" s="50"/>
+      <c r="C38" s="33"/>
       <c r="D38" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="19"/>
-      <c r="B39" s="26" t="s">
+      <c r="A39" s="20"/>
+      <c r="B39" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="C39" s="23"/>
+      <c r="C39" s="24"/>
       <c r="D39" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="19"/>
-      <c r="B40" s="26" t="s">
+      <c r="A40" s="20"/>
+      <c r="B40" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="23"/>
+      <c r="C40" s="24"/>
       <c r="D40" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="19"/>
-      <c r="B41" s="26"/>
-      <c r="C41" s="23"/>
+      <c r="A41" s="20"/>
+      <c r="B41" s="23"/>
+      <c r="C41" s="24"/>
       <c r="D41" s="8"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="19"/>
+      <c r="A42" s="20"/>
       <c r="B42" s="2" t="s">
         <v>6</v>
       </c>
@@ -1730,55 +1748,55 @@
       </c>
     </row>
     <row r="43" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="35"/>
-      <c r="B43" s="32" t="s">
+      <c r="A43" s="28"/>
+      <c r="B43" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C43" s="33"/>
-      <c r="D43" s="34"/>
+      <c r="C43" s="30"/>
+      <c r="D43" s="31"/>
     </row>
     <row r="44" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="18">
+      <c r="A44" s="19">
         <v>46163</v>
       </c>
-      <c r="B44" s="20" t="s">
+      <c r="B44" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="C44" s="21"/>
+      <c r="C44" s="22"/>
       <c r="D44" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="19"/>
-      <c r="B45" s="26" t="s">
+      <c r="A45" s="20"/>
+      <c r="B45" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="C45" s="23"/>
+      <c r="C45" s="24"/>
       <c r="D45" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="19"/>
-      <c r="B46" s="26"/>
-      <c r="C46" s="23"/>
+      <c r="A46" s="20"/>
+      <c r="B46" s="23"/>
+      <c r="C46" s="24"/>
       <c r="D46" s="8"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="19"/>
-      <c r="B47" s="26"/>
-      <c r="C47" s="23"/>
+      <c r="A47" s="20"/>
+      <c r="B47" s="23"/>
+      <c r="C47" s="24"/>
       <c r="D47" s="8"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="19"/>
-      <c r="B48" s="26"/>
-      <c r="C48" s="23"/>
+      <c r="A48" s="20"/>
+      <c r="B48" s="23"/>
+      <c r="C48" s="24"/>
       <c r="D48" s="8"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="19"/>
+      <c r="A49" s="20"/>
       <c r="B49" s="2" t="s">
         <v>6</v>
       </c>
@@ -1791,280 +1809,389 @@
       </c>
     </row>
     <row r="50" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="35"/>
-      <c r="B50" s="32" t="s">
+      <c r="A50" s="28"/>
+      <c r="B50" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C50" s="33"/>
-      <c r="D50" s="34"/>
+      <c r="C50" s="30"/>
+      <c r="D50" s="31"/>
     </row>
     <row r="51" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="18"/>
-      <c r="B51" s="20"/>
-      <c r="C51" s="21"/>
-      <c r="D51" s="7"/>
+      <c r="A51" s="19">
+        <v>46164</v>
+      </c>
+      <c r="B51" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="C51" s="22"/>
+      <c r="D51" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="19"/>
-      <c r="B52" s="26"/>
-      <c r="C52" s="23"/>
-      <c r="D52" s="8"/>
+      <c r="A52" s="20"/>
+      <c r="B52" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="C52" s="24"/>
+      <c r="D52" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="19"/>
-      <c r="B53" s="26"/>
-      <c r="C53" s="23"/>
-      <c r="D53" s="8"/>
+      <c r="A53" s="20"/>
+      <c r="B53" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="C53" s="24"/>
+      <c r="D53" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="19"/>
-      <c r="B54" s="26"/>
-      <c r="C54" s="23"/>
-      <c r="D54" s="8"/>
+      <c r="A54" s="20"/>
+      <c r="B54" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="C54" s="24"/>
+      <c r="D54" s="8">
+        <v>2</v>
+      </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" s="19"/>
-      <c r="B55" s="26"/>
-      <c r="C55" s="23"/>
-      <c r="D55" s="8"/>
+      <c r="A55" s="20"/>
+      <c r="B55" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="C55" s="24"/>
+      <c r="D55" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="19"/>
-      <c r="B56" s="2" t="s">
+      <c r="A56" s="20"/>
+      <c r="B56" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C56" s="15"/>
+      <c r="D56" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" s="20"/>
+      <c r="B57" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C57" s="15"/>
+      <c r="D57" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" s="20"/>
+      <c r="B58" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C56" s="3" t="s">
+      <c r="C58" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D56" s="9">
-        <f>SUM(D51:D55)</f>
+      <c r="D58" s="9">
+        <f>SUM(D51:D57)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="28"/>
+      <c r="B59" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="C59" s="30"/>
+      <c r="D59" s="31"/>
+    </row>
+    <row r="60" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="19"/>
+      <c r="B60" s="21"/>
+      <c r="C60" s="22"/>
+      <c r="D60" s="7"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" s="20"/>
+      <c r="B61" s="23"/>
+      <c r="C61" s="24"/>
+      <c r="D61" s="8"/>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" s="20"/>
+      <c r="B62" s="23"/>
+      <c r="C62" s="24"/>
+      <c r="D62" s="8"/>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" s="20"/>
+      <c r="B63" s="23"/>
+      <c r="C63" s="24"/>
+      <c r="D63" s="8"/>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" s="20"/>
+      <c r="B64" s="23"/>
+      <c r="C64" s="24"/>
+      <c r="D64" s="8"/>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" s="20"/>
+      <c r="B65" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D65" s="9">
+        <f>SUM(D60:D64)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="35"/>
-      <c r="B57" s="32"/>
-      <c r="C57" s="33"/>
-      <c r="D57" s="34"/>
-    </row>
-    <row r="58" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="18"/>
-      <c r="B58" s="20"/>
-      <c r="C58" s="21"/>
-      <c r="D58" s="7"/>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A59" s="19"/>
-      <c r="B59" s="26"/>
-      <c r="C59" s="23"/>
-      <c r="D59" s="8"/>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" s="19"/>
-      <c r="B60" s="26"/>
-      <c r="C60" s="23"/>
-      <c r="D60" s="8"/>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" s="19"/>
-      <c r="B61" s="26"/>
-      <c r="C61" s="23"/>
-      <c r="D61" s="8"/>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="19"/>
-      <c r="B62" s="26"/>
-      <c r="C62" s="23"/>
-      <c r="D62" s="8"/>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="19"/>
-      <c r="B63" s="2" t="s">
+    <row r="66" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="28"/>
+      <c r="B66" s="29"/>
+      <c r="C66" s="30"/>
+      <c r="D66" s="31"/>
+    </row>
+    <row r="67" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="19"/>
+      <c r="B67" s="21"/>
+      <c r="C67" s="22"/>
+      <c r="D67" s="7"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" s="20"/>
+      <c r="B68" s="23"/>
+      <c r="C68" s="24"/>
+      <c r="D68" s="8"/>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A69" s="20"/>
+      <c r="B69" s="23"/>
+      <c r="C69" s="24"/>
+      <c r="D69" s="8"/>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" s="20"/>
+      <c r="B70" s="23"/>
+      <c r="C70" s="24"/>
+      <c r="D70" s="8"/>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A71" s="20"/>
+      <c r="B71" s="23"/>
+      <c r="C71" s="24"/>
+      <c r="D71" s="8"/>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A72" s="20"/>
+      <c r="B72" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C63" s="3" t="s">
+      <c r="C72" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D63" s="9">
-        <f>SUM(D58:D62)</f>
+      <c r="D72" s="9">
+        <f>SUM(D67:D71)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="35"/>
-      <c r="B64" s="32"/>
-      <c r="C64" s="33"/>
-      <c r="D64" s="34"/>
-    </row>
-    <row r="65" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="18"/>
-      <c r="B65" s="20"/>
-      <c r="C65" s="21"/>
-      <c r="D65" s="7"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" s="19"/>
-      <c r="B66" s="26"/>
-      <c r="C66" s="23"/>
-      <c r="D66" s="8"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="19"/>
-      <c r="B67" s="26"/>
-      <c r="C67" s="23"/>
-      <c r="D67" s="8"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="19"/>
-      <c r="B68" s="26"/>
-      <c r="C68" s="23"/>
-      <c r="D68" s="8"/>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="19"/>
-      <c r="B69" s="26"/>
-      <c r="C69" s="23"/>
-      <c r="D69" s="8"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="19"/>
-      <c r="B70" s="2" t="s">
+    <row r="73" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="20"/>
+      <c r="B73" s="25"/>
+      <c r="C73" s="26"/>
+      <c r="D73" s="27"/>
+    </row>
+    <row r="74" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="19"/>
+      <c r="B74" s="21"/>
+      <c r="C74" s="22"/>
+      <c r="D74" s="7"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" s="20"/>
+      <c r="B75" s="23"/>
+      <c r="C75" s="24"/>
+      <c r="D75" s="8"/>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" s="20"/>
+      <c r="B76" s="23"/>
+      <c r="C76" s="24"/>
+      <c r="D76" s="8"/>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" s="20"/>
+      <c r="B77" s="23"/>
+      <c r="C77" s="24"/>
+      <c r="D77" s="8"/>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" s="20"/>
+      <c r="B78" s="23"/>
+      <c r="C78" s="24"/>
+      <c r="D78" s="8"/>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" s="20"/>
+      <c r="B79" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C70" s="3" t="s">
+      <c r="C79" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D70" s="9">
-        <f>SUM(D65:D69)</f>
+      <c r="D79" s="9">
+        <f>SUM(D74:D78)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="19"/>
-      <c r="B71" s="27"/>
-      <c r="C71" s="28"/>
-      <c r="D71" s="29"/>
-    </row>
-    <row r="72" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="18"/>
-      <c r="B72" s="20"/>
-      <c r="C72" s="21"/>
-      <c r="D72" s="7"/>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" s="19"/>
-      <c r="B73" s="26"/>
-      <c r="C73" s="23"/>
-      <c r="D73" s="8"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="19"/>
-      <c r="B74" s="26"/>
-      <c r="C74" s="23"/>
-      <c r="D74" s="8"/>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="19"/>
-      <c r="B75" s="26"/>
-      <c r="C75" s="23"/>
-      <c r="D75" s="8"/>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="19"/>
-      <c r="B76" s="26"/>
-      <c r="C76" s="23"/>
-      <c r="D76" s="8"/>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="19"/>
-      <c r="B77" s="2" t="s">
+    <row r="80" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A80" s="28"/>
+      <c r="B80" s="29"/>
+      <c r="C80" s="30"/>
+      <c r="D80" s="31"/>
+    </row>
+    <row r="81" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="19"/>
+      <c r="B81" s="21"/>
+      <c r="C81" s="22"/>
+      <c r="D81" s="7"/>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" s="20"/>
+      <c r="B82" s="23"/>
+      <c r="C82" s="24"/>
+      <c r="D82" s="8"/>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" s="20"/>
+      <c r="B83" s="23"/>
+      <c r="C83" s="24"/>
+      <c r="D83" s="8"/>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A84" s="20"/>
+      <c r="B84" s="23"/>
+      <c r="C84" s="24"/>
+      <c r="D84" s="8"/>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A85" s="20"/>
+      <c r="B85" s="23"/>
+      <c r="C85" s="24"/>
+      <c r="D85" s="8"/>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A86" s="20"/>
+      <c r="B86" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C77" s="3" t="s">
+      <c r="C86" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D77" s="9">
-        <f>SUM(D72:D76)</f>
+      <c r="D86" s="9">
+        <f>SUM(D81:D85)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="35"/>
-      <c r="B78" s="32"/>
-      <c r="C78" s="33"/>
-      <c r="D78" s="34"/>
-    </row>
-    <row r="79" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="18"/>
-      <c r="B79" s="20"/>
-      <c r="C79" s="21"/>
-      <c r="D79" s="7"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" s="19"/>
-      <c r="B80" s="26"/>
-      <c r="C80" s="23"/>
-      <c r="D80" s="8"/>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A81" s="19"/>
-      <c r="B81" s="26"/>
-      <c r="C81" s="23"/>
-      <c r="D81" s="8"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" s="19"/>
-      <c r="B82" s="26"/>
-      <c r="C82" s="23"/>
-      <c r="D82" s="8"/>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" s="19"/>
-      <c r="B83" s="26"/>
-      <c r="C83" s="23"/>
-      <c r="D83" s="8"/>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="19"/>
-      <c r="B84" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C84" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D84" s="9">
-        <f>SUM(D79:D83)</f>
+    <row r="87" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A87" s="28"/>
+      <c r="B87" s="29"/>
+      <c r="C87" s="30"/>
+      <c r="D87" s="31"/>
+    </row>
+    <row r="88" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A88" s="11"/>
+      <c r="B88" s="10"/>
+      <c r="C88" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D88" s="12">
+        <f>D11+D18+D26+D35+D42+D49+D58+D65+D72+D79+D86</f>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A89" s="18" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="85" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="35"/>
-      <c r="B85" s="32"/>
-      <c r="C85" s="33"/>
-      <c r="D85" s="34"/>
-    </row>
-    <row r="86" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="11"/>
-      <c r="B86" s="10"/>
-      <c r="C86" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D86" s="12">
-        <f>D11+D18+D26+D35+D42+D49+D56+D63+D70+D77+D84</f>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A87" s="48" t="s">
-        <v>0</v>
-      </c>
-      <c r="B87" s="48"/>
-      <c r="C87" s="48"/>
-      <c r="D87" s="48"/>
+      <c r="B89" s="18"/>
+      <c r="C89" s="18"/>
+      <c r="D89" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="81">
-    <mergeCell ref="A87:D87"/>
+    <mergeCell ref="A20:A27"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="A81:A87"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B87:D87"/>
+    <mergeCell ref="A51:A59"/>
+    <mergeCell ref="A74:A80"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="B78:C78"/>
+    <mergeCell ref="B80:D80"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="A60:A66"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="A44:A50"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="A67:A73"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="B68:C68"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B73:D73"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="A6:A12"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B4:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A89:D89"/>
     <mergeCell ref="A13:A19"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
@@ -2080,71 +2207,6 @@
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="A37:A43"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="A6:A12"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B4:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A65:A71"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="B68:C68"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="B71:D71"/>
-    <mergeCell ref="A44:A50"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="A51:A57"/>
-    <mergeCell ref="A72:A78"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="B75:C75"/>
-    <mergeCell ref="B76:C76"/>
-    <mergeCell ref="B78:D78"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B57:D57"/>
-    <mergeCell ref="A58:A64"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="A79:A85"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="B80:C80"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B85:D85"/>
-    <mergeCell ref="B59:C59"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="A20:A27"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B23:C23"/>
   </mergeCells>
   <conditionalFormatting sqref="D6:D11 D13:D14 D16:D18 D20:D23 D25:D26">
     <cfRule type="containsText" dxfId="19" priority="23" operator="containsText" text="Terminé">
@@ -2178,7 +2240,7 @@
       <formula>NOT(ISERROR(SEARCH("En cours",D44)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D51:D56">
+  <conditionalFormatting sqref="D51:D58">
     <cfRule type="containsText" dxfId="11" priority="7" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D51)))</formula>
     </cfRule>
@@ -2186,44 +2248,44 @@
       <formula>NOT(ISERROR(SEARCH("En cours",D51)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D58:D63">
+  <conditionalFormatting sqref="D60:D65">
     <cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D58)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D60)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="8" priority="6" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D58)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D60)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D65:D70">
+  <conditionalFormatting sqref="D67:D72">
     <cfRule type="containsText" dxfId="7" priority="15" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D65)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D67)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="6" priority="16" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D65)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D67)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D72:D77">
+  <conditionalFormatting sqref="D74:D79">
     <cfRule type="containsText" dxfId="5" priority="13" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D72)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D74)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="4" priority="14" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D72)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D74)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D79:D84">
+  <conditionalFormatting sqref="D81:D86">
     <cfRule type="containsText" dxfId="3" priority="11" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D79)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D81)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="2" priority="12" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D79)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D81)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D86">
+  <conditionalFormatting sqref="D88">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D86)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D88)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D86)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D88)))</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
@@ -2236,7 +2298,7 @@
   </headerFooter>
   <rowBreaks count="2" manualBreakCount="2">
     <brk id="50" max="16383" man="1"/>
-    <brk id="86" max="3" man="1"/>
+    <brk id="88" max="3" man="1"/>
   </rowBreaks>
   <legacyDrawingHF r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(server): pipeline d'analyse complet et documentation Swagger
- Pipeline d'analyse fonctionnel (création, exécution, résultats)
- Documentation Swagger des routes
- Suppression des modèles inutilisés
- Mise à jour du journal, du planning et du rapport
</commit_message>
<xml_diff>
--- a/doc/GAMEZ_Journal.xlsx
+++ b/doc/GAMEZ_Journal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/thibaudfrederic_gamez_studentfr_ch/Documents/TPI/tpi2026-codementor/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="144" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2BA4BDF-C0F2-4C4A-8205-E3EDB440E1B7}"/>
+  <xr:revisionPtr revIDLastSave="153" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69EF6B18-716C-4D1C-A2E6-3717D768DB96}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="51">
   <si>
     <t>Insérer les lignes au-dessus de celle-ci !</t>
   </si>
@@ -220,6 +220,12 @@
   </si>
   <si>
     <t>Je me suis rendu compte après implémentation des modèles qu'ils étaient en fait inutile, j'ai donc décider de les retiré du code. L'implementation de l'authentification via github fonctionne parfaitement, les endpoints de projet sont fait et la récuperation des fichiers et projets git hub aussi. Je rattrapes mon leger retard</t>
+  </si>
+  <si>
+    <t>Mise en place de la queue en mémoire</t>
+  </si>
+  <si>
+    <t>Mise en place de l'analyse via le LLM</t>
   </si>
 </sst>
 </file>
@@ -605,135 +611,135 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1338,93 +1344,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
     </row>
     <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="43"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="47"/>
       <c r="D2" s="4">
         <v>151446</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="37"/>
+      <c r="C4" s="41"/>
       <c r="D4" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="38"/>
-      <c r="B5" s="38"/>
-      <c r="C5" s="39"/>
+      <c r="A5" s="42"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="43"/>
       <c r="D5" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="34">
+      <c r="A6" s="38">
         <v>46153</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="41"/>
+      <c r="C6" s="45"/>
       <c r="D6" s="7">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="20"/>
-      <c r="B7" s="23" t="s">
+      <c r="A7" s="19"/>
+      <c r="B7" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="24"/>
+      <c r="C7" s="23"/>
       <c r="D7" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="20"/>
-      <c r="B8" s="23" t="s">
+      <c r="A8" s="19"/>
+      <c r="B8" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="24"/>
+      <c r="C8" s="23"/>
       <c r="D8" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="20"/>
-      <c r="B9" s="44" t="s">
+      <c r="A9" s="19"/>
+      <c r="B9" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="45"/>
+      <c r="C9" s="37"/>
       <c r="D9" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="20"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="24"/>
+      <c r="A10" s="19"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="23"/>
       <c r="D10" s="8"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="20"/>
+      <c r="A11" s="19"/>
       <c r="B11" s="2" t="s">
         <v>6</v>
       </c>
@@ -1437,37 +1443,37 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="20"/>
-      <c r="B12" s="25" t="s">
+      <c r="A12" s="19"/>
+      <c r="B12" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="26"/>
-      <c r="D12" s="27"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="29"/>
     </row>
     <row r="13" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="19">
+      <c r="A13" s="18">
         <v>46154</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="22"/>
+      <c r="C13" s="21"/>
       <c r="D13" s="7">
         <v>0.5</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="20"/>
-      <c r="B14" s="23" t="s">
+      <c r="A14" s="19"/>
+      <c r="B14" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="24"/>
+      <c r="C14" s="23"/>
       <c r="D14" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="20"/>
+      <c r="A15" s="19"/>
       <c r="B15" s="13" t="s">
         <v>18</v>
       </c>
@@ -1476,23 +1482,23 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="20"/>
-      <c r="B16" s="23" t="s">
+      <c r="A16" s="19"/>
+      <c r="B16" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="24"/>
+      <c r="C16" s="23"/>
       <c r="D16" s="8">
         <v>1.5</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="20"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="24"/>
+      <c r="A17" s="19"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="23"/>
       <c r="D17" s="8"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="20"/>
+      <c r="A18" s="19"/>
       <c r="B18" s="2" t="s">
         <v>6</v>
       </c>
@@ -1505,75 +1511,75 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="20"/>
-      <c r="B19" s="25" t="s">
+      <c r="A19" s="19"/>
+      <c r="B19" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="26"/>
-      <c r="D19" s="27"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="29"/>
     </row>
     <row r="20" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="19">
+      <c r="A20" s="18">
         <v>46157</v>
       </c>
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="22"/>
+      <c r="C20" s="21"/>
       <c r="D20" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="20"/>
-      <c r="B21" s="46" t="s">
+      <c r="A21" s="19"/>
+      <c r="B21" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="24"/>
+      <c r="C21" s="23"/>
       <c r="D21" s="8">
         <v>2.5</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="20"/>
-      <c r="B22" s="47" t="s">
+      <c r="A22" s="19"/>
+      <c r="B22" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="48"/>
+      <c r="C22" s="25"/>
       <c r="D22" s="8"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="20"/>
-      <c r="B23" s="49" t="s">
+      <c r="A23" s="19"/>
+      <c r="B23" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="50"/>
+      <c r="C23" s="31"/>
       <c r="D23" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="20"/>
-      <c r="B24" s="23" t="s">
+      <c r="A24" s="19"/>
+      <c r="B24" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="24"/>
+      <c r="C24" s="23"/>
       <c r="D24" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="20"/>
-      <c r="B25" s="23" t="s">
+      <c r="A25" s="19"/>
+      <c r="B25" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="C25" s="24"/>
+      <c r="C25" s="23"/>
       <c r="D25" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="20"/>
+      <c r="A26" s="19"/>
       <c r="B26" s="2" t="s">
         <v>6</v>
       </c>
@@ -1586,57 +1592,57 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="20"/>
-      <c r="B27" s="25" t="s">
+      <c r="A27" s="19"/>
+      <c r="B27" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="26"/>
-      <c r="D27" s="27"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="29"/>
     </row>
     <row r="28" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="19">
+      <c r="A28" s="18">
         <v>46160</v>
       </c>
-      <c r="B28" s="21" t="s">
+      <c r="B28" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="22"/>
+      <c r="C28" s="21"/>
       <c r="D28" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="20"/>
-      <c r="B29" s="23" t="s">
+      <c r="A29" s="19"/>
+      <c r="B29" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="24"/>
+      <c r="C29" s="23"/>
       <c r="D29" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="20"/>
-      <c r="B30" s="23" t="s">
+      <c r="A30" s="19"/>
+      <c r="B30" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="24"/>
+      <c r="C30" s="23"/>
       <c r="D30" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="20"/>
-      <c r="B31" s="23" t="s">
+      <c r="A31" s="19"/>
+      <c r="B31" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="24"/>
+      <c r="C31" s="23"/>
       <c r="D31" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="20"/>
+      <c r="A32" s="19"/>
       <c r="B32" s="14" t="s">
         <v>31</v>
       </c>
@@ -1646,7 +1652,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="20"/>
+      <c r="A33" s="19"/>
       <c r="B33" s="14" t="s">
         <v>32</v>
       </c>
@@ -1656,17 +1662,17 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="20"/>
-      <c r="B34" s="23" t="s">
+      <c r="A34" s="19"/>
+      <c r="B34" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="24"/>
+      <c r="C34" s="23"/>
       <c r="D34" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="20"/>
+      <c r="A35" s="19"/>
       <c r="B35" s="2" t="s">
         <v>6</v>
       </c>
@@ -1679,15 +1685,15 @@
       </c>
     </row>
     <row r="36" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="28"/>
-      <c r="B36" s="29" t="s">
+      <c r="A36" s="35"/>
+      <c r="B36" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="C36" s="30"/>
-      <c r="D36" s="31"/>
+      <c r="C36" s="33"/>
+      <c r="D36" s="34"/>
     </row>
     <row r="37" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="19">
+      <c r="A37" s="18">
         <v>46161</v>
       </c>
       <c r="B37" s="16" t="s">
@@ -1699,43 +1705,43 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="20"/>
-      <c r="B38" s="32" t="s">
+      <c r="A38" s="19"/>
+      <c r="B38" s="49" t="s">
         <v>36</v>
       </c>
-      <c r="C38" s="33"/>
+      <c r="C38" s="50"/>
       <c r="D38" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="20"/>
-      <c r="B39" s="23" t="s">
+      <c r="A39" s="19"/>
+      <c r="B39" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="C39" s="24"/>
+      <c r="C39" s="23"/>
       <c r="D39" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="20"/>
-      <c r="B40" s="23" t="s">
+      <c r="A40" s="19"/>
+      <c r="B40" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="24"/>
+      <c r="C40" s="23"/>
       <c r="D40" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="20"/>
-      <c r="B41" s="23"/>
-      <c r="C41" s="24"/>
+      <c r="A41" s="19"/>
+      <c r="B41" s="26"/>
+      <c r="C41" s="23"/>
       <c r="D41" s="8"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="20"/>
+      <c r="A42" s="19"/>
       <c r="B42" s="2" t="s">
         <v>6</v>
       </c>
@@ -1748,55 +1754,55 @@
       </c>
     </row>
     <row r="43" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="28"/>
-      <c r="B43" s="29" t="s">
+      <c r="A43" s="35"/>
+      <c r="B43" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="C43" s="30"/>
-      <c r="D43" s="31"/>
+      <c r="C43" s="33"/>
+      <c r="D43" s="34"/>
     </row>
     <row r="44" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="19">
+      <c r="A44" s="18">
         <v>46163</v>
       </c>
-      <c r="B44" s="21" t="s">
+      <c r="B44" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="C44" s="22"/>
+      <c r="C44" s="21"/>
       <c r="D44" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="20"/>
-      <c r="B45" s="23" t="s">
+      <c r="A45" s="19"/>
+      <c r="B45" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="C45" s="24"/>
+      <c r="C45" s="23"/>
       <c r="D45" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="20"/>
-      <c r="B46" s="23"/>
-      <c r="C46" s="24"/>
+      <c r="A46" s="19"/>
+      <c r="B46" s="26"/>
+      <c r="C46" s="23"/>
       <c r="D46" s="8"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="20"/>
-      <c r="B47" s="23"/>
-      <c r="C47" s="24"/>
+      <c r="A47" s="19"/>
+      <c r="B47" s="26"/>
+      <c r="C47" s="23"/>
       <c r="D47" s="8"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="20"/>
-      <c r="B48" s="23"/>
-      <c r="C48" s="24"/>
+      <c r="A48" s="19"/>
+      <c r="B48" s="26"/>
+      <c r="C48" s="23"/>
       <c r="D48" s="8"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="20"/>
+      <c r="A49" s="19"/>
       <c r="B49" s="2" t="s">
         <v>6</v>
       </c>
@@ -1809,67 +1815,67 @@
       </c>
     </row>
     <row r="50" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="28"/>
-      <c r="B50" s="29" t="s">
+      <c r="A50" s="35"/>
+      <c r="B50" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="C50" s="30"/>
-      <c r="D50" s="31"/>
+      <c r="C50" s="33"/>
+      <c r="D50" s="34"/>
     </row>
     <row r="51" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="19">
+      <c r="A51" s="18">
         <v>46164</v>
       </c>
-      <c r="B51" s="21" t="s">
+      <c r="B51" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="C51" s="22"/>
+      <c r="C51" s="21"/>
       <c r="D51" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="20"/>
-      <c r="B52" s="23" t="s">
+      <c r="A52" s="19"/>
+      <c r="B52" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="C52" s="24"/>
+      <c r="C52" s="23"/>
       <c r="D52" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="20"/>
-      <c r="B53" s="23" t="s">
+      <c r="A53" s="19"/>
+      <c r="B53" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="C53" s="24"/>
+      <c r="C53" s="23"/>
       <c r="D53" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="20"/>
-      <c r="B54" s="23" t="s">
+      <c r="A54" s="19"/>
+      <c r="B54" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="C54" s="24"/>
+      <c r="C54" s="23"/>
       <c r="D54" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" s="20"/>
-      <c r="B55" s="23" t="s">
+      <c r="A55" s="19"/>
+      <c r="B55" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="C55" s="24"/>
+      <c r="C55" s="23"/>
       <c r="D55" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="20"/>
+      <c r="A56" s="19"/>
       <c r="B56" s="14" t="s">
         <v>38</v>
       </c>
@@ -1879,7 +1885,7 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" s="20"/>
+      <c r="A57" s="19"/>
       <c r="B57" s="14" t="s">
         <v>46</v>
       </c>
@@ -1889,7 +1895,7 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" s="20"/>
+      <c r="A58" s="19"/>
       <c r="B58" s="2" t="s">
         <v>6</v>
       </c>
@@ -1901,46 +1907,56 @@
         <v>8</v>
       </c>
     </row>
-    <row r="59" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="28"/>
-      <c r="B59" s="29" t="s">
+    <row r="59" spans="1:4" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="35"/>
+      <c r="B59" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="C59" s="30"/>
-      <c r="D59" s="31"/>
+      <c r="C59" s="33"/>
+      <c r="D59" s="34"/>
     </row>
     <row r="60" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="19"/>
-      <c r="B60" s="21"/>
-      <c r="C60" s="22"/>
-      <c r="D60" s="7"/>
+      <c r="A60" s="18">
+        <v>46171</v>
+      </c>
+      <c r="B60" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C60" s="21"/>
+      <c r="D60" s="7">
+        <v>2</v>
+      </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" s="20"/>
-      <c r="B61" s="23"/>
-      <c r="C61" s="24"/>
-      <c r="D61" s="8"/>
+      <c r="A61" s="19"/>
+      <c r="B61" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="C61" s="23"/>
+      <c r="D61" s="8">
+        <v>2</v>
+      </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="20"/>
-      <c r="B62" s="23"/>
-      <c r="C62" s="24"/>
+      <c r="A62" s="19"/>
+      <c r="B62" s="26"/>
+      <c r="C62" s="23"/>
       <c r="D62" s="8"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="20"/>
-      <c r="B63" s="23"/>
-      <c r="C63" s="24"/>
+      <c r="A63" s="19"/>
+      <c r="B63" s="26"/>
+      <c r="C63" s="23"/>
       <c r="D63" s="8"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="20"/>
-      <c r="B64" s="23"/>
-      <c r="C64" s="24"/>
+      <c r="A64" s="19"/>
+      <c r="B64" s="26"/>
+      <c r="C64" s="23"/>
       <c r="D64" s="8"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" s="20"/>
+      <c r="A65" s="19"/>
       <c r="B65" s="2" t="s">
         <v>6</v>
       </c>
@@ -1949,47 +1965,47 @@
       </c>
       <c r="D65" s="9">
         <f>SUM(D60:D64)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="28"/>
-      <c r="B66" s="29"/>
-      <c r="C66" s="30"/>
-      <c r="D66" s="31"/>
+      <c r="A66" s="35"/>
+      <c r="B66" s="32"/>
+      <c r="C66" s="33"/>
+      <c r="D66" s="34"/>
     </row>
     <row r="67" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="19"/>
-      <c r="B67" s="21"/>
-      <c r="C67" s="22"/>
+      <c r="A67" s="18"/>
+      <c r="B67" s="20"/>
+      <c r="C67" s="21"/>
       <c r="D67" s="7"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="20"/>
-      <c r="B68" s="23"/>
-      <c r="C68" s="24"/>
+      <c r="A68" s="19"/>
+      <c r="B68" s="26"/>
+      <c r="C68" s="23"/>
       <c r="D68" s="8"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="20"/>
-      <c r="B69" s="23"/>
-      <c r="C69" s="24"/>
+      <c r="A69" s="19"/>
+      <c r="B69" s="26"/>
+      <c r="C69" s="23"/>
       <c r="D69" s="8"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="20"/>
-      <c r="B70" s="23"/>
-      <c r="C70" s="24"/>
+      <c r="A70" s="19"/>
+      <c r="B70" s="26"/>
+      <c r="C70" s="23"/>
       <c r="D70" s="8"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" s="20"/>
-      <c r="B71" s="23"/>
-      <c r="C71" s="24"/>
+      <c r="A71" s="19"/>
+      <c r="B71" s="26"/>
+      <c r="C71" s="23"/>
       <c r="D71" s="8"/>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="20"/>
+      <c r="A72" s="19"/>
       <c r="B72" s="2" t="s">
         <v>6</v>
       </c>
@@ -2002,43 +2018,43 @@
       </c>
     </row>
     <row r="73" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="20"/>
-      <c r="B73" s="25"/>
-      <c r="C73" s="26"/>
-      <c r="D73" s="27"/>
+      <c r="A73" s="19"/>
+      <c r="B73" s="27"/>
+      <c r="C73" s="28"/>
+      <c r="D73" s="29"/>
     </row>
     <row r="74" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="19"/>
-      <c r="B74" s="21"/>
-      <c r="C74" s="22"/>
+      <c r="A74" s="18"/>
+      <c r="B74" s="20"/>
+      <c r="C74" s="21"/>
       <c r="D74" s="7"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="20"/>
-      <c r="B75" s="23"/>
-      <c r="C75" s="24"/>
+      <c r="A75" s="19"/>
+      <c r="B75" s="26"/>
+      <c r="C75" s="23"/>
       <c r="D75" s="8"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="20"/>
-      <c r="B76" s="23"/>
-      <c r="C76" s="24"/>
+      <c r="A76" s="19"/>
+      <c r="B76" s="26"/>
+      <c r="C76" s="23"/>
       <c r="D76" s="8"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="20"/>
-      <c r="B77" s="23"/>
-      <c r="C77" s="24"/>
+      <c r="A77" s="19"/>
+      <c r="B77" s="26"/>
+      <c r="C77" s="23"/>
       <c r="D77" s="8"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="20"/>
-      <c r="B78" s="23"/>
-      <c r="C78" s="24"/>
+      <c r="A78" s="19"/>
+      <c r="B78" s="26"/>
+      <c r="C78" s="23"/>
       <c r="D78" s="8"/>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="20"/>
+      <c r="A79" s="19"/>
       <c r="B79" s="2" t="s">
         <v>6</v>
       </c>
@@ -2051,43 +2067,43 @@
       </c>
     </row>
     <row r="80" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="28"/>
-      <c r="B80" s="29"/>
-      <c r="C80" s="30"/>
-      <c r="D80" s="31"/>
+      <c r="A80" s="35"/>
+      <c r="B80" s="32"/>
+      <c r="C80" s="33"/>
+      <c r="D80" s="34"/>
     </row>
     <row r="81" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="19"/>
-      <c r="B81" s="21"/>
-      <c r="C81" s="22"/>
+      <c r="A81" s="18"/>
+      <c r="B81" s="20"/>
+      <c r="C81" s="21"/>
       <c r="D81" s="7"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" s="20"/>
-      <c r="B82" s="23"/>
-      <c r="C82" s="24"/>
+      <c r="A82" s="19"/>
+      <c r="B82" s="26"/>
+      <c r="C82" s="23"/>
       <c r="D82" s="8"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" s="20"/>
-      <c r="B83" s="23"/>
-      <c r="C83" s="24"/>
+      <c r="A83" s="19"/>
+      <c r="B83" s="26"/>
+      <c r="C83" s="23"/>
       <c r="D83" s="8"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="20"/>
-      <c r="B84" s="23"/>
-      <c r="C84" s="24"/>
+      <c r="A84" s="19"/>
+      <c r="B84" s="26"/>
+      <c r="C84" s="23"/>
       <c r="D84" s="8"/>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A85" s="20"/>
-      <c r="B85" s="23"/>
-      <c r="C85" s="24"/>
+      <c r="A85" s="19"/>
+      <c r="B85" s="26"/>
+      <c r="C85" s="23"/>
       <c r="D85" s="8"/>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A86" s="20"/>
+      <c r="A86" s="19"/>
       <c r="B86" s="2" t="s">
         <v>6</v>
       </c>
@@ -2100,10 +2116,10 @@
       </c>
     </row>
     <row r="87" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A87" s="28"/>
-      <c r="B87" s="29"/>
-      <c r="C87" s="30"/>
-      <c r="D87" s="31"/>
+      <c r="A87" s="35"/>
+      <c r="B87" s="32"/>
+      <c r="C87" s="33"/>
+      <c r="D87" s="34"/>
     </row>
     <row r="88" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="11"/>
@@ -2113,39 +2129,64 @@
       </c>
       <c r="D88" s="12">
         <f>D11+D18+D26+D35+D42+D49+D58+D65+D72+D79+D86</f>
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A89" s="18" t="s">
+      <c r="A89" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B89" s="18"/>
-      <c r="C89" s="18"/>
-      <c r="D89" s="18"/>
+      <c r="B89" s="48"/>
+      <c r="C89" s="48"/>
+      <c r="D89" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="81">
-    <mergeCell ref="A20:A27"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="B66:D66"/>
-    <mergeCell ref="A81:A87"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="B87:D87"/>
+    <mergeCell ref="A89:D89"/>
+    <mergeCell ref="A13:A19"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="A28:A36"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="A37:A43"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="A6:A12"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B4:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="A67:A73"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="B68:C68"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B73:D73"/>
+    <mergeCell ref="A44:A50"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B50:D50"/>
     <mergeCell ref="A51:A59"/>
     <mergeCell ref="A74:A80"/>
     <mergeCell ref="B74:C74"/>
@@ -2162,51 +2203,26 @@
     <mergeCell ref="B59:D59"/>
     <mergeCell ref="A60:A66"/>
     <mergeCell ref="B60:C60"/>
-    <mergeCell ref="A44:A50"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="A67:A73"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="B68:C68"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B73:D73"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A6:A12"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B4:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A89:D89"/>
-    <mergeCell ref="A13:A19"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A28:A36"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="A37:A43"/>
-    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="A81:A87"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B87:D87"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="B66:D66"/>
+    <mergeCell ref="A20:A27"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B23:C23"/>
   </mergeCells>
   <conditionalFormatting sqref="D6:D11 D13:D14 D16:D18 D20:D23 D25:D26">
     <cfRule type="containsText" dxfId="19" priority="23" operator="containsText" text="Terminé">

</xml_diff>

<commit_message>
docs: mise à jour du planning
</commit_message>
<xml_diff>
--- a/doc/GAMEZ_Journal.xlsx
+++ b/doc/GAMEZ_Journal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/thibaudfrederic_gamez_studentfr_ch/Documents/TPI/tpi2026-codementor/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="153" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69EF6B18-716C-4D1C-A2E6-3717D768DB96}"/>
+  <xr:revisionPtr revIDLastSave="176" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6544A02D-3E1F-4D6C-AFFA-6E8542C90FAB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="8" r:id="rId1"/>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Journal!$A$5:$HI$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Journal!$B:$D,Journal!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$D$88</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$D$91</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="57">
   <si>
     <t>Insérer les lignes au-dessus de celle-ci !</t>
   </si>
@@ -226,6 +226,24 @@
   </si>
   <si>
     <t>Mise en place de l'analyse via le LLM</t>
+  </si>
+  <si>
+    <t>Endpoint de suivi d'état des tâches</t>
+  </si>
+  <si>
+    <t>Documentation swagger</t>
+  </si>
+  <si>
+    <t>Rendez-vous avec les experts</t>
+  </si>
+  <si>
+    <t>Sécurisation des accès (projet / analyse)</t>
+  </si>
+  <si>
+    <t>Système prompt llm</t>
+  </si>
+  <si>
+    <t>La journée s'est bien passé, les différents endpoints fonctionnes et je suis confiant pour la suite</t>
   </si>
 </sst>
 </file>
@@ -545,7 +563,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -611,6 +629,11 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -628,13 +651,101 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
@@ -643,103 +754,11 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -747,29 +766,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="18">
     <dxf>
       <font>
         <strike val="0"/>
@@ -1333,7 +1330,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D89"/>
+  <dimension ref="A1:D92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5703125" style="1"/>
@@ -1344,93 +1341,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
     </row>
     <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="47"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="44"/>
       <c r="D2" s="4">
         <v>151446</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="41"/>
+      <c r="C4" s="38"/>
       <c r="D4" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="42"/>
-      <c r="B5" s="42"/>
-      <c r="C5" s="43"/>
+      <c r="A5" s="39"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="40"/>
       <c r="D5" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="38">
+      <c r="A6" s="35">
         <v>46153</v>
       </c>
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="45"/>
+      <c r="C6" s="42"/>
       <c r="D6" s="7">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="19"/>
-      <c r="B7" s="26" t="s">
+      <c r="A7" s="21"/>
+      <c r="B7" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="23"/>
+      <c r="C7" s="25"/>
       <c r="D7" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="19"/>
-      <c r="B8" s="26" t="s">
+      <c r="A8" s="21"/>
+      <c r="B8" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="23"/>
+      <c r="C8" s="25"/>
       <c r="D8" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="19"/>
-      <c r="B9" s="36" t="s">
+      <c r="A9" s="21"/>
+      <c r="B9" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="37"/>
+      <c r="C9" s="46"/>
       <c r="D9" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="19"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="23"/>
+      <c r="A10" s="21"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="25"/>
       <c r="D10" s="8"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="19"/>
+      <c r="A11" s="21"/>
       <c r="B11" s="2" t="s">
         <v>6</v>
       </c>
@@ -1443,37 +1440,37 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="19"/>
-      <c r="B12" s="27" t="s">
+      <c r="A12" s="21"/>
+      <c r="B12" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="28"/>
-      <c r="D12" s="29"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="28"/>
     </row>
     <row r="13" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="18">
+      <c r="A13" s="20">
         <v>46154</v>
       </c>
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="21"/>
+      <c r="C13" s="23"/>
       <c r="D13" s="7">
         <v>0.5</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="19"/>
-      <c r="B14" s="26" t="s">
+      <c r="A14" s="21"/>
+      <c r="B14" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="23"/>
+      <c r="C14" s="25"/>
       <c r="D14" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="19"/>
+      <c r="A15" s="21"/>
       <c r="B15" s="13" t="s">
         <v>18</v>
       </c>
@@ -1482,23 +1479,23 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="19"/>
-      <c r="B16" s="26" t="s">
+      <c r="A16" s="21"/>
+      <c r="B16" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="23"/>
+      <c r="C16" s="25"/>
       <c r="D16" s="8">
         <v>1.5</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="19"/>
-      <c r="B17" s="26"/>
-      <c r="C17" s="23"/>
+      <c r="A17" s="21"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="25"/>
       <c r="D17" s="8"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="19"/>
+      <c r="A18" s="21"/>
       <c r="B18" s="2" t="s">
         <v>6</v>
       </c>
@@ -1511,75 +1508,75 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="19"/>
-      <c r="B19" s="27" t="s">
+      <c r="A19" s="21"/>
+      <c r="B19" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="28"/>
-      <c r="D19" s="29"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="28"/>
     </row>
     <row r="20" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="18">
+      <c r="A20" s="20">
         <v>46157</v>
       </c>
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="21"/>
+      <c r="C20" s="23"/>
       <c r="D20" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="19"/>
-      <c r="B21" s="22" t="s">
+      <c r="A21" s="21"/>
+      <c r="B21" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="23"/>
+      <c r="C21" s="25"/>
       <c r="D21" s="8">
         <v>2.5</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="19"/>
-      <c r="B22" s="24" t="s">
+      <c r="A22" s="21"/>
+      <c r="B22" s="48" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="25"/>
+      <c r="C22" s="49"/>
       <c r="D22" s="8"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="19"/>
-      <c r="B23" s="30" t="s">
+      <c r="A23" s="21"/>
+      <c r="B23" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="31"/>
+      <c r="C23" s="51"/>
       <c r="D23" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="19"/>
-      <c r="B24" s="26" t="s">
+      <c r="A24" s="21"/>
+      <c r="B24" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="23"/>
+      <c r="C24" s="25"/>
       <c r="D24" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="19"/>
-      <c r="B25" s="26" t="s">
+      <c r="A25" s="21"/>
+      <c r="B25" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="C25" s="23"/>
+      <c r="C25" s="25"/>
       <c r="D25" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="19"/>
+      <c r="A26" s="21"/>
       <c r="B26" s="2" t="s">
         <v>6</v>
       </c>
@@ -1592,57 +1589,57 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="19"/>
-      <c r="B27" s="27" t="s">
+      <c r="A27" s="21"/>
+      <c r="B27" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="28"/>
-      <c r="D27" s="29"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="28"/>
     </row>
     <row r="28" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="18">
+      <c r="A28" s="20">
         <v>46160</v>
       </c>
-      <c r="B28" s="20" t="s">
+      <c r="B28" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="21"/>
+      <c r="C28" s="23"/>
       <c r="D28" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="19"/>
-      <c r="B29" s="26" t="s">
+      <c r="A29" s="21"/>
+      <c r="B29" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="23"/>
+      <c r="C29" s="25"/>
       <c r="D29" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="19"/>
-      <c r="B30" s="26" t="s">
+      <c r="A30" s="21"/>
+      <c r="B30" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="23"/>
+      <c r="C30" s="25"/>
       <c r="D30" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="19"/>
-      <c r="B31" s="26" t="s">
+      <c r="A31" s="21"/>
+      <c r="B31" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="23"/>
+      <c r="C31" s="25"/>
       <c r="D31" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="19"/>
+      <c r="A32" s="21"/>
       <c r="B32" s="14" t="s">
         <v>31</v>
       </c>
@@ -1652,7 +1649,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="19"/>
+      <c r="A33" s="21"/>
       <c r="B33" s="14" t="s">
         <v>32</v>
       </c>
@@ -1662,17 +1659,17 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="19"/>
-      <c r="B34" s="26" t="s">
+      <c r="A34" s="21"/>
+      <c r="B34" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="23"/>
+      <c r="C34" s="25"/>
       <c r="D34" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="19"/>
+      <c r="A35" s="21"/>
       <c r="B35" s="2" t="s">
         <v>6</v>
       </c>
@@ -1685,15 +1682,15 @@
       </c>
     </row>
     <row r="36" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="35"/>
-      <c r="B36" s="32" t="s">
+      <c r="A36" s="29"/>
+      <c r="B36" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="C36" s="33"/>
-      <c r="D36" s="34"/>
+      <c r="C36" s="31"/>
+      <c r="D36" s="32"/>
     </row>
     <row r="37" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="18">
+      <c r="A37" s="20">
         <v>46161</v>
       </c>
       <c r="B37" s="16" t="s">
@@ -1705,43 +1702,43 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="19"/>
-      <c r="B38" s="49" t="s">
+      <c r="A38" s="21"/>
+      <c r="B38" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="C38" s="50"/>
+      <c r="C38" s="34"/>
       <c r="D38" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="19"/>
-      <c r="B39" s="26" t="s">
+      <c r="A39" s="21"/>
+      <c r="B39" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="C39" s="23"/>
+      <c r="C39" s="25"/>
       <c r="D39" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="19"/>
-      <c r="B40" s="26" t="s">
+      <c r="A40" s="21"/>
+      <c r="B40" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="23"/>
+      <c r="C40" s="25"/>
       <c r="D40" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="19"/>
-      <c r="B41" s="26"/>
-      <c r="C41" s="23"/>
+      <c r="A41" s="21"/>
+      <c r="B41" s="24"/>
+      <c r="C41" s="25"/>
       <c r="D41" s="8"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="19"/>
+      <c r="A42" s="21"/>
       <c r="B42" s="2" t="s">
         <v>6</v>
       </c>
@@ -1754,55 +1751,55 @@
       </c>
     </row>
     <row r="43" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="35"/>
-      <c r="B43" s="32" t="s">
+      <c r="A43" s="29"/>
+      <c r="B43" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="C43" s="33"/>
-      <c r="D43" s="34"/>
+      <c r="C43" s="31"/>
+      <c r="D43" s="32"/>
     </row>
     <row r="44" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="18">
+      <c r="A44" s="20">
         <v>46163</v>
       </c>
-      <c r="B44" s="20" t="s">
+      <c r="B44" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="C44" s="21"/>
+      <c r="C44" s="23"/>
       <c r="D44" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="19"/>
-      <c r="B45" s="26" t="s">
+      <c r="A45" s="21"/>
+      <c r="B45" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="C45" s="23"/>
+      <c r="C45" s="25"/>
       <c r="D45" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="19"/>
-      <c r="B46" s="26"/>
-      <c r="C46" s="23"/>
+      <c r="A46" s="21"/>
+      <c r="B46" s="24"/>
+      <c r="C46" s="25"/>
       <c r="D46" s="8"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="19"/>
-      <c r="B47" s="26"/>
-      <c r="C47" s="23"/>
+      <c r="A47" s="21"/>
+      <c r="B47" s="24"/>
+      <c r="C47" s="25"/>
       <c r="D47" s="8"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="19"/>
-      <c r="B48" s="26"/>
-      <c r="C48" s="23"/>
+      <c r="A48" s="21"/>
+      <c r="B48" s="24"/>
+      <c r="C48" s="25"/>
       <c r="D48" s="8"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="19"/>
+      <c r="A49" s="21"/>
       <c r="B49" s="2" t="s">
         <v>6</v>
       </c>
@@ -1815,67 +1812,67 @@
       </c>
     </row>
     <row r="50" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="35"/>
-      <c r="B50" s="32" t="s">
+      <c r="A50" s="29"/>
+      <c r="B50" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="C50" s="33"/>
-      <c r="D50" s="34"/>
+      <c r="C50" s="31"/>
+      <c r="D50" s="32"/>
     </row>
     <row r="51" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="18">
+      <c r="A51" s="20">
         <v>46164</v>
       </c>
-      <c r="B51" s="20" t="s">
+      <c r="B51" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="C51" s="21"/>
+      <c r="C51" s="23"/>
       <c r="D51" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="19"/>
-      <c r="B52" s="26" t="s">
+      <c r="A52" s="21"/>
+      <c r="B52" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="C52" s="23"/>
+      <c r="C52" s="25"/>
       <c r="D52" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="19"/>
-      <c r="B53" s="26" t="s">
+      <c r="A53" s="21"/>
+      <c r="B53" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="C53" s="23"/>
+      <c r="C53" s="25"/>
       <c r="D53" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="19"/>
-      <c r="B54" s="26" t="s">
+      <c r="A54" s="21"/>
+      <c r="B54" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="C54" s="23"/>
+      <c r="C54" s="25"/>
       <c r="D54" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" s="19"/>
-      <c r="B55" s="26" t="s">
+      <c r="A55" s="21"/>
+      <c r="B55" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="C55" s="23"/>
+      <c r="C55" s="25"/>
       <c r="D55" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="19"/>
+      <c r="A56" s="21"/>
       <c r="B56" s="14" t="s">
         <v>38</v>
       </c>
@@ -1885,7 +1882,7 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" s="19"/>
+      <c r="A57" s="21"/>
       <c r="B57" s="14" t="s">
         <v>46</v>
       </c>
@@ -1895,7 +1892,7 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" s="19"/>
+      <c r="A58" s="21"/>
       <c r="B58" s="2" t="s">
         <v>6</v>
       </c>
@@ -1908,241 +1905,343 @@
       </c>
     </row>
     <row r="59" spans="1:4" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="35"/>
-      <c r="B59" s="32" t="s">
+      <c r="A59" s="29"/>
+      <c r="B59" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="C59" s="33"/>
-      <c r="D59" s="34"/>
+      <c r="C59" s="31"/>
+      <c r="D59" s="32"/>
     </row>
     <row r="60" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="18">
+      <c r="A60" s="20">
         <v>46171</v>
       </c>
-      <c r="B60" s="20" t="s">
+      <c r="B60" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="C60" s="21"/>
+      <c r="C60" s="23"/>
       <c r="D60" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" s="19"/>
-      <c r="B61" s="26" t="s">
+      <c r="A61" s="21"/>
+      <c r="B61" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="C61" s="23"/>
+      <c r="C61" s="25"/>
       <c r="D61" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="19"/>
-      <c r="B62" s="26"/>
-      <c r="C62" s="23"/>
-      <c r="D62" s="8"/>
+      <c r="A62" s="21"/>
+      <c r="B62" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C62" s="15"/>
+      <c r="D62" s="8">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="19"/>
-      <c r="B63" s="26"/>
-      <c r="C63" s="23"/>
-      <c r="D63" s="8"/>
+      <c r="A63" s="21"/>
+      <c r="B63" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="C63" s="25"/>
+      <c r="D63" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="19"/>
-      <c r="B64" s="26"/>
-      <c r="C64" s="23"/>
-      <c r="D64" s="8"/>
+      <c r="A64" s="21"/>
+      <c r="B64" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="C64" s="15"/>
+      <c r="D64" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" s="19"/>
-      <c r="B65" s="2" t="s">
+      <c r="A65" s="21"/>
+      <c r="B65" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="C65" s="25"/>
+      <c r="D65" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" s="21"/>
+      <c r="B66" s="45" t="s">
+        <v>53</v>
+      </c>
+      <c r="C66" s="46"/>
+      <c r="D66" s="8">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" s="21"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" s="21"/>
+      <c r="B68" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C65" s="3" t="s">
+      <c r="C68" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D65" s="9">
-        <f>SUM(D60:D64)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="35"/>
-      <c r="B66" s="32"/>
-      <c r="C66" s="33"/>
-      <c r="D66" s="34"/>
-    </row>
-    <row r="67" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="18"/>
-      <c r="B67" s="20"/>
-      <c r="C67" s="21"/>
-      <c r="D67" s="7"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="19"/>
-      <c r="B68" s="26"/>
-      <c r="C68" s="23"/>
-      <c r="D68" s="8"/>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="19"/>
-      <c r="B69" s="26"/>
-      <c r="C69" s="23"/>
-      <c r="D69" s="8"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="19"/>
-      <c r="B70" s="26"/>
+      <c r="D68" s="9">
+        <f>SUM(D60:D66)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="29"/>
+      <c r="B69" s="30" t="s">
+        <v>56</v>
+      </c>
+      <c r="C69" s="31"/>
+      <c r="D69" s="32"/>
+    </row>
+    <row r="70" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="20"/>
+      <c r="B70" s="22"/>
       <c r="C70" s="23"/>
-      <c r="D70" s="8"/>
+      <c r="D70" s="7"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" s="19"/>
-      <c r="B71" s="26"/>
-      <c r="C71" s="23"/>
+      <c r="A71" s="21"/>
+      <c r="B71" s="24"/>
+      <c r="C71" s="25"/>
       <c r="D71" s="8"/>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="19"/>
-      <c r="B72" s="2" t="s">
+      <c r="A72" s="21"/>
+      <c r="B72" s="24"/>
+      <c r="C72" s="25"/>
+      <c r="D72" s="8"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A73" s="21"/>
+      <c r="B73" s="24"/>
+      <c r="C73" s="25"/>
+      <c r="D73" s="8"/>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" s="21"/>
+      <c r="B74" s="24"/>
+      <c r="C74" s="25"/>
+      <c r="D74" s="8"/>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" s="21"/>
+      <c r="B75" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C72" s="3" t="s">
+      <c r="C75" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D72" s="9">
-        <f>SUM(D67:D71)</f>
+      <c r="D75" s="9">
+        <f>SUM(D70:D74)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="19"/>
-      <c r="B73" s="27"/>
-      <c r="C73" s="28"/>
-      <c r="D73" s="29"/>
-    </row>
-    <row r="74" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="18"/>
-      <c r="B74" s="20"/>
-      <c r="C74" s="21"/>
-      <c r="D74" s="7"/>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="19"/>
-      <c r="B75" s="26"/>
-      <c r="C75" s="23"/>
-      <c r="D75" s="8"/>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="19"/>
+    <row r="76" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A76" s="21"/>
       <c r="B76" s="26"/>
-      <c r="C76" s="23"/>
-      <c r="D76" s="8"/>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="19"/>
-      <c r="B77" s="26"/>
+      <c r="C76" s="27"/>
+      <c r="D76" s="28"/>
+    </row>
+    <row r="77" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A77" s="20"/>
+      <c r="B77" s="22"/>
       <c r="C77" s="23"/>
-      <c r="D77" s="8"/>
+      <c r="D77" s="7"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="19"/>
-      <c r="B78" s="26"/>
-      <c r="C78" s="23"/>
+      <c r="A78" s="21"/>
+      <c r="B78" s="24"/>
+      <c r="C78" s="25"/>
       <c r="D78" s="8"/>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="19"/>
-      <c r="B79" s="2" t="s">
+      <c r="A79" s="21"/>
+      <c r="B79" s="24"/>
+      <c r="C79" s="25"/>
+      <c r="D79" s="8"/>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" s="21"/>
+      <c r="B80" s="24"/>
+      <c r="C80" s="25"/>
+      <c r="D80" s="8"/>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A81" s="21"/>
+      <c r="B81" s="24"/>
+      <c r="C81" s="25"/>
+      <c r="D81" s="8"/>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" s="21"/>
+      <c r="B82" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C79" s="3" t="s">
+      <c r="C82" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D79" s="9">
-        <f>SUM(D74:D78)</f>
+      <c r="D82" s="9">
+        <f>SUM(D77:D81)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="35"/>
-      <c r="B80" s="32"/>
-      <c r="C80" s="33"/>
-      <c r="D80" s="34"/>
-    </row>
-    <row r="81" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="18"/>
-      <c r="B81" s="20"/>
-      <c r="C81" s="21"/>
-      <c r="D81" s="7"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" s="19"/>
-      <c r="B82" s="26"/>
-      <c r="C82" s="23"/>
-      <c r="D82" s="8"/>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" s="19"/>
-      <c r="B83" s="26"/>
-      <c r="C83" s="23"/>
-      <c r="D83" s="8"/>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="19"/>
-      <c r="B84" s="26"/>
+    <row r="83" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A83" s="29"/>
+      <c r="B83" s="30"/>
+      <c r="C83" s="31"/>
+      <c r="D83" s="32"/>
+    </row>
+    <row r="84" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A84" s="20"/>
+      <c r="B84" s="22"/>
       <c r="C84" s="23"/>
-      <c r="D84" s="8"/>
+      <c r="D84" s="7"/>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A85" s="19"/>
-      <c r="B85" s="26"/>
-      <c r="C85" s="23"/>
+      <c r="A85" s="21"/>
+      <c r="B85" s="24"/>
+      <c r="C85" s="25"/>
       <c r="D85" s="8"/>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A86" s="19"/>
-      <c r="B86" s="2" t="s">
+      <c r="A86" s="21"/>
+      <c r="B86" s="24"/>
+      <c r="C86" s="25"/>
+      <c r="D86" s="8"/>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A87" s="21"/>
+      <c r="B87" s="24"/>
+      <c r="C87" s="25"/>
+      <c r="D87" s="8"/>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A88" s="21"/>
+      <c r="B88" s="24"/>
+      <c r="C88" s="25"/>
+      <c r="D88" s="8"/>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A89" s="21"/>
+      <c r="B89" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C86" s="3" t="s">
+      <c r="C89" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D86" s="9">
-        <f>SUM(D81:D85)</f>
+      <c r="D89" s="9">
+        <f>SUM(D84:D88)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A87" s="35"/>
-      <c r="B87" s="32"/>
-      <c r="C87" s="33"/>
-      <c r="D87" s="34"/>
-    </row>
-    <row r="88" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A88" s="11"/>
-      <c r="B88" s="10"/>
-      <c r="C88" s="3" t="s">
+    <row r="90" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A90" s="29"/>
+      <c r="B90" s="30"/>
+      <c r="C90" s="31"/>
+      <c r="D90" s="32"/>
+    </row>
+    <row r="91" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A91" s="11"/>
+      <c r="B91" s="10"/>
+      <c r="C91" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D88" s="12">
-        <f>D11+D18+D26+D35+D42+D49+D58+D65+D72+D79+D86</f>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A89" s="48" t="s">
+      <c r="D91" s="12">
+        <f>D11+D18+D26+D35+D42+D49+D58+D68+D75+D82+D89</f>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A92" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B89" s="48"/>
-      <c r="C89" s="48"/>
-      <c r="D89" s="48"/>
+      <c r="B92" s="19"/>
+      <c r="C92" s="19"/>
+      <c r="D92" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="81">
-    <mergeCell ref="A89:D89"/>
+    <mergeCell ref="A20:A27"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B69:D69"/>
+    <mergeCell ref="A84:A90"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="B87:C87"/>
+    <mergeCell ref="B88:C88"/>
+    <mergeCell ref="B90:D90"/>
+    <mergeCell ref="A51:A59"/>
+    <mergeCell ref="A77:A83"/>
+    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="B78:C78"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B83:D83"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="A60:A69"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="A44:A50"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="A70:A76"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="B76:D76"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="A6:A12"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B4:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A92:D92"/>
     <mergeCell ref="A13:A19"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
@@ -2158,150 +2257,77 @@
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="A37:A43"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="A6:A12"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B4:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A67:A73"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="B68:C68"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B73:D73"/>
-    <mergeCell ref="A44:A50"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="A51:A59"/>
-    <mergeCell ref="A74:A80"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="B75:C75"/>
-    <mergeCell ref="B76:C76"/>
-    <mergeCell ref="B77:C77"/>
-    <mergeCell ref="B78:C78"/>
-    <mergeCell ref="B80:D80"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B59:D59"/>
-    <mergeCell ref="A60:A66"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="A81:A87"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="B87:D87"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="B66:D66"/>
-    <mergeCell ref="A20:A27"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B23:C23"/>
   </mergeCells>
-  <conditionalFormatting sqref="D6:D11 D13:D14 D16:D18 D20:D23 D25:D26">
-    <cfRule type="containsText" dxfId="19" priority="23" operator="containsText" text="Terminé">
+  <conditionalFormatting sqref="D6:D11 D13:D14 D16:D18 D20:D23 D25:D26 D60:D66 D68">
+    <cfRule type="containsText" dxfId="17" priority="23" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="24" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="16" priority="24" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D28:D35">
-    <cfRule type="containsText" dxfId="17" priority="19" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="15" priority="19" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D28)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="20" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="14" priority="20" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D28)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D37:D42">
-    <cfRule type="containsText" dxfId="15" priority="17" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="13" priority="17" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D37)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="18" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="12" priority="18" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D37)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D44:D49">
-    <cfRule type="containsText" dxfId="13" priority="9" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="11" priority="9" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D44)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="10" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="10" priority="10" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D44)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D51:D58">
-    <cfRule type="containsText" dxfId="11" priority="7" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="9" priority="7" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D51)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="8" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="8" priority="8" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D51)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D60:D65">
-    <cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D60)))</formula>
+  <conditionalFormatting sqref="D70:D75">
+    <cfRule type="containsText" dxfId="7" priority="15" operator="containsText" text="Terminé">
+      <formula>NOT(ISERROR(SEARCH("Terminé",D70)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="6" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D60)))</formula>
+    <cfRule type="containsText" dxfId="6" priority="16" operator="containsText" text="En cours">
+      <formula>NOT(ISERROR(SEARCH("En cours",D70)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D67:D72">
-    <cfRule type="containsText" dxfId="7" priority="15" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D67)))</formula>
+  <conditionalFormatting sqref="D77:D82">
+    <cfRule type="containsText" dxfId="5" priority="13" operator="containsText" text="Terminé">
+      <formula>NOT(ISERROR(SEARCH("Terminé",D77)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="16" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D67)))</formula>
+    <cfRule type="containsText" dxfId="4" priority="14" operator="containsText" text="En cours">
+      <formula>NOT(ISERROR(SEARCH("En cours",D77)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D74:D79">
-    <cfRule type="containsText" dxfId="5" priority="13" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D74)))</formula>
+  <conditionalFormatting sqref="D84:D89">
+    <cfRule type="containsText" dxfId="3" priority="11" operator="containsText" text="Terminé">
+      <formula>NOT(ISERROR(SEARCH("Terminé",D84)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="14" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D74)))</formula>
+    <cfRule type="containsText" dxfId="2" priority="12" operator="containsText" text="En cours">
+      <formula>NOT(ISERROR(SEARCH("En cours",D84)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D81:D86">
-    <cfRule type="containsText" dxfId="3" priority="11" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D81)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="12" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D81)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D88">
+  <conditionalFormatting sqref="D91">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D88)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D91)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D88)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D91)))</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
@@ -2314,7 +2340,7 @@
   </headerFooter>
   <rowBreaks count="2" manualBreakCount="2">
     <brk id="50" max="16383" man="1"/>
-    <brk id="88" max="3" man="1"/>
+    <brk id="91" max="3" man="1"/>
   </rowBreaks>
   <legacyDrawingHF r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: moteur d'analyse IA opérationnel et frontend Vue 3 complet
- server : orchestration de l'analyse (exécution, parallélisation des
  fichiers), intégration OpenRouter, chiffrement AES du token GitHub
- client : application Vue 3 (router, store Pinia, service API), pages
  connexion/projets/détail, polling de progression, rendu Mermaid
  (zoom/pan), filtre des erreurs par sévérité
- docs : planning et journal mis à jour
</commit_message>
<xml_diff>
--- a/doc/GAMEZ_Journal.xlsx
+++ b/doc/GAMEZ_Journal.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr checkCompatibility="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/thibaudfrederic_gamez_studentfr_ch/Documents/TPI/tpi2026-codementor/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="176" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6544A02D-3E1F-4D6C-AFFA-6E8542C90FAB}"/>
+  <xr:revisionPtr revIDLastSave="230" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B021B99C-051A-41C2-8A72-0C4F5D28EE49}"/>
   <bookViews>
-    <workbookView xWindow="1470" yWindow="1470" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2985" yWindow="2985" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="8" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Journal!$A$5:$HI$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$D$96</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Journal!$B:$D,Journal!$1:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$D$91</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="68">
   <si>
     <t>Insérer les lignes au-dessus de celle-ci !</t>
   </si>
@@ -244,6 +244,39 @@
   </si>
   <si>
     <t>La journée s'est bien passé, les différents endpoints fonctionnes et je suis confiant pour la suite</t>
+  </si>
+  <si>
+    <t>Mise en place du projet Vue.js + structure de base</t>
+  </si>
+  <si>
+    <t>Configuration du routing</t>
+  </si>
+  <si>
+    <t>Service API + interception du token</t>
+  </si>
+  <si>
+    <t>Page de connexion</t>
+  </si>
+  <si>
+    <t>Page de liste et création des projets</t>
+  </si>
+  <si>
+    <t>Page de détail projet (Detected Errors, Suggested Fixes)</t>
+  </si>
+  <si>
+    <t>Intégration du polling de la progression</t>
+  </si>
+  <si>
+    <t>Traitement des analyses super lent</t>
+  </si>
+  <si>
+    <t>Traitement par lots parallèles avec "Promise.all"</t>
+  </si>
+  <si>
+    <t>La journée a bien avancé, le frontend est fonctionnel de bout en bout et communique correctement avec le backend. Il me reste surtout à peaufiner le design et surtout documenté le tout. Je ne pensais pas que les requêtes LLM seraient si lentes, j'ai du ajouter un traitemnet parallèles pour analysé plusieurs fichiers en même temps</t>
+  </si>
+  <si>
+    <t>Amélioration backend</t>
   </si>
 </sst>
 </file>
@@ -563,7 +596,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -630,135 +663,143 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -766,29 +807,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="16">
     <dxf>
       <font>
         <strike val="0"/>
@@ -1330,8 +1349,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D92"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D97"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5703125" style="1"/>
     <col min="2" max="3" width="31.7109375" style="1" customWidth="1"/>
@@ -1341,93 +1360,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
     </row>
     <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="49" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="44"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="50"/>
       <c r="D2" s="4">
         <v>151446</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="37" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="37" t="s">
+      <c r="A4" s="43" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="38"/>
+      <c r="C4" s="44"/>
       <c r="D4" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="39"/>
-      <c r="B5" s="39"/>
-      <c r="C5" s="40"/>
+      <c r="A5" s="45"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="46"/>
       <c r="D5" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="35">
+      <c r="A6" s="41">
         <v>46153</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="42"/>
+      <c r="C6" s="48"/>
       <c r="D6" s="7">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="21"/>
-      <c r="B7" s="24" t="s">
+      <c r="A7" s="22"/>
+      <c r="B7" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="25"/>
+      <c r="C7" s="26"/>
       <c r="D7" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="21"/>
-      <c r="B8" s="24" t="s">
+      <c r="A8" s="22"/>
+      <c r="B8" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="25"/>
+      <c r="C8" s="26"/>
       <c r="D8" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="21"/>
-      <c r="B9" s="45" t="s">
+      <c r="A9" s="22"/>
+      <c r="B9" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="46"/>
+      <c r="C9" s="36"/>
       <c r="D9" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="21"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="25"/>
+      <c r="A10" s="22"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="26"/>
       <c r="D10" s="8"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="21"/>
+      <c r="A11" s="22"/>
       <c r="B11" s="2" t="s">
         <v>6</v>
       </c>
@@ -1440,37 +1459,37 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="21"/>
-      <c r="B12" s="26" t="s">
+      <c r="A12" s="22"/>
+      <c r="B12" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="27"/>
-      <c r="D12" s="28"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="32"/>
     </row>
     <row r="13" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="20">
+      <c r="A13" s="21">
         <v>46154</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="23"/>
+      <c r="C13" s="24"/>
       <c r="D13" s="7">
         <v>0.5</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="21"/>
-      <c r="B14" s="24" t="s">
+      <c r="A14" s="22"/>
+      <c r="B14" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="25"/>
+      <c r="C14" s="26"/>
       <c r="D14" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="21"/>
+      <c r="A15" s="22"/>
       <c r="B15" s="13" t="s">
         <v>18</v>
       </c>
@@ -1479,23 +1498,23 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="21"/>
-      <c r="B16" s="24" t="s">
+      <c r="A16" s="22"/>
+      <c r="B16" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="25"/>
+      <c r="C16" s="26"/>
       <c r="D16" s="8">
         <v>1.5</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="21"/>
-      <c r="B17" s="24"/>
-      <c r="C17" s="25"/>
+      <c r="A17" s="22"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="26"/>
       <c r="D17" s="8"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="21"/>
+      <c r="A18" s="22"/>
       <c r="B18" s="2" t="s">
         <v>6</v>
       </c>
@@ -1508,75 +1527,75 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="21"/>
-      <c r="B19" s="26" t="s">
+      <c r="A19" s="22"/>
+      <c r="B19" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="27"/>
-      <c r="D19" s="28"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="32"/>
     </row>
     <row r="20" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="20">
+      <c r="A20" s="21">
         <v>46157</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="23"/>
+      <c r="C20" s="24"/>
       <c r="D20" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="21"/>
-      <c r="B21" s="47" t="s">
+      <c r="A21" s="22"/>
+      <c r="B21" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="25"/>
+      <c r="C21" s="26"/>
       <c r="D21" s="8">
         <v>2.5</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="21"/>
-      <c r="B22" s="48" t="s">
+      <c r="A22" s="22"/>
+      <c r="B22" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="49"/>
+      <c r="C22" s="28"/>
       <c r="D22" s="8"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="21"/>
-      <c r="B23" s="50" t="s">
+      <c r="A23" s="22"/>
+      <c r="B23" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="51"/>
+      <c r="C23" s="34"/>
       <c r="D23" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="21"/>
-      <c r="B24" s="24" t="s">
+      <c r="A24" s="22"/>
+      <c r="B24" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="25"/>
+      <c r="C24" s="26"/>
       <c r="D24" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="21"/>
-      <c r="B25" s="24" t="s">
+      <c r="A25" s="22"/>
+      <c r="B25" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="C25" s="25"/>
+      <c r="C25" s="26"/>
       <c r="D25" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="21"/>
+      <c r="A26" s="22"/>
       <c r="B26" s="2" t="s">
         <v>6</v>
       </c>
@@ -1589,57 +1608,57 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="26" t="s">
+      <c r="A27" s="22"/>
+      <c r="B27" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="27"/>
-      <c r="D27" s="28"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="32"/>
     </row>
     <row r="28" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="20">
+      <c r="A28" s="21">
         <v>46160</v>
       </c>
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="23"/>
+      <c r="C28" s="24"/>
       <c r="D28" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="21"/>
-      <c r="B29" s="24" t="s">
+      <c r="A29" s="22"/>
+      <c r="B29" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="25"/>
+      <c r="C29" s="26"/>
       <c r="D29" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="21"/>
-      <c r="B30" s="24" t="s">
+      <c r="A30" s="22"/>
+      <c r="B30" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="25"/>
+      <c r="C30" s="26"/>
       <c r="D30" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="21"/>
-      <c r="B31" s="24" t="s">
+      <c r="A31" s="22"/>
+      <c r="B31" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="25"/>
+      <c r="C31" s="26"/>
       <c r="D31" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="21"/>
+      <c r="A32" s="22"/>
       <c r="B32" s="14" t="s">
         <v>31</v>
       </c>
@@ -1649,7 +1668,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="21"/>
+      <c r="A33" s="22"/>
       <c r="B33" s="14" t="s">
         <v>32</v>
       </c>
@@ -1659,17 +1678,17 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="21"/>
-      <c r="B34" s="24" t="s">
+      <c r="A34" s="22"/>
+      <c r="B34" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="25"/>
+      <c r="C34" s="26"/>
       <c r="D34" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="21"/>
+      <c r="A35" s="22"/>
       <c r="B35" s="2" t="s">
         <v>6</v>
       </c>
@@ -1682,15 +1701,15 @@
       </c>
     </row>
     <row r="36" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="29"/>
-      <c r="B36" s="30" t="s">
+      <c r="A36" s="40"/>
+      <c r="B36" s="37" t="s">
         <v>34</v>
       </c>
-      <c r="C36" s="31"/>
-      <c r="D36" s="32"/>
+      <c r="C36" s="38"/>
+      <c r="D36" s="39"/>
     </row>
     <row r="37" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="20">
+      <c r="A37" s="21">
         <v>46161</v>
       </c>
       <c r="B37" s="16" t="s">
@@ -1702,43 +1721,43 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="21"/>
-      <c r="B38" s="33" t="s">
+      <c r="A38" s="22"/>
+      <c r="B38" s="52" t="s">
         <v>36</v>
       </c>
-      <c r="C38" s="34"/>
+      <c r="C38" s="53"/>
       <c r="D38" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="21"/>
-      <c r="B39" s="24" t="s">
+      <c r="A39" s="22"/>
+      <c r="B39" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="C39" s="25"/>
+      <c r="C39" s="26"/>
       <c r="D39" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="21"/>
-      <c r="B40" s="24" t="s">
+      <c r="A40" s="22"/>
+      <c r="B40" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="25"/>
+      <c r="C40" s="26"/>
       <c r="D40" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="21"/>
-      <c r="B41" s="24"/>
-      <c r="C41" s="25"/>
+      <c r="A41" s="22"/>
+      <c r="B41" s="29"/>
+      <c r="C41" s="26"/>
       <c r="D41" s="8"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="21"/>
+      <c r="A42" s="22"/>
       <c r="B42" s="2" t="s">
         <v>6</v>
       </c>
@@ -1751,55 +1770,55 @@
       </c>
     </row>
     <row r="43" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="29"/>
-      <c r="B43" s="30" t="s">
+      <c r="A43" s="40"/>
+      <c r="B43" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="C43" s="31"/>
-      <c r="D43" s="32"/>
+      <c r="C43" s="38"/>
+      <c r="D43" s="39"/>
     </row>
     <row r="44" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="20">
+      <c r="A44" s="21">
         <v>46163</v>
       </c>
-      <c r="B44" s="22" t="s">
+      <c r="B44" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="C44" s="23"/>
+      <c r="C44" s="24"/>
       <c r="D44" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="21"/>
-      <c r="B45" s="24" t="s">
+      <c r="A45" s="22"/>
+      <c r="B45" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="C45" s="25"/>
+      <c r="C45" s="26"/>
       <c r="D45" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="21"/>
-      <c r="B46" s="24"/>
-      <c r="C46" s="25"/>
+      <c r="A46" s="22"/>
+      <c r="B46" s="29"/>
+      <c r="C46" s="26"/>
       <c r="D46" s="8"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="21"/>
-      <c r="B47" s="24"/>
-      <c r="C47" s="25"/>
+      <c r="A47" s="22"/>
+      <c r="B47" s="29"/>
+      <c r="C47" s="26"/>
       <c r="D47" s="8"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="21"/>
-      <c r="B48" s="24"/>
-      <c r="C48" s="25"/>
+      <c r="A48" s="22"/>
+      <c r="B48" s="29"/>
+      <c r="C48" s="26"/>
       <c r="D48" s="8"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="21"/>
+      <c r="A49" s="22"/>
       <c r="B49" s="2" t="s">
         <v>6</v>
       </c>
@@ -1812,67 +1831,67 @@
       </c>
     </row>
     <row r="50" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="29"/>
-      <c r="B50" s="30" t="s">
+      <c r="A50" s="40"/>
+      <c r="B50" s="37" t="s">
         <v>42</v>
       </c>
-      <c r="C50" s="31"/>
-      <c r="D50" s="32"/>
+      <c r="C50" s="38"/>
+      <c r="D50" s="39"/>
     </row>
     <row r="51" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="20">
+      <c r="A51" s="21">
         <v>46164</v>
       </c>
-      <c r="B51" s="22" t="s">
+      <c r="B51" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="C51" s="23"/>
+      <c r="C51" s="24"/>
       <c r="D51" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="21"/>
-      <c r="B52" s="24" t="s">
+      <c r="A52" s="22"/>
+      <c r="B52" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="C52" s="25"/>
+      <c r="C52" s="26"/>
       <c r="D52" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="21"/>
-      <c r="B53" s="24" t="s">
+      <c r="A53" s="22"/>
+      <c r="B53" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="C53" s="25"/>
+      <c r="C53" s="26"/>
       <c r="D53" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="21"/>
-      <c r="B54" s="24" t="s">
+      <c r="A54" s="22"/>
+      <c r="B54" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="C54" s="25"/>
+      <c r="C54" s="26"/>
       <c r="D54" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" s="21"/>
-      <c r="B55" s="24" t="s">
+      <c r="A55" s="22"/>
+      <c r="B55" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="C55" s="25"/>
+      <c r="C55" s="26"/>
       <c r="D55" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="21"/>
+      <c r="A56" s="22"/>
       <c r="B56" s="14" t="s">
         <v>38</v>
       </c>
@@ -1882,7 +1901,7 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" s="21"/>
+      <c r="A57" s="22"/>
       <c r="B57" s="14" t="s">
         <v>46</v>
       </c>
@@ -1892,7 +1911,7 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" s="21"/>
+      <c r="A58" s="22"/>
       <c r="B58" s="2" t="s">
         <v>6</v>
       </c>
@@ -1905,37 +1924,37 @@
       </c>
     </row>
     <row r="59" spans="1:4" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="29"/>
-      <c r="B59" s="30" t="s">
+      <c r="A59" s="40"/>
+      <c r="B59" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="C59" s="31"/>
-      <c r="D59" s="32"/>
+      <c r="C59" s="38"/>
+      <c r="D59" s="39"/>
     </row>
     <row r="60" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="20">
+      <c r="A60" s="21">
         <v>46171</v>
       </c>
-      <c r="B60" s="22" t="s">
+      <c r="B60" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="C60" s="23"/>
+      <c r="C60" s="24"/>
       <c r="D60" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" s="21"/>
-      <c r="B61" s="24" t="s">
+      <c r="A61" s="22"/>
+      <c r="B61" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="C61" s="25"/>
+      <c r="C61" s="26"/>
       <c r="D61" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="21"/>
+      <c r="A62" s="22"/>
       <c r="B62" s="14" t="s">
         <v>55</v>
       </c>
@@ -1945,17 +1964,17 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="21"/>
-      <c r="B63" s="24" t="s">
+      <c r="A63" s="22"/>
+      <c r="B63" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="C63" s="25"/>
+      <c r="C63" s="26"/>
       <c r="D63" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="21"/>
+      <c r="A64" s="22"/>
       <c r="B64" s="18" t="s">
         <v>54</v>
       </c>
@@ -1965,30 +1984,30 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" s="21"/>
-      <c r="B65" s="24" t="s">
+      <c r="A65" s="22"/>
+      <c r="B65" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="C65" s="25"/>
+      <c r="C65" s="26"/>
       <c r="D65" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" s="21"/>
-      <c r="B66" s="45" t="s">
+      <c r="A66" s="22"/>
+      <c r="B66" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="C66" s="46"/>
+      <c r="C66" s="36"/>
       <c r="D66" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="21"/>
+      <c r="A67" s="22"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="21"/>
+      <c r="A68" s="22"/>
       <c r="B68" s="2" t="s">
         <v>6</v>
       </c>
@@ -2001,247 +2020,253 @@
       </c>
     </row>
     <row r="69" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="29"/>
-      <c r="B69" s="30" t="s">
+      <c r="A69" s="40"/>
+      <c r="B69" s="37" t="s">
         <v>56</v>
       </c>
-      <c r="C69" s="31"/>
-      <c r="D69" s="32"/>
+      <c r="C69" s="38"/>
+      <c r="D69" s="39"/>
     </row>
     <row r="70" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="20"/>
-      <c r="B70" s="22"/>
-      <c r="C70" s="23"/>
-      <c r="D70" s="7"/>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" s="21"/>
-      <c r="B71" s="24"/>
-      <c r="C71" s="25"/>
-      <c r="D71" s="8"/>
+      <c r="A70" s="21">
+        <v>46174</v>
+      </c>
+      <c r="B70" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="C70" s="24"/>
+      <c r="D70" s="7">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="22"/>
+      <c r="B71" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="C71" s="15"/>
+      <c r="D71" s="7">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="21"/>
-      <c r="B72" s="24"/>
-      <c r="C72" s="25"/>
-      <c r="D72" s="8"/>
+      <c r="A72" s="22"/>
+      <c r="B72" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="C72" s="26"/>
+      <c r="D72" s="7">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" s="21"/>
-      <c r="B73" s="24"/>
-      <c r="C73" s="25"/>
-      <c r="D73" s="8"/>
+      <c r="A73" s="22"/>
+      <c r="B73" s="29" t="s">
+        <v>59</v>
+      </c>
+      <c r="C73" s="26"/>
+      <c r="D73" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="21"/>
-      <c r="B74" s="24"/>
-      <c r="C74" s="25"/>
-      <c r="D74" s="8"/>
+      <c r="A74" s="22"/>
+      <c r="B74" s="29" t="s">
+        <v>60</v>
+      </c>
+      <c r="C74" s="26"/>
+      <c r="D74" s="8">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="21"/>
-      <c r="B75" s="2" t="s">
+      <c r="A75" s="22"/>
+      <c r="B75" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C75" s="15"/>
+      <c r="D75" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" s="22"/>
+      <c r="B76" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C76" s="15"/>
+      <c r="D76" s="8">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" s="22"/>
+      <c r="B77" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="C77" s="15"/>
+      <c r="D77" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" s="22"/>
+      <c r="B78" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="C78" s="20"/>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" s="22"/>
+      <c r="B79" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C79" s="34"/>
+      <c r="D79" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" s="22"/>
+      <c r="B80" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C75" s="3" t="s">
+      <c r="C80" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D75" s="9">
-        <f>SUM(D70:D74)</f>
+      <c r="D80" s="9">
+        <f>SUM(D70:D79)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A81" s="22"/>
+      <c r="B81" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="C81" s="31"/>
+      <c r="D81" s="32"/>
+    </row>
+    <row r="82" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="21"/>
+      <c r="B82" s="23"/>
+      <c r="C82" s="24"/>
+      <c r="D82" s="7"/>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" s="22"/>
+      <c r="B83" s="29"/>
+      <c r="C83" s="26"/>
+      <c r="D83" s="8"/>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A84" s="22"/>
+      <c r="B84" s="29"/>
+      <c r="C84" s="26"/>
+      <c r="D84" s="8"/>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A85" s="22"/>
+      <c r="B85" s="29"/>
+      <c r="C85" s="26"/>
+      <c r="D85" s="8"/>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A86" s="22"/>
+      <c r="B86" s="29"/>
+      <c r="C86" s="26"/>
+      <c r="D86" s="8"/>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A87" s="22"/>
+      <c r="B87" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D87" s="9">
+        <f>SUM(D82:D86)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="21"/>
-      <c r="B76" s="26"/>
-      <c r="C76" s="27"/>
-      <c r="D76" s="28"/>
-    </row>
-    <row r="77" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="20"/>
-      <c r="B77" s="22"/>
-      <c r="C77" s="23"/>
-      <c r="D77" s="7"/>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="21"/>
-      <c r="B78" s="24"/>
-      <c r="C78" s="25"/>
-      <c r="D78" s="8"/>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="21"/>
-      <c r="B79" s="24"/>
-      <c r="C79" s="25"/>
-      <c r="D79" s="8"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" s="21"/>
-      <c r="B80" s="24"/>
-      <c r="C80" s="25"/>
-      <c r="D80" s="8"/>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A81" s="21"/>
-      <c r="B81" s="24"/>
-      <c r="C81" s="25"/>
-      <c r="D81" s="8"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" s="21"/>
-      <c r="B82" s="2" t="s">
+    <row r="88" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A88" s="40"/>
+      <c r="B88" s="37"/>
+      <c r="C88" s="38"/>
+      <c r="D88" s="39"/>
+    </row>
+    <row r="89" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A89" s="21"/>
+      <c r="B89" s="23"/>
+      <c r="C89" s="24"/>
+      <c r="D89" s="7"/>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A90" s="22"/>
+      <c r="B90" s="29"/>
+      <c r="C90" s="26"/>
+      <c r="D90" s="8"/>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A91" s="22"/>
+      <c r="B91" s="29"/>
+      <c r="C91" s="26"/>
+      <c r="D91" s="8"/>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A92" s="22"/>
+      <c r="B92" s="29"/>
+      <c r="C92" s="26"/>
+      <c r="D92" s="8"/>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A93" s="22"/>
+      <c r="B93" s="29"/>
+      <c r="C93" s="26"/>
+      <c r="D93" s="8"/>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A94" s="22"/>
+      <c r="B94" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C82" s="3" t="s">
+      <c r="C94" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D82" s="9">
-        <f>SUM(D77:D81)</f>
+      <c r="D94" s="9">
+        <f>SUM(D89:D93)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="29"/>
-      <c r="B83" s="30"/>
-      <c r="C83" s="31"/>
-      <c r="D83" s="32"/>
-    </row>
-    <row r="84" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="20"/>
-      <c r="B84" s="22"/>
-      <c r="C84" s="23"/>
-      <c r="D84" s="7"/>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A85" s="21"/>
-      <c r="B85" s="24"/>
-      <c r="C85" s="25"/>
-      <c r="D85" s="8"/>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A86" s="21"/>
-      <c r="B86" s="24"/>
-      <c r="C86" s="25"/>
-      <c r="D86" s="8"/>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A87" s="21"/>
-      <c r="B87" s="24"/>
-      <c r="C87" s="25"/>
-      <c r="D87" s="8"/>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A88" s="21"/>
-      <c r="B88" s="24"/>
-      <c r="C88" s="25"/>
-      <c r="D88" s="8"/>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A89" s="21"/>
-      <c r="B89" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C89" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D89" s="9">
-        <f>SUM(D84:D88)</f>
+    <row r="95" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A95" s="40"/>
+      <c r="B95" s="37"/>
+      <c r="C95" s="38"/>
+      <c r="D95" s="39"/>
+    </row>
+    <row r="96" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A96" s="11"/>
+      <c r="B96" s="10"/>
+      <c r="C96" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D96" s="12">
+        <f>D11+D18+D26+D35+D42+D49+D58+D68+D80+D87+D94</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A97" s="51" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="29"/>
-      <c r="B90" s="30"/>
-      <c r="C90" s="31"/>
-      <c r="D90" s="32"/>
-    </row>
-    <row r="91" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A91" s="11"/>
-      <c r="B91" s="10"/>
-      <c r="C91" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D91" s="12">
-        <f>D11+D18+D26+D35+D42+D49+D58+D68+D75+D82+D89</f>
-        <v>52</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A92" s="19" t="s">
-        <v>0</v>
-      </c>
-      <c r="B92" s="19"/>
-      <c r="C92" s="19"/>
-      <c r="D92" s="19"/>
+      <c r="B97" s="51"/>
+      <c r="C97" s="51"/>
+      <c r="D97" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="81">
-    <mergeCell ref="A20:A27"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B69:D69"/>
-    <mergeCell ref="A84:A90"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="B86:C86"/>
-    <mergeCell ref="B87:C87"/>
-    <mergeCell ref="B88:C88"/>
-    <mergeCell ref="B90:D90"/>
-    <mergeCell ref="A51:A59"/>
-    <mergeCell ref="A77:A83"/>
-    <mergeCell ref="B77:C77"/>
-    <mergeCell ref="B78:C78"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="B80:C80"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B83:D83"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B59:D59"/>
-    <mergeCell ref="A60:A69"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="A44:A50"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="A70:A76"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="B76:D76"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A6:A12"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B4:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A92:D92"/>
+    <mergeCell ref="A97:D97"/>
     <mergeCell ref="A13:A19"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
@@ -2257,77 +2282,135 @@
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="A37:A43"/>
     <mergeCell ref="B38:C38"/>
+    <mergeCell ref="A6:A12"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B4:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="A70:A81"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="B81:D81"/>
+    <mergeCell ref="A44:A50"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="A51:A59"/>
+    <mergeCell ref="A82:A88"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="B88:D88"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="A60:A69"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="A89:A95"/>
+    <mergeCell ref="B89:C89"/>
+    <mergeCell ref="B90:C90"/>
+    <mergeCell ref="B91:C91"/>
+    <mergeCell ref="B92:C92"/>
+    <mergeCell ref="B93:C93"/>
+    <mergeCell ref="B95:D95"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B69:D69"/>
+    <mergeCell ref="A20:A27"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B23:C23"/>
   </mergeCells>
-  <conditionalFormatting sqref="D6:D11 D13:D14 D16:D18 D20:D23 D25:D26 D60:D66 D68">
-    <cfRule type="containsText" dxfId="17" priority="23" operator="containsText" text="Terminé">
+  <phoneticPr fontId="4" type="noConversion"/>
+  <conditionalFormatting sqref="D6:D11 D13:D14 D16:D18 D20:D23 D25:D26 D60:D66 D68 D70:D72 D74:D76 D79:D80">
+    <cfRule type="containsText" dxfId="15" priority="23" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="24" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="14" priority="24" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D28:D35">
-    <cfRule type="containsText" dxfId="15" priority="19" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="13" priority="19" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D28)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="20" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="12" priority="20" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D28)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D37:D42">
-    <cfRule type="containsText" dxfId="13" priority="17" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="11" priority="17" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D37)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="18" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="10" priority="18" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D37)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D44:D49">
-    <cfRule type="containsText" dxfId="11" priority="9" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="9" priority="9" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D44)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="10" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="8" priority="10" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D44)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D51:D58">
-    <cfRule type="containsText" dxfId="9" priority="7" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="7" priority="7" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D51)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="8" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="6" priority="8" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D51)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D70:D75">
-    <cfRule type="containsText" dxfId="7" priority="15" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D70)))</formula>
+  <conditionalFormatting sqref="D82:D87">
+    <cfRule type="containsText" dxfId="5" priority="13" operator="containsText" text="Terminé">
+      <formula>NOT(ISERROR(SEARCH("Terminé",D82)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="16" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D70)))</formula>
+    <cfRule type="containsText" dxfId="4" priority="14" operator="containsText" text="En cours">
+      <formula>NOT(ISERROR(SEARCH("En cours",D82)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D77:D82">
-    <cfRule type="containsText" dxfId="5" priority="13" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D77)))</formula>
+  <conditionalFormatting sqref="D89:D94">
+    <cfRule type="containsText" dxfId="3" priority="11" operator="containsText" text="Terminé">
+      <formula>NOT(ISERROR(SEARCH("Terminé",D89)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="14" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D77)))</formula>
+    <cfRule type="containsText" dxfId="2" priority="12" operator="containsText" text="En cours">
+      <formula>NOT(ISERROR(SEARCH("En cours",D89)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D84:D89">
-    <cfRule type="containsText" dxfId="3" priority="11" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D84)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="12" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D84)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D91">
+  <conditionalFormatting sqref="D96">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Terminé">
-      <formula>NOT(ISERROR(SEARCH("Terminé",D91)))</formula>
+      <formula>NOT(ISERROR(SEARCH("Terminé",D96)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="En cours">
-      <formula>NOT(ISERROR(SEARCH("En cours",D91)))</formula>
+      <formula>NOT(ISERROR(SEARCH("En cours",D96)))</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
@@ -2340,7 +2423,7 @@
   </headerFooter>
   <rowBreaks count="2" manualBreakCount="2">
     <brk id="50" max="16383" man="1"/>
-    <brk id="91" max="3" man="1"/>
+    <brk id="96" max="3" man="1"/>
   </rowBreaks>
   <legacyDrawingHF r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(server): fiabilise l'analyse IA
- Prompt anti-faux-positifs
- Réduction du coût des appels au modèle
- Diagramme Mermaid enrichi
- Mise à jour du rapport, du planning et du journal
</commit_message>
<xml_diff>
--- a/doc/GAMEZ_Journal.xlsx
+++ b/doc/GAMEZ_Journal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/thibaudfrederic_gamez_studentfr_ch/Documents/TPI/tpi2026-codementor/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="230" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B021B99C-051A-41C2-8A72-0C4F5D28EE49}"/>
+  <xr:revisionPtr revIDLastSave="240" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{615AB853-4C0E-43A9-B2D9-5F3B002F816D}"/>
   <bookViews>
-    <workbookView xWindow="2985" yWindow="2985" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="8" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Journal!$B:$D,Journal!$1:$5</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="72">
   <si>
     <t>Insérer les lignes au-dessus de celle-ci !</t>
   </si>
@@ -277,6 +278,18 @@
   </si>
   <si>
     <t>Amélioration backend</t>
+  </si>
+  <si>
+    <t>Responsive design et correction design</t>
+  </si>
+  <si>
+    <t>Tests de différents modèles et analyse de leurs retours</t>
+  </si>
+  <si>
+    <t>Correction erreurs dans schémas EA</t>
+  </si>
+  <si>
+    <t>J'ai terminé la partie frontend, j'ai aussi bien avancé la documentation et j'ai pu faire des tests sur différents LLM afin de constaté les différents et adapté le système prompt. Le retard est rattrapé, j'ai plus de doutes sur la faisabilité du projet.</t>
   </si>
 </sst>
 </file>
@@ -671,6 +684,10 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -688,118 +705,114 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1360,93 +1373,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
     </row>
     <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="50"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="46"/>
       <c r="D2" s="4">
         <v>151446</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="43" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="43" t="s">
+      <c r="A4" s="39" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="44"/>
+      <c r="C4" s="40"/>
       <c r="D4" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="45"/>
-      <c r="B5" s="45"/>
-      <c r="C5" s="46"/>
+      <c r="A5" s="41"/>
+      <c r="B5" s="41"/>
+      <c r="C5" s="42"/>
       <c r="D5" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="41">
+      <c r="A6" s="37">
         <v>46153</v>
       </c>
-      <c r="B6" s="47" t="s">
+      <c r="B6" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="48"/>
+      <c r="C6" s="44"/>
       <c r="D6" s="7">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="22"/>
-      <c r="B7" s="29" t="s">
+      <c r="A7" s="23"/>
+      <c r="B7" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="26"/>
+      <c r="C7" s="27"/>
       <c r="D7" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="22"/>
-      <c r="B8" s="29" t="s">
+      <c r="A8" s="23"/>
+      <c r="B8" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="26"/>
+      <c r="C8" s="27"/>
       <c r="D8" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="22"/>
-      <c r="B9" s="35" t="s">
+      <c r="A9" s="23"/>
+      <c r="B9" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="36"/>
+      <c r="C9" s="48"/>
       <c r="D9" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="22"/>
-      <c r="B10" s="29"/>
-      <c r="C10" s="26"/>
+      <c r="A10" s="23"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="27"/>
       <c r="D10" s="8"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="22"/>
+      <c r="A11" s="23"/>
       <c r="B11" s="2" t="s">
         <v>6</v>
       </c>
@@ -1459,37 +1472,37 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="22"/>
-      <c r="B12" s="30" t="s">
+      <c r="A12" s="23"/>
+      <c r="B12" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="31"/>
-      <c r="D12" s="32"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="30"/>
     </row>
     <row r="13" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="21">
+      <c r="A13" s="22">
         <v>46154</v>
       </c>
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="24"/>
+      <c r="C13" s="25"/>
       <c r="D13" s="7">
         <v>0.5</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="22"/>
-      <c r="B14" s="29" t="s">
+      <c r="A14" s="23"/>
+      <c r="B14" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="26"/>
+      <c r="C14" s="27"/>
       <c r="D14" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="22"/>
+      <c r="A15" s="23"/>
       <c r="B15" s="13" t="s">
         <v>18</v>
       </c>
@@ -1498,23 +1511,23 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="22"/>
-      <c r="B16" s="29" t="s">
+      <c r="A16" s="23"/>
+      <c r="B16" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="26"/>
+      <c r="C16" s="27"/>
       <c r="D16" s="8">
         <v>1.5</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="22"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="26"/>
+      <c r="A17" s="23"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="27"/>
       <c r="D17" s="8"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="22"/>
+      <c r="A18" s="23"/>
       <c r="B18" s="2" t="s">
         <v>6</v>
       </c>
@@ -1527,75 +1540,75 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="22"/>
-      <c r="B19" s="30" t="s">
+      <c r="A19" s="23"/>
+      <c r="B19" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="31"/>
-      <c r="D19" s="32"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="30"/>
     </row>
     <row r="20" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="21">
+      <c r="A20" s="22">
         <v>46157</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="24"/>
+      <c r="C20" s="25"/>
       <c r="D20" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="22"/>
-      <c r="B21" s="25" t="s">
+      <c r="A21" s="23"/>
+      <c r="B21" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="26"/>
+      <c r="C21" s="27"/>
       <c r="D21" s="8">
         <v>2.5</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="22"/>
-      <c r="B22" s="27" t="s">
+      <c r="A22" s="23"/>
+      <c r="B22" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="28"/>
+      <c r="C22" s="53"/>
       <c r="D22" s="8"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="22"/>
-      <c r="B23" s="33" t="s">
+      <c r="A23" s="23"/>
+      <c r="B23" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="34"/>
+      <c r="C23" s="50"/>
       <c r="D23" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="22"/>
-      <c r="B24" s="29" t="s">
+      <c r="A24" s="23"/>
+      <c r="B24" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="26"/>
+      <c r="C24" s="27"/>
       <c r="D24" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="22"/>
-      <c r="B25" s="29" t="s">
+      <c r="A25" s="23"/>
+      <c r="B25" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="C25" s="26"/>
+      <c r="C25" s="27"/>
       <c r="D25" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="22"/>
+      <c r="A26" s="23"/>
       <c r="B26" s="2" t="s">
         <v>6</v>
       </c>
@@ -1608,57 +1621,57 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="22"/>
-      <c r="B27" s="30" t="s">
+      <c r="A27" s="23"/>
+      <c r="B27" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="31"/>
-      <c r="D27" s="32"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="30"/>
     </row>
     <row r="28" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="21">
+      <c r="A28" s="22">
         <v>46160</v>
       </c>
-      <c r="B28" s="23" t="s">
+      <c r="B28" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="24"/>
+      <c r="C28" s="25"/>
       <c r="D28" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="22"/>
-      <c r="B29" s="29" t="s">
+      <c r="A29" s="23"/>
+      <c r="B29" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="26"/>
+      <c r="C29" s="27"/>
       <c r="D29" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="22"/>
-      <c r="B30" s="29" t="s">
+      <c r="A30" s="23"/>
+      <c r="B30" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="26"/>
+      <c r="C30" s="27"/>
       <c r="D30" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="22"/>
-      <c r="B31" s="29" t="s">
+      <c r="A31" s="23"/>
+      <c r="B31" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="26"/>
+      <c r="C31" s="27"/>
       <c r="D31" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="22"/>
+      <c r="A32" s="23"/>
       <c r="B32" s="14" t="s">
         <v>31</v>
       </c>
@@ -1668,7 +1681,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="22"/>
+      <c r="A33" s="23"/>
       <c r="B33" s="14" t="s">
         <v>32</v>
       </c>
@@ -1678,17 +1691,17 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="22"/>
-      <c r="B34" s="29" t="s">
+      <c r="A34" s="23"/>
+      <c r="B34" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="26"/>
+      <c r="C34" s="27"/>
       <c r="D34" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="22"/>
+      <c r="A35" s="23"/>
       <c r="B35" s="2" t="s">
         <v>6</v>
       </c>
@@ -1701,15 +1714,15 @@
       </c>
     </row>
     <row r="36" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="40"/>
-      <c r="B36" s="37" t="s">
+      <c r="A36" s="31"/>
+      <c r="B36" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="C36" s="38"/>
-      <c r="D36" s="39"/>
+      <c r="C36" s="33"/>
+      <c r="D36" s="34"/>
     </row>
     <row r="37" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="21">
+      <c r="A37" s="22">
         <v>46161</v>
       </c>
       <c r="B37" s="16" t="s">
@@ -1721,43 +1734,43 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="22"/>
-      <c r="B38" s="52" t="s">
+      <c r="A38" s="23"/>
+      <c r="B38" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="C38" s="53"/>
+      <c r="C38" s="36"/>
       <c r="D38" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="22"/>
-      <c r="B39" s="29" t="s">
+      <c r="A39" s="23"/>
+      <c r="B39" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="C39" s="26"/>
+      <c r="C39" s="27"/>
       <c r="D39" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="22"/>
-      <c r="B40" s="29" t="s">
+      <c r="A40" s="23"/>
+      <c r="B40" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="26"/>
+      <c r="C40" s="27"/>
       <c r="D40" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="22"/>
-      <c r="B41" s="29"/>
-      <c r="C41" s="26"/>
+      <c r="A41" s="23"/>
+      <c r="B41" s="26"/>
+      <c r="C41" s="27"/>
       <c r="D41" s="8"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="22"/>
+      <c r="A42" s="23"/>
       <c r="B42" s="2" t="s">
         <v>6</v>
       </c>
@@ -1770,55 +1783,55 @@
       </c>
     </row>
     <row r="43" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="40"/>
-      <c r="B43" s="37" t="s">
+      <c r="A43" s="31"/>
+      <c r="B43" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="C43" s="38"/>
-      <c r="D43" s="39"/>
+      <c r="C43" s="33"/>
+      <c r="D43" s="34"/>
     </row>
     <row r="44" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="21">
+      <c r="A44" s="22">
         <v>46163</v>
       </c>
-      <c r="B44" s="23" t="s">
+      <c r="B44" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="C44" s="24"/>
+      <c r="C44" s="25"/>
       <c r="D44" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="22"/>
-      <c r="B45" s="29" t="s">
+      <c r="A45" s="23"/>
+      <c r="B45" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="C45" s="26"/>
+      <c r="C45" s="27"/>
       <c r="D45" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="22"/>
-      <c r="B46" s="29"/>
-      <c r="C46" s="26"/>
+      <c r="A46" s="23"/>
+      <c r="B46" s="26"/>
+      <c r="C46" s="27"/>
       <c r="D46" s="8"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="22"/>
-      <c r="B47" s="29"/>
-      <c r="C47" s="26"/>
+      <c r="A47" s="23"/>
+      <c r="B47" s="26"/>
+      <c r="C47" s="27"/>
       <c r="D47" s="8"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="22"/>
-      <c r="B48" s="29"/>
-      <c r="C48" s="26"/>
+      <c r="A48" s="23"/>
+      <c r="B48" s="26"/>
+      <c r="C48" s="27"/>
       <c r="D48" s="8"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="22"/>
+      <c r="A49" s="23"/>
       <c r="B49" s="2" t="s">
         <v>6</v>
       </c>
@@ -1831,67 +1844,67 @@
       </c>
     </row>
     <row r="50" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="40"/>
-      <c r="B50" s="37" t="s">
+      <c r="A50" s="31"/>
+      <c r="B50" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="C50" s="38"/>
-      <c r="D50" s="39"/>
+      <c r="C50" s="33"/>
+      <c r="D50" s="34"/>
     </row>
     <row r="51" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="21">
+      <c r="A51" s="22">
         <v>46164</v>
       </c>
-      <c r="B51" s="23" t="s">
+      <c r="B51" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="C51" s="24"/>
+      <c r="C51" s="25"/>
       <c r="D51" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="22"/>
-      <c r="B52" s="29" t="s">
+      <c r="A52" s="23"/>
+      <c r="B52" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="C52" s="26"/>
+      <c r="C52" s="27"/>
       <c r="D52" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="22"/>
-      <c r="B53" s="29" t="s">
+      <c r="A53" s="23"/>
+      <c r="B53" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="C53" s="26"/>
+      <c r="C53" s="27"/>
       <c r="D53" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="22"/>
-      <c r="B54" s="29" t="s">
+      <c r="A54" s="23"/>
+      <c r="B54" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="C54" s="26"/>
+      <c r="C54" s="27"/>
       <c r="D54" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" s="22"/>
-      <c r="B55" s="29" t="s">
+      <c r="A55" s="23"/>
+      <c r="B55" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="C55" s="26"/>
+      <c r="C55" s="27"/>
       <c r="D55" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="22"/>
+      <c r="A56" s="23"/>
       <c r="B56" s="14" t="s">
         <v>38</v>
       </c>
@@ -1901,7 +1914,7 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" s="22"/>
+      <c r="A57" s="23"/>
       <c r="B57" s="14" t="s">
         <v>46</v>
       </c>
@@ -1911,7 +1924,7 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" s="22"/>
+      <c r="A58" s="23"/>
       <c r="B58" s="2" t="s">
         <v>6</v>
       </c>
@@ -1924,37 +1937,37 @@
       </c>
     </row>
     <row r="59" spans="1:4" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="40"/>
-      <c r="B59" s="37" t="s">
+      <c r="A59" s="31"/>
+      <c r="B59" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="C59" s="38"/>
-      <c r="D59" s="39"/>
+      <c r="C59" s="33"/>
+      <c r="D59" s="34"/>
     </row>
     <row r="60" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="21">
+      <c r="A60" s="22">
         <v>46171</v>
       </c>
-      <c r="B60" s="23" t="s">
+      <c r="B60" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="C60" s="24"/>
+      <c r="C60" s="25"/>
       <c r="D60" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" s="22"/>
-      <c r="B61" s="29" t="s">
+      <c r="A61" s="23"/>
+      <c r="B61" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="C61" s="26"/>
+      <c r="C61" s="27"/>
       <c r="D61" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="22"/>
+      <c r="A62" s="23"/>
       <c r="B62" s="14" t="s">
         <v>55</v>
       </c>
@@ -1964,17 +1977,17 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="22"/>
-      <c r="B63" s="29" t="s">
+      <c r="A63" s="23"/>
+      <c r="B63" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="C63" s="26"/>
+      <c r="C63" s="27"/>
       <c r="D63" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="22"/>
+      <c r="A64" s="23"/>
       <c r="B64" s="18" t="s">
         <v>54</v>
       </c>
@@ -1984,30 +1997,30 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" s="22"/>
-      <c r="B65" s="29" t="s">
+      <c r="A65" s="23"/>
+      <c r="B65" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="C65" s="26"/>
+      <c r="C65" s="27"/>
       <c r="D65" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" s="22"/>
-      <c r="B66" s="35" t="s">
+      <c r="A66" s="23"/>
+      <c r="B66" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="C66" s="36"/>
+      <c r="C66" s="48"/>
       <c r="D66" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="22"/>
+      <c r="A67" s="23"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="22"/>
+      <c r="A68" s="23"/>
       <c r="B68" s="2" t="s">
         <v>6</v>
       </c>
@@ -2020,27 +2033,27 @@
       </c>
     </row>
     <row r="69" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="40"/>
-      <c r="B69" s="37" t="s">
+      <c r="A69" s="31"/>
+      <c r="B69" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="C69" s="38"/>
-      <c r="D69" s="39"/>
+      <c r="C69" s="33"/>
+      <c r="D69" s="34"/>
     </row>
     <row r="70" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="21">
+      <c r="A70" s="22">
         <v>46174</v>
       </c>
-      <c r="B70" s="23" t="s">
+      <c r="B70" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="C70" s="24"/>
+      <c r="C70" s="25"/>
       <c r="D70" s="7">
         <v>0.5</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="22"/>
+      <c r="A71" s="23"/>
       <c r="B71" s="14" t="s">
         <v>57</v>
       </c>
@@ -2050,37 +2063,37 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="22"/>
-      <c r="B72" s="29" t="s">
+      <c r="A72" s="23"/>
+      <c r="B72" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="C72" s="26"/>
+      <c r="C72" s="27"/>
       <c r="D72" s="7">
         <v>0.75</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" s="22"/>
-      <c r="B73" s="29" t="s">
+      <c r="A73" s="23"/>
+      <c r="B73" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="C73" s="26"/>
+      <c r="C73" s="27"/>
       <c r="D73" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="22"/>
-      <c r="B74" s="29" t="s">
+      <c r="A74" s="23"/>
+      <c r="B74" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="C74" s="26"/>
+      <c r="C74" s="27"/>
       <c r="D74" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="22"/>
+      <c r="A75" s="23"/>
       <c r="B75" s="14" t="s">
         <v>61</v>
       </c>
@@ -2090,7 +2103,7 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="22"/>
+      <c r="A76" s="23"/>
       <c r="B76" s="14" t="s">
         <v>62</v>
       </c>
@@ -2100,7 +2113,7 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="22"/>
+      <c r="A77" s="23"/>
       <c r="B77" s="14" t="s">
         <v>63</v>
       </c>
@@ -2110,24 +2123,24 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="22"/>
+      <c r="A78" s="23"/>
       <c r="B78" s="19" t="s">
         <v>64</v>
       </c>
       <c r="C78" s="20"/>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="22"/>
-      <c r="B79" s="33" t="s">
+      <c r="A79" s="23"/>
+      <c r="B79" s="49" t="s">
         <v>65</v>
       </c>
-      <c r="C79" s="34"/>
+      <c r="C79" s="50"/>
       <c r="D79" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" s="22"/>
+      <c r="A80" s="23"/>
       <c r="B80" s="2" t="s">
         <v>6</v>
       </c>
@@ -2140,45 +2153,63 @@
       </c>
     </row>
     <row r="81" spans="1:4" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="22"/>
-      <c r="B81" s="30" t="s">
+      <c r="A81" s="23"/>
+      <c r="B81" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="C81" s="31"/>
-      <c r="D81" s="32"/>
+      <c r="C81" s="29"/>
+      <c r="D81" s="30"/>
     </row>
     <row r="82" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="21"/>
-      <c r="B82" s="23"/>
-      <c r="C82" s="24"/>
-      <c r="D82" s="7"/>
+      <c r="A82" s="22">
+        <v>46175</v>
+      </c>
+      <c r="B82" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="C82" s="25"/>
+      <c r="D82" s="7">
+        <v>2</v>
+      </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" s="22"/>
-      <c r="B83" s="29"/>
-      <c r="C83" s="26"/>
-      <c r="D83" s="8"/>
+      <c r="A83" s="23"/>
+      <c r="B83" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C83" s="27"/>
+      <c r="D83" s="8">
+        <v>3</v>
+      </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="22"/>
-      <c r="B84" s="29"/>
-      <c r="C84" s="26"/>
-      <c r="D84" s="8"/>
+      <c r="A84" s="23"/>
+      <c r="B84" s="26" t="s">
+        <v>69</v>
+      </c>
+      <c r="C84" s="27"/>
+      <c r="D84" s="8">
+        <v>2</v>
+      </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A85" s="22"/>
-      <c r="B85" s="29"/>
-      <c r="C85" s="26"/>
-      <c r="D85" s="8"/>
+      <c r="A85" s="23"/>
+      <c r="B85" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="C85" s="27"/>
+      <c r="D85" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A86" s="22"/>
-      <c r="B86" s="29"/>
-      <c r="C86" s="26"/>
+      <c r="A86" s="23"/>
+      <c r="B86" s="26"/>
+      <c r="C86" s="27"/>
       <c r="D86" s="8"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A87" s="22"/>
+      <c r="A87" s="23"/>
       <c r="B87" s="2" t="s">
         <v>6</v>
       </c>
@@ -2187,47 +2218,49 @@
       </c>
       <c r="D87" s="9">
         <f>SUM(D82:D86)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="88" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A88" s="40"/>
-      <c r="B88" s="37"/>
-      <c r="C88" s="38"/>
-      <c r="D88" s="39"/>
+      <c r="A88" s="31"/>
+      <c r="B88" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="C88" s="33"/>
+      <c r="D88" s="34"/>
     </row>
     <row r="89" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A89" s="21"/>
-      <c r="B89" s="23"/>
-      <c r="C89" s="24"/>
+      <c r="A89" s="22"/>
+      <c r="B89" s="24"/>
+      <c r="C89" s="25"/>
       <c r="D89" s="7"/>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A90" s="22"/>
-      <c r="B90" s="29"/>
-      <c r="C90" s="26"/>
+      <c r="A90" s="23"/>
+      <c r="B90" s="26"/>
+      <c r="C90" s="27"/>
       <c r="D90" s="8"/>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A91" s="22"/>
-      <c r="B91" s="29"/>
-      <c r="C91" s="26"/>
+      <c r="A91" s="23"/>
+      <c r="B91" s="26"/>
+      <c r="C91" s="27"/>
       <c r="D91" s="8"/>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A92" s="22"/>
-      <c r="B92" s="29"/>
-      <c r="C92" s="26"/>
+      <c r="A92" s="23"/>
+      <c r="B92" s="26"/>
+      <c r="C92" s="27"/>
       <c r="D92" s="8"/>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A93" s="22"/>
-      <c r="B93" s="29"/>
-      <c r="C93" s="26"/>
+      <c r="A93" s="23"/>
+      <c r="B93" s="26"/>
+      <c r="C93" s="27"/>
       <c r="D93" s="8"/>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A94" s="22"/>
+      <c r="A94" s="23"/>
       <c r="B94" s="2" t="s">
         <v>6</v>
       </c>
@@ -2240,10 +2273,10 @@
       </c>
     </row>
     <row r="95" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A95" s="40"/>
-      <c r="B95" s="37"/>
-      <c r="C95" s="38"/>
-      <c r="D95" s="39"/>
+      <c r="A95" s="31"/>
+      <c r="B95" s="32"/>
+      <c r="C95" s="33"/>
+      <c r="D95" s="34"/>
     </row>
     <row r="96" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="11"/>
@@ -2253,19 +2286,84 @@
       </c>
       <c r="D96" s="12">
         <f>D11+D18+D26+D35+D42+D49+D58+D68+D80+D87+D94</f>
-        <v>60</v>
+        <v>68</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A97" s="51" t="s">
+      <c r="A97" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B97" s="51"/>
-      <c r="C97" s="51"/>
-      <c r="D97" s="51"/>
+      <c r="B97" s="21"/>
+      <c r="C97" s="21"/>
+      <c r="D97" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="81">
+    <mergeCell ref="A20:A27"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B69:D69"/>
+    <mergeCell ref="A89:A95"/>
+    <mergeCell ref="B89:C89"/>
+    <mergeCell ref="B90:C90"/>
+    <mergeCell ref="B91:C91"/>
+    <mergeCell ref="B92:C92"/>
+    <mergeCell ref="B93:C93"/>
+    <mergeCell ref="B95:D95"/>
+    <mergeCell ref="A51:A59"/>
+    <mergeCell ref="A82:A88"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="B88:D88"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="A60:A69"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="A44:A50"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="A70:A81"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="B81:D81"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="A6:A12"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B4:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:A5"/>
     <mergeCell ref="A97:D97"/>
     <mergeCell ref="A13:A19"/>
     <mergeCell ref="B13:C13"/>
@@ -2282,71 +2380,6 @@
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="A37:A43"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="A6:A12"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B4:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A70:A81"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="B81:D81"/>
-    <mergeCell ref="A44:A50"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="A51:A59"/>
-    <mergeCell ref="A82:A88"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="B86:C86"/>
-    <mergeCell ref="B88:D88"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B59:D59"/>
-    <mergeCell ref="A60:A69"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="A89:A95"/>
-    <mergeCell ref="B89:C89"/>
-    <mergeCell ref="B90:C90"/>
-    <mergeCell ref="B91:C91"/>
-    <mergeCell ref="B92:C92"/>
-    <mergeCell ref="B93:C93"/>
-    <mergeCell ref="B95:D95"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B69:D69"/>
-    <mergeCell ref="A20:A27"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B23:C23"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="D6:D11 D13:D14 D16:D18 D20:D23 D25:D26 D60:D66 D68 D70:D72 D74:D76 D79:D80">

</xml_diff>

<commit_message>
docs: finalisation du rapport, du journal, du planning et de la documentation du code
</commit_message>
<xml_diff>
--- a/doc/GAMEZ_Journal.xlsx
+++ b/doc/GAMEZ_Journal.xlsx
@@ -1,24 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
-  <workbookPr checkCompatibility="1"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduetatfr-my.sharepoint.com/personal/thibaudfrederic_gamez_studentfr_ch/Documents/TPI/tpi2026-codementor/doc/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Informatique\tpi2026-codementor\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="254" documentId="13_ncr:1_{13CFF3CE-B7E9-4BCF-976F-778AB771C7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FF827D2-0799-4AF2-809F-03673E581825}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84CED5C3-B9F5-470E-A3BA-D040CB0A5D62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Journal" sheetId="8" r:id="rId1"/>
+    <sheet name="Journal" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Journal!$A$5:$HI$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$D$96</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">Journal!$B:$D,Journal!$1:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">Journal!$1:$5,Journal!$B:$D</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,6 +28,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,274 +37,246 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="80">
+  <si>
+    <t>Projet : CodeMentor</t>
+  </si>
+  <si>
+    <t>Gamez Thibaud</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Travail effectué</t>
+  </si>
+  <si>
+    <t>Temps</t>
+  </si>
+  <si>
+    <t>[H.h]</t>
+  </si>
+  <si>
+    <t>Lecture cahier des charges et préparation</t>
+  </si>
+  <si>
+    <t>Planning</t>
+  </si>
+  <si>
+    <t>Documentation des technos et cahier des charges</t>
+  </si>
+  <si>
+    <t>Préparation de la réunion et réunion</t>
+  </si>
+  <si>
+    <t>Réflexion personnelle ↓↓↓</t>
+  </si>
+  <si>
+    <t>Total &gt;</t>
+  </si>
+  <si>
+    <t>Début du TPI, j'ai pris plus de temps que prévu pour le planning et la documentation</t>
+  </si>
+  <si>
+    <t>Rédaction du PV et envoi</t>
+  </si>
+  <si>
+    <t>Création du diagramme des cas d'utilisation</t>
+  </si>
+  <si>
+    <t>Diagramme ER de base de données</t>
+  </si>
+  <si>
+    <t>Travail sur le diagramme de séquence système</t>
+  </si>
+  <si>
+    <t>Second jour, j'ai pu rattraper un peu le retard en avançant plus vite que prévu sur le diagramme ER et le diagramme des cas d'utilisation</t>
+  </si>
+  <si>
+    <t>Finalisation des diagrammes de séquence système (DSS2 et DSS3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Création des 3 diagrammes d'activité (Ajouter, Consulter résultats, Supprimer un projet) </t>
+  </si>
+  <si>
+    <t>Découverte d'un bug dans le diagramme des cas d'utilisation</t>
+  </si>
+  <si>
+    <t>Réparation du diagramme des cas d'utilisation</t>
+  </si>
+  <si>
+    <t>Maquette Stitch</t>
+  </si>
+  <si>
+    <t>Création du diagramme de base de données</t>
+  </si>
+  <si>
+    <t>J'ai bien avancé. J'ai découvert que mon diagramme des cas d'utilisation était cassé et j'ai dû le refaire, sinon la conception commence bien.</t>
+  </si>
+  <si>
+    <t>Diagramme de classes frontend</t>
+  </si>
+  <si>
+    <t>Diagramme de classes backend</t>
+  </si>
+  <si>
+    <t>Conception des endpoints API REST</t>
+  </si>
+  <si>
+    <t>Conception des tests</t>
+  </si>
+  <si>
+    <t>Structure MVC de base</t>
+  </si>
+  <si>
+    <t>Création de la base de données</t>
+  </si>
+  <si>
+    <t>Documentation de la conception</t>
+  </si>
+  <si>
+    <t>Cette journée s'est bien passée, j'ai pu commencer l'implémentation du backend en créant la structure de base et la base de données. Je suis confiant.</t>
+  </si>
+  <si>
+    <t>La table "suggested_fix" complique les choses et n'est pas très utile</t>
+  </si>
+  <si>
+    <t>Suppression et changement des schémas et de la structure du code</t>
+  </si>
+  <si>
+    <t>Ajout des tâches de la to-do list</t>
+  </si>
+  <si>
+    <t>Documentation</t>
+  </si>
+  <si>
+    <t>J'ai pris du retard sur l'implémentation, mais je ne pense pas que ça posera problème.</t>
+  </si>
+  <si>
+    <t>Finalisation de la documentation d'analyse</t>
+  </si>
+  <si>
+    <t>Finalisation de la documentation de conception</t>
+  </si>
+  <si>
+    <t>J'ai fait uniquement de la documentation, je suis donc toujours en retard, mais je vais pouvoir le rattraper demain.</t>
+  </si>
+  <si>
+    <t>Réflexion sur les modèles et décision de ne pas en faire</t>
+  </si>
+  <si>
+    <t>Implémentation de l'authentification GitHub</t>
+  </si>
+  <si>
+    <t>Rendez-vous avec Meylan</t>
+  </si>
+  <si>
+    <t>Service et endpoints des projets</t>
+  </si>
+  <si>
+    <t>Implémentation du service GitHub</t>
+  </si>
+  <si>
+    <t>Je me suis rendu compte après l'implémentation des modèles qu'ils étaient en fait inutiles, j'ai donc décidé de les retirer du code. L'implémentation de l'authentification via GitHub fonctionne parfaitement, les endpoints de projets sont faits et la récupération des fichiers et projets GitHub aussi. Je rattrape mon léger retard.</t>
+  </si>
+  <si>
+    <t>Mise en place de la queue en mémoire</t>
+  </si>
+  <si>
+    <t>Mise en place de l'analyse via le LLM</t>
+  </si>
+  <si>
+    <t>Prompt système du LLM</t>
+  </si>
+  <si>
+    <t>Endpoint de suivi de l'état des tâches</t>
+  </si>
+  <si>
+    <t>Sécurisation des accès (projets / analyses)</t>
+  </si>
+  <si>
+    <t>Documentation Swagger</t>
+  </si>
+  <si>
+    <t>Rendez-vous avec les experts</t>
+  </si>
+  <si>
+    <t>La journée s'est bien passée, les différents endpoints fonctionnent et je suis confiant pour la suite.</t>
+  </si>
+  <si>
+    <t>Amélioration backend</t>
+  </si>
+  <si>
+    <t>Mise en place du projet Vue.js + structure de base</t>
+  </si>
+  <si>
+    <t>Configuration du routing</t>
+  </si>
+  <si>
+    <t>Service API + interception du token</t>
+  </si>
+  <si>
+    <t>Page de connexion</t>
+  </si>
+  <si>
+    <t>Page de liste et création des projets</t>
+  </si>
+  <si>
+    <t>Page de détail de projet (Detected Errors, Suggested Fixes)</t>
+  </si>
+  <si>
+    <t>Intégration du polling de la progression</t>
+  </si>
+  <si>
+    <t>Traitement des analyses très lent</t>
+  </si>
+  <si>
+    <t>Traitement par lots parallèles avec "Promise.all"</t>
+  </si>
+  <si>
+    <t>La journée a bien avancé, le frontend est fonctionnel de bout en bout et communique correctement avec le backend. Il me reste surtout à peaufiner le design et à documenter le tout. Je ne pensais pas que les requêtes LLM seraient si lentes, j'ai dû ajouter un traitement parallèle pour analyser plusieurs fichiers en même temps.</t>
+  </si>
+  <si>
+    <t>Responsive design et corrections de design</t>
+  </si>
+  <si>
+    <t>Tests de différents modèles et analyse de leurs retours</t>
+  </si>
+  <si>
+    <t>Correction des erreurs dans les schémas EA</t>
+  </si>
+  <si>
+    <t>J'ai terminé la partie frontend, j'ai aussi bien avancé la documentation et j'ai pu faire des tests sur différents LLM afin de constater les différences et d'adapter le prompt système. Le retard est rattrapé, je n'ai plus de doutes sur la faisabilité du projet.</t>
+  </si>
+  <si>
+    <t>Travail sur la documentation</t>
+  </si>
+  <si>
+    <t>Tests du backend</t>
+  </si>
+  <si>
+    <t>Tests du frontend</t>
+  </si>
+  <si>
+    <t>Tests de sécurité</t>
+  </si>
+  <si>
+    <t>La documentation a bien avancé, il manque encore quelques points à perfectionner, sinon tout est OK.</t>
+  </si>
+  <si>
+    <t>Finalisation du rapport et préparation du rendu</t>
+  </si>
+  <si>
+    <t>Remise du projet (code, documentation, journal de travail)</t>
+  </si>
+  <si>
+    <t>Dernier jour du TPI. J'ai finalisé le rapport de projet, vérifié tous les livrables et effectué la remise du projet. Tout s'est bien déroulé.</t>
+  </si>
+  <si>
+    <t>Total général &gt;</t>
+  </si>
   <si>
     <t>Insérer les lignes au-dessus de celle-ci !</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Travail effectué</t>
-  </si>
-  <si>
-    <t>[H.h]</t>
-  </si>
-  <si>
-    <t>Temps</t>
-  </si>
-  <si>
-    <t>Total &gt;</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Réflexion personnelle </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>↓↓↓</t>
-    </r>
-  </si>
-  <si>
-    <t>Total général &gt;</t>
-  </si>
-  <si>
-    <r>
-      <t>Projet :</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>CodeMentor</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="16"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">                      </t>
-    </r>
-  </si>
-  <si>
-    <t>Gamez Thibaud</t>
-  </si>
-  <si>
-    <t>Lecture cahier des charges et préparation</t>
-  </si>
-  <si>
-    <t>Planning</t>
-  </si>
-  <si>
-    <t>Documentation des technos et cahier des charges</t>
-  </si>
-  <si>
-    <t>Préparation de la réunion et réunion</t>
-  </si>
-  <si>
-    <t>Rédaction du PV et envoie</t>
-  </si>
-  <si>
-    <t>Création du diagramme usecase</t>
-  </si>
-  <si>
-    <t>Travail sur le diagramme de séquence système</t>
-  </si>
-  <si>
-    <t>Début du TPI, j'ai pris plus de temps que prévu pour le planning et la documentation</t>
-  </si>
-  <si>
-    <t>diagramme ER de base de données</t>
-  </si>
-  <si>
-    <t>Second jour, j'ai pu rattraper un peu le retard en avancant plus vite que prévu sur le diagramme ER et le usecase</t>
-  </si>
-  <si>
-    <t>Finalisation diagrammes de séquence système (DSS2 et DSS3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Création des 3 diagrammes d'activité (Ajouter, Consulter résultats, Supprimer un projet) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réparation du diagramme des cas d'utilisation </t>
-  </si>
-  <si>
-    <t>Decouverte d'un bug dans le diagramme des cas d'utilisation</t>
-  </si>
-  <si>
-    <t>Maquette Stitch</t>
-  </si>
-  <si>
-    <t>Création du diagramme de base de donnée</t>
-  </si>
-  <si>
-    <t>J'ai bien avancé, j'ai découvert que mon usecase était cassé et j'ai du le refaire sinon la conception commence bien</t>
-  </si>
-  <si>
-    <t>Diagramme de classe frontend</t>
-  </si>
-  <si>
-    <t>Diagramme de classe backend</t>
-  </si>
-  <si>
-    <t>Conception des endpoints API REST</t>
-  </si>
-  <si>
-    <t>Conception des tests</t>
-  </si>
-  <si>
-    <t>Structure MVC de base</t>
-  </si>
-  <si>
-    <t>Création base de donnée</t>
-  </si>
-  <si>
-    <t>Documentation conception</t>
-  </si>
-  <si>
-    <t>Cette journée s'est bien passé, j'ai pu commencer l'implementation du backend en faisant la structure de base et la base de donnée. Je suis confiant</t>
-  </si>
-  <si>
-    <t>La table "suggested_fix" complique les choses et n'est pas très utile</t>
-  </si>
-  <si>
-    <t>Supression et changement des schémas et de la structure du code</t>
-  </si>
-  <si>
-    <t>Ajout des tâches todolist</t>
-  </si>
-  <si>
-    <t>Documentation</t>
-  </si>
-  <si>
-    <t>J'ai pris du retard sur l'implémentation mais je pense pas que ca poseras problème</t>
-  </si>
-  <si>
-    <t>Finalisation doc analyse</t>
-  </si>
-  <si>
-    <t>Finalisation doc conception</t>
-  </si>
-  <si>
-    <t>J'ai fais que de la documentation, toujours en retard du coup mais vais pouvoir le rattraper demain</t>
-  </si>
-  <si>
-    <t>Réflexion sur les modèles et décision de ne pas en faire</t>
-  </si>
-  <si>
-    <t>Implémentation authentification github</t>
-  </si>
-  <si>
-    <t>Rendez-vous avec Meylan</t>
-  </si>
-  <si>
-    <t>Implémentation du service github</t>
-  </si>
-  <si>
-    <t>Service et endspoints projets</t>
-  </si>
-  <si>
-    <t>Je me suis rendu compte après implémentation des modèles qu'ils étaient en fait inutile, j'ai donc décider de les retiré du code. L'implementation de l'authentification via github fonctionne parfaitement, les endpoints de projet sont fait et la récuperation des fichiers et projets git hub aussi. Je rattrapes mon leger retard</t>
-  </si>
-  <si>
-    <t>Mise en place de la queue en mémoire</t>
-  </si>
-  <si>
-    <t>Mise en place de l'analyse via le LLM</t>
-  </si>
-  <si>
-    <t>Endpoint de suivi d'état des tâches</t>
-  </si>
-  <si>
-    <t>Documentation swagger</t>
-  </si>
-  <si>
-    <t>Rendez-vous avec les experts</t>
-  </si>
-  <si>
-    <t>Sécurisation des accès (projet / analyse)</t>
-  </si>
-  <si>
-    <t>Système prompt llm</t>
-  </si>
-  <si>
-    <t>La journée s'est bien passé, les différents endpoints fonctionnes et je suis confiant pour la suite</t>
-  </si>
-  <si>
-    <t>Mise en place du projet Vue.js + structure de base</t>
-  </si>
-  <si>
-    <t>Configuration du routing</t>
-  </si>
-  <si>
-    <t>Service API + interception du token</t>
-  </si>
-  <si>
-    <t>Page de connexion</t>
-  </si>
-  <si>
-    <t>Page de liste et création des projets</t>
-  </si>
-  <si>
-    <t>Page de détail projet (Detected Errors, Suggested Fixes)</t>
-  </si>
-  <si>
-    <t>Intégration du polling de la progression</t>
-  </si>
-  <si>
-    <t>Traitement des analyses super lent</t>
-  </si>
-  <si>
-    <t>Traitement par lots parallèles avec "Promise.all"</t>
-  </si>
-  <si>
-    <t>La journée a bien avancé, le frontend est fonctionnel de bout en bout et communique correctement avec le backend. Il me reste surtout à peaufiner le design et surtout documenté le tout. Je ne pensais pas que les requêtes LLM seraient si lentes, j'ai du ajouter un traitemnet parallèles pour analysé plusieurs fichiers en même temps</t>
-  </si>
-  <si>
-    <t>Amélioration backend</t>
-  </si>
-  <si>
-    <t>Responsive design et correction design</t>
-  </si>
-  <si>
-    <t>Tests de différents modèles et analyse de leurs retours</t>
-  </si>
-  <si>
-    <t>Correction erreurs dans schémas EA</t>
-  </si>
-  <si>
-    <t>J'ai terminé la partie frontend, j'ai aussi bien avancé la documentation et j'ai pu faire des tests sur différents LLM afin de constaté les différents et adapté le système prompt. Le retard est rattrapé, j'ai plus de doutes sur la faisabilité du projet.</t>
-  </si>
-  <si>
-    <t>Travail sur la documentation</t>
-  </si>
-  <si>
-    <t>Tests backend</t>
-  </si>
-  <si>
-    <t>Tests frontend</t>
-  </si>
-  <si>
-    <t>Tests sécurité</t>
-  </si>
-  <si>
-    <t>La documentation à bien avancé, il manque encore quelques points à perfectionner sinon tout est ok.</t>
   </si>
 </sst>
 </file>
@@ -311,10 +284,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="dd/mm/yy;@"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -326,12 +299,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
@@ -339,11 +306,6 @@
     </font>
     <font>
       <sz val="8"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="16"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -361,11 +323,6 @@
     <font>
       <sz val="9"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
@@ -518,7 +475,18 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top style="medium">
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom/>
@@ -530,40 +498,7 @@
       </left>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -619,24 +554,52 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
@@ -644,190 +607,193 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1022,10 +988,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1376,109 +1338,110 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D102"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="1"/>
+    <col min="1" max="1" width="11.5703125" style="1" customWidth="1"/>
     <col min="2" max="3" width="31.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="15.7109375" style="1" customWidth="1"/>
     <col min="5" max="217" width="9.140625" style="1" customWidth="1"/>
-    <col min="218" max="16384" width="11.5703125" style="1"/>
+    <col min="218" max="218" width="11.5703125" style="1" customWidth="1"/>
+    <col min="219" max="16384" width="11.5703125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-    </row>
-    <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="49" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="50"/>
+    <row r="1" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="61" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+    </row>
+    <row r="2" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="59" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="45"/>
+      <c r="C2" s="27"/>
       <c r="D2" s="4">
         <v>151446</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="43" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="43" t="s">
+      <c r="A4" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="44"/>
+      <c r="B4" s="46" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="36"/>
       <c r="D4" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="45"/>
-      <c r="B5" s="45"/>
-      <c r="C5" s="46"/>
+    <row r="5" spans="1:4" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="47"/>
+      <c r="B5" s="47"/>
+      <c r="C5" s="48"/>
       <c r="D5" s="6" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="41">
+      <c r="A6" s="63">
         <v>46153</v>
       </c>
-      <c r="B6" s="47" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="48"/>
+      <c r="B6" s="52" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="53"/>
       <c r="D6" s="7">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="22"/>
-      <c r="B7" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="26"/>
+      <c r="A7" s="31"/>
+      <c r="B7" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="27"/>
       <c r="D7" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="22"/>
-      <c r="B8" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="26"/>
+      <c r="A8" s="31"/>
+      <c r="B8" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="27"/>
       <c r="D8" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="22"/>
-      <c r="B9" s="35" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="36"/>
+      <c r="A9" s="31"/>
+      <c r="B9" s="43" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="27"/>
       <c r="D9" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="22"/>
-      <c r="B10" s="29"/>
-      <c r="C10" s="26"/>
+      <c r="A10" s="31"/>
+      <c r="B10" s="26"/>
+      <c r="C10" s="27"/>
       <c r="D10" s="8"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="22"/>
+      <c r="A11" s="31"/>
       <c r="B11" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D11" s="9">
         <f>SUM(D6:D10)</f>
@@ -1486,67 +1449,67 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="22"/>
-      <c r="B12" s="30" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="31"/>
-      <c r="D12" s="32"/>
+      <c r="A12" s="31"/>
+      <c r="B12" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="45"/>
+      <c r="D12" s="27"/>
     </row>
     <row r="13" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="21">
+      <c r="A13" s="30">
         <v>46154</v>
       </c>
-      <c r="B13" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" s="24"/>
+      <c r="B13" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="36"/>
       <c r="D13" s="7">
         <v>0.5</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="22"/>
-      <c r="B14" s="29" t="s">
+      <c r="A14" s="31"/>
+      <c r="B14" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="27"/>
+      <c r="D14" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="31"/>
+      <c r="B15" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="26"/>
-      <c r="D14" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="22"/>
-      <c r="B15" s="13" t="s">
-        <v>18</v>
-      </c>
       <c r="D15" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="22"/>
-      <c r="B16" s="29" t="s">
+      <c r="A16" s="31"/>
+      <c r="B16" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="26"/>
+      <c r="C16" s="27"/>
       <c r="D16" s="8">
         <v>1.5</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="22"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="26"/>
+      <c r="A17" s="31"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="27"/>
       <c r="D17" s="8"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="22"/>
+      <c r="A18" s="31"/>
       <c r="B18" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D18" s="9">
         <f>SUM(D13:D17)</f>
@@ -1554,80 +1517,80 @@
       </c>
     </row>
     <row r="19" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="22"/>
-      <c r="B19" s="30" t="s">
-        <v>19</v>
-      </c>
-      <c r="C19" s="31"/>
-      <c r="D19" s="32"/>
+      <c r="A19" s="31"/>
+      <c r="B19" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="45"/>
+      <c r="D19" s="27"/>
     </row>
     <row r="20" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="21">
+      <c r="A20" s="30">
         <v>46157</v>
       </c>
-      <c r="B20" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="C20" s="24"/>
+      <c r="B20" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="36"/>
       <c r="D20" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="22"/>
-      <c r="B21" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="C21" s="26"/>
+      <c r="A21" s="31"/>
+      <c r="B21" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="27"/>
       <c r="D21" s="8">
         <v>2.5</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="22"/>
-      <c r="B22" s="27" t="s">
-        <v>23</v>
-      </c>
-      <c r="C22" s="28"/>
+      <c r="A22" s="31"/>
+      <c r="B22" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="27"/>
       <c r="D22" s="8"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="22"/>
-      <c r="B23" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="C23" s="34"/>
+      <c r="A23" s="31"/>
+      <c r="B23" s="54" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" s="27"/>
       <c r="D23" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="22"/>
-      <c r="B24" s="29" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="26"/>
+      <c r="A24" s="31"/>
+      <c r="B24" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="27"/>
       <c r="D24" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="22"/>
-      <c r="B25" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="C25" s="26"/>
+      <c r="A25" s="31"/>
+      <c r="B25" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" s="27"/>
       <c r="D25" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="22"/>
+      <c r="A26" s="31"/>
       <c r="B26" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D26" s="9">
         <f>SUM(D20:D25)</f>
@@ -1635,59 +1598,59 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="22"/>
-      <c r="B27" s="30" t="s">
+      <c r="A27" s="31"/>
+      <c r="B27" s="44" t="s">
+        <v>24</v>
+      </c>
+      <c r="C27" s="45"/>
+      <c r="D27" s="27"/>
+    </row>
+    <row r="28" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="38">
+        <v>46160</v>
+      </c>
+      <c r="B28" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="C28" s="36"/>
+      <c r="D28" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" s="31"/>
+      <c r="B29" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="31"/>
-      <c r="D27" s="32"/>
-    </row>
-    <row r="28" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="21">
-        <v>46160</v>
-      </c>
-      <c r="B28" s="23" t="s">
+      <c r="C29" s="27"/>
+      <c r="D29" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" s="31"/>
+      <c r="B30" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="24"/>
-      <c r="D28" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="22"/>
-      <c r="B29" s="29" t="s">
+      <c r="C30" s="27"/>
+      <c r="D30" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="31"/>
+      <c r="B31" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="26"/>
-      <c r="D29" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="22"/>
-      <c r="B30" s="29" t="s">
+      <c r="C31" s="27"/>
+      <c r="D31" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="31"/>
+      <c r="B32" s="14" t="s">
         <v>29</v>
-      </c>
-      <c r="C30" s="26"/>
-      <c r="D30" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="22"/>
-      <c r="B31" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="C31" s="26"/>
-      <c r="D31" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="22"/>
-      <c r="B32" s="14" t="s">
-        <v>31</v>
       </c>
       <c r="C32" s="15"/>
       <c r="D32" s="8">
@@ -1695,9 +1658,9 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="22"/>
+      <c r="A33" s="31"/>
       <c r="B33" s="14" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C33" s="15"/>
       <c r="D33" s="8">
@@ -1705,22 +1668,22 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="22"/>
-      <c r="B34" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="C34" s="26"/>
+      <c r="A34" s="31"/>
+      <c r="B34" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="C34" s="27"/>
       <c r="D34" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="22"/>
+      <c r="A35" s="31"/>
       <c r="B35" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D35" s="9">
         <f>SUM(D28:D34)</f>
@@ -1728,19 +1691,19 @@
       </c>
     </row>
     <row r="36" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="40"/>
-      <c r="B36" s="37" t="s">
-        <v>34</v>
-      </c>
-      <c r="C36" s="38"/>
-      <c r="D36" s="39"/>
+      <c r="A36" s="39"/>
+      <c r="B36" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="C36" s="41"/>
+      <c r="D36" s="42"/>
     </row>
     <row r="37" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="21">
+      <c r="A37" s="38">
         <v>46161</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C37" s="17"/>
       <c r="D37" s="7">
@@ -1748,48 +1711,48 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="22"/>
-      <c r="B38" s="52" t="s">
-        <v>36</v>
-      </c>
-      <c r="C38" s="53"/>
+      <c r="A38" s="31"/>
+      <c r="B38" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="C38" s="36"/>
       <c r="D38" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="22"/>
-      <c r="B39" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="C39" s="26"/>
+      <c r="A39" s="31"/>
+      <c r="B39" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="C39" s="27"/>
       <c r="D39" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="22"/>
-      <c r="B40" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="C40" s="26"/>
+      <c r="A40" s="31"/>
+      <c r="B40" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="C40" s="27"/>
       <c r="D40" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="22"/>
-      <c r="B41" s="29"/>
-      <c r="C41" s="26"/>
+      <c r="A41" s="31"/>
+      <c r="B41" s="26"/>
+      <c r="C41" s="27"/>
       <c r="D41" s="8"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="22"/>
+      <c r="A42" s="31"/>
       <c r="B42" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D42" s="9">
         <f>SUM(D37:D41)</f>
@@ -1797,60 +1760,60 @@
       </c>
     </row>
     <row r="43" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="40"/>
-      <c r="B43" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="C43" s="38"/>
-      <c r="D43" s="39"/>
+      <c r="A43" s="39"/>
+      <c r="B43" s="40" t="s">
+        <v>37</v>
+      </c>
+      <c r="C43" s="41"/>
+      <c r="D43" s="42"/>
     </row>
     <row r="44" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="21">
+      <c r="A44" s="38">
         <v>46163</v>
       </c>
-      <c r="B44" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="C44" s="24"/>
+      <c r="B44" s="35" t="s">
+        <v>38</v>
+      </c>
+      <c r="C44" s="36"/>
       <c r="D44" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="22"/>
-      <c r="B45" s="29" t="s">
-        <v>41</v>
-      </c>
-      <c r="C45" s="26"/>
+      <c r="A45" s="31"/>
+      <c r="B45" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="C45" s="27"/>
       <c r="D45" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="22"/>
-      <c r="B46" s="29"/>
-      <c r="C46" s="26"/>
+      <c r="A46" s="31"/>
+      <c r="B46" s="26"/>
+      <c r="C46" s="27"/>
       <c r="D46" s="8"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="22"/>
-      <c r="B47" s="29"/>
-      <c r="C47" s="26"/>
+      <c r="A47" s="31"/>
+      <c r="B47" s="26"/>
+      <c r="C47" s="27"/>
       <c r="D47" s="8"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="22"/>
-      <c r="B48" s="29"/>
-      <c r="C48" s="26"/>
+      <c r="A48" s="31"/>
+      <c r="B48" s="26"/>
+      <c r="C48" s="27"/>
       <c r="D48" s="8"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="22"/>
+      <c r="A49" s="31"/>
       <c r="B49" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D49" s="9">
         <f>SUM(D44:D48)</f>
@@ -1858,69 +1821,69 @@
       </c>
     </row>
     <row r="50" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="40"/>
-      <c r="B50" s="37" t="s">
+      <c r="A50" s="39"/>
+      <c r="B50" s="40" t="s">
+        <v>40</v>
+      </c>
+      <c r="C50" s="41"/>
+      <c r="D50" s="42"/>
+    </row>
+    <row r="51" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="38">
+        <v>46164</v>
+      </c>
+      <c r="B51" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="C51" s="36"/>
+      <c r="D51" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" s="31"/>
+      <c r="B52" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="C50" s="38"/>
-      <c r="D50" s="39"/>
-    </row>
-    <row r="51" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="21">
-        <v>46164</v>
-      </c>
-      <c r="B51" s="23" t="s">
+      <c r="C52" s="27"/>
+      <c r="D52" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" s="31"/>
+      <c r="B53" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="C51" s="24"/>
-      <c r="D51" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="22"/>
-      <c r="B52" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="C52" s="26"/>
-      <c r="D52" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="22"/>
-      <c r="B53" s="29" t="s">
-        <v>45</v>
-      </c>
-      <c r="C53" s="26"/>
+      <c r="C53" s="27"/>
       <c r="D53" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="22"/>
-      <c r="B54" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="C54" s="26"/>
+      <c r="A54" s="31"/>
+      <c r="B54" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="C54" s="27"/>
       <c r="D54" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" s="22"/>
-      <c r="B55" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="C55" s="26"/>
+      <c r="A55" s="31"/>
+      <c r="B55" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="C55" s="27"/>
       <c r="D55" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="22"/>
+      <c r="A56" s="31"/>
       <c r="B56" s="14" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C56" s="15"/>
       <c r="D56" s="8">
@@ -1928,9 +1891,9 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" s="22"/>
+      <c r="A57" s="31"/>
       <c r="B57" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C57" s="15"/>
       <c r="D57" s="8">
@@ -1938,12 +1901,12 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" s="22"/>
+      <c r="A58" s="31"/>
       <c r="B58" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D58" s="9">
         <f>SUM(D51:D57)</f>
@@ -1951,39 +1914,39 @@
       </c>
     </row>
     <row r="59" spans="1:4" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="40"/>
-      <c r="B59" s="37" t="s">
-        <v>48</v>
-      </c>
-      <c r="C59" s="38"/>
-      <c r="D59" s="39"/>
+      <c r="A59" s="39"/>
+      <c r="B59" s="40" t="s">
+        <v>46</v>
+      </c>
+      <c r="C59" s="41"/>
+      <c r="D59" s="42"/>
     </row>
     <row r="60" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="21">
+      <c r="A60" s="38">
         <v>46171</v>
       </c>
-      <c r="B60" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="C60" s="24"/>
+      <c r="B60" s="35" t="s">
+        <v>47</v>
+      </c>
+      <c r="C60" s="36"/>
       <c r="D60" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" s="22"/>
-      <c r="B61" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="C61" s="26"/>
+      <c r="A61" s="31"/>
+      <c r="B61" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="C61" s="27"/>
       <c r="D61" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="22"/>
+      <c r="A62" s="31"/>
       <c r="B62" s="14" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C62" s="15"/>
       <c r="D62" s="8">
@@ -1991,19 +1954,19 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="22"/>
-      <c r="B63" s="29" t="s">
+      <c r="A63" s="31"/>
+      <c r="B63" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="C63" s="27"/>
+      <c r="D63" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" s="31"/>
+      <c r="B64" s="18" t="s">
         <v>51</v>
-      </c>
-      <c r="C63" s="26"/>
-      <c r="D63" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="22"/>
-      <c r="B64" s="18" t="s">
-        <v>54</v>
       </c>
       <c r="C64" s="15"/>
       <c r="D64" s="8">
@@ -2011,35 +1974,35 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" s="22"/>
-      <c r="B65" s="29" t="s">
+      <c r="A65" s="31"/>
+      <c r="B65" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="C65" s="26"/>
+      <c r="C65" s="27"/>
       <c r="D65" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" s="22"/>
-      <c r="B66" s="35" t="s">
+      <c r="A66" s="31"/>
+      <c r="B66" s="43" t="s">
         <v>53</v>
       </c>
-      <c r="C66" s="36"/>
+      <c r="C66" s="27"/>
       <c r="D66" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="22"/>
+      <c r="A67" s="31"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="22"/>
+      <c r="A68" s="31"/>
       <c r="B68" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D68" s="9">
         <f>SUM(D60:D66)</f>
@@ -2047,29 +2010,29 @@
       </c>
     </row>
     <row r="69" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="40"/>
-      <c r="B69" s="37" t="s">
-        <v>56</v>
-      </c>
-      <c r="C69" s="38"/>
-      <c r="D69" s="39"/>
+      <c r="A69" s="39"/>
+      <c r="B69" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="C69" s="41"/>
+      <c r="D69" s="42"/>
     </row>
     <row r="70" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="21">
+      <c r="A70" s="30">
         <v>46174</v>
       </c>
-      <c r="B70" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="C70" s="24"/>
+      <c r="B70" s="35" t="s">
+        <v>55</v>
+      </c>
+      <c r="C70" s="36"/>
       <c r="D70" s="7">
         <v>0.5</v>
       </c>
     </row>
     <row r="71" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="22"/>
+      <c r="A71" s="31"/>
       <c r="B71" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C71" s="15"/>
       <c r="D71" s="7">
@@ -2077,39 +2040,39 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="22"/>
-      <c r="B72" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="C72" s="26"/>
+      <c r="A72" s="31"/>
+      <c r="B72" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="C72" s="27"/>
       <c r="D72" s="7">
         <v>0.75</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" s="22"/>
-      <c r="B73" s="29" t="s">
+      <c r="A73" s="31"/>
+      <c r="B73" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="C73" s="27"/>
+      <c r="D73" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" s="31"/>
+      <c r="B74" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="C73" s="26"/>
-      <c r="D73" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="22"/>
-      <c r="B74" s="29" t="s">
-        <v>60</v>
-      </c>
-      <c r="C74" s="26"/>
+      <c r="C74" s="27"/>
       <c r="D74" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="22"/>
+      <c r="A75" s="31"/>
       <c r="B75" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C75" s="15"/>
       <c r="D75" s="8">
@@ -2117,9 +2080,9 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="22"/>
+      <c r="A76" s="31"/>
       <c r="B76" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C76" s="15"/>
       <c r="D76" s="8">
@@ -2127,9 +2090,9 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="22"/>
+      <c r="A77" s="31"/>
       <c r="B77" s="14" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C77" s="15"/>
       <c r="D77" s="1">
@@ -2137,29 +2100,29 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="22"/>
+      <c r="A78" s="31"/>
       <c r="B78" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="C78" s="20"/>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" s="31"/>
+      <c r="B79" s="54" t="s">
         <v>64</v>
       </c>
-      <c r="C78" s="20"/>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="22"/>
-      <c r="B79" s="33" t="s">
-        <v>65</v>
-      </c>
-      <c r="C79" s="34"/>
+      <c r="C79" s="27"/>
       <c r="D79" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" s="22"/>
+      <c r="A80" s="31"/>
       <c r="B80" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D80" s="9">
         <f>SUM(D70:D79)</f>
@@ -2167,68 +2130,68 @@
       </c>
     </row>
     <row r="81" spans="1:4" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="22"/>
-      <c r="B81" s="30" t="s">
+      <c r="A81" s="31"/>
+      <c r="B81" s="44" t="s">
+        <v>65</v>
+      </c>
+      <c r="C81" s="45"/>
+      <c r="D81" s="27"/>
+    </row>
+    <row r="82" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A82" s="38">
+        <v>46175</v>
+      </c>
+      <c r="B82" s="35" t="s">
         <v>66</v>
       </c>
-      <c r="C81" s="31"/>
-      <c r="D81" s="32"/>
-    </row>
-    <row r="82" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="21">
-        <v>46175</v>
-      </c>
-      <c r="B82" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="C82" s="24"/>
+      <c r="C82" s="36"/>
       <c r="D82" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" s="22"/>
-      <c r="B83" s="29" t="s">
-        <v>38</v>
-      </c>
-      <c r="C83" s="26"/>
+      <c r="A83" s="31"/>
+      <c r="B83" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="C83" s="27"/>
       <c r="D83" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="22"/>
-      <c r="B84" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="C84" s="26"/>
+      <c r="A84" s="31"/>
+      <c r="B84" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="C84" s="27"/>
       <c r="D84" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A85" s="22"/>
-      <c r="B85" s="29" t="s">
-        <v>70</v>
-      </c>
-      <c r="C85" s="26"/>
+      <c r="A85" s="31"/>
+      <c r="B85" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="C85" s="27"/>
       <c r="D85" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A86" s="22"/>
-      <c r="B86" s="29"/>
-      <c r="C86" s="26"/>
+      <c r="A86" s="31"/>
+      <c r="B86" s="26"/>
+      <c r="C86" s="27"/>
       <c r="D86" s="8"/>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A87" s="22"/>
+      <c r="A87" s="31"/>
       <c r="B87" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D87" s="9">
         <f>SUM(D82:D86)</f>
@@ -2236,68 +2199,68 @@
       </c>
     </row>
     <row r="88" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A88" s="40"/>
-      <c r="B88" s="37" t="s">
-        <v>71</v>
-      </c>
-      <c r="C88" s="38"/>
-      <c r="D88" s="39"/>
+      <c r="A88" s="39"/>
+      <c r="B88" s="40" t="s">
+        <v>69</v>
+      </c>
+      <c r="C88" s="41"/>
+      <c r="D88" s="42"/>
     </row>
     <row r="89" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A89" s="21">
+      <c r="A89" s="38">
         <v>46178</v>
       </c>
-      <c r="B89" s="23" t="s">
-        <v>72</v>
-      </c>
-      <c r="C89" s="24"/>
+      <c r="B89" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C89" s="36"/>
       <c r="D89" s="7">
         <v>4</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A90" s="22"/>
-      <c r="B90" s="29" t="s">
-        <v>73</v>
-      </c>
-      <c r="C90" s="26"/>
+      <c r="A90" s="31"/>
+      <c r="B90" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="C90" s="27"/>
       <c r="D90" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A91" s="22"/>
-      <c r="B91" s="29" t="s">
-        <v>74</v>
-      </c>
-      <c r="C91" s="26"/>
+      <c r="A91" s="31"/>
+      <c r="B91" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="C91" s="27"/>
       <c r="D91" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A92" s="22"/>
-      <c r="B92" s="29" t="s">
-        <v>75</v>
-      </c>
-      <c r="C92" s="26"/>
+      <c r="A92" s="31"/>
+      <c r="B92" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="C92" s="27"/>
       <c r="D92" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A93" s="22"/>
-      <c r="B93" s="29"/>
-      <c r="C93" s="26"/>
+      <c r="A93" s="31"/>
+      <c r="B93" s="26"/>
+      <c r="C93" s="27"/>
       <c r="D93" s="8"/>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A94" s="22"/>
+      <c r="A94" s="31"/>
       <c r="B94" s="2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D94" s="9">
         <f>SUM(D89:D93)</f>
@@ -2305,117 +2268,170 @@
       </c>
     </row>
     <row r="95" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A95" s="40"/>
-      <c r="B95" s="37" t="s">
+      <c r="A95" s="39"/>
+      <c r="B95" s="40" t="s">
+        <v>74</v>
+      </c>
+      <c r="C95" s="41"/>
+      <c r="D95" s="42"/>
+    </row>
+    <row r="96" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A96" s="32">
+        <v>46181</v>
+      </c>
+      <c r="B96" s="57" t="s">
+        <v>75</v>
+      </c>
+      <c r="C96" s="58"/>
+      <c r="D96" s="21">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A97" s="33"/>
+      <c r="B97" s="55" t="s">
         <v>76</v>
       </c>
-      <c r="C95" s="38"/>
-      <c r="D95" s="39"/>
-    </row>
-    <row r="96" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="11"/>
-      <c r="B96" s="10"/>
-      <c r="C96" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D96" s="12">
-        <f>D11+D18+D26+D35+D42+D49+D58+D68+D80+D87+D94</f>
-        <v>76</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A97" s="51" t="s">
-        <v>0</v>
-      </c>
-      <c r="B97" s="51"/>
-      <c r="C97" s="51"/>
-      <c r="D97" s="51"/>
+      <c r="C97" s="56"/>
+      <c r="D97" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A98" s="33"/>
+      <c r="B98" s="55"/>
+      <c r="C98" s="56"/>
+      <c r="D98" s="22"/>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A99" s="33"/>
+      <c r="B99" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C99" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D99" s="25">
+        <f>SUM(D96:D98)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A100" s="34"/>
+      <c r="B100" s="49" t="s">
+        <v>77</v>
+      </c>
+      <c r="C100" s="50"/>
+      <c r="D100" s="51"/>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A101" s="11"/>
+      <c r="B101" s="10"/>
+      <c r="C101" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D101" s="12">
+        <f>D11+D18+D26+D35+D42+D49+D58+D68+D80+D87+D94+D99</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A102" s="60" t="s">
+        <v>79</v>
+      </c>
+      <c r="B102" s="45"/>
+      <c r="C102" s="45"/>
+      <c r="D102" s="45"/>
     </row>
   </sheetData>
-  <mergeCells count="81">
-    <mergeCell ref="A97:D97"/>
-    <mergeCell ref="A13:A19"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B16:C16"/>
+  <mergeCells count="86">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="A70:A81"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="A37:A43"/>
+    <mergeCell ref="B69:D69"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A102:D102"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B98:C98"/>
+    <mergeCell ref="A60:A69"/>
+    <mergeCell ref="B60:C60"/>
     <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="A28:A36"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="A37:A43"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="A6:A12"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B4:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A70:A81"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="B81:D81"/>
-    <mergeCell ref="A44:A50"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="A51:A59"/>
-    <mergeCell ref="A82:A88"/>
     <mergeCell ref="B82:C82"/>
     <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B92:C92"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="A89:A95"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B100:D100"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="A20:A27"/>
+    <mergeCell ref="B89:C89"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="B97:C97"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B96:C96"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B95:D95"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="A44:A50"/>
+    <mergeCell ref="B4:C5"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A51:A59"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="A6:A12"/>
+    <mergeCell ref="A13:A19"/>
+    <mergeCell ref="A96:A100"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="A28:A36"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="A82:A88"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B91:C91"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B93:C93"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B90:C90"/>
+    <mergeCell ref="B88:D88"/>
+    <mergeCell ref="B66:C66"/>
     <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="B86:C86"/>
-    <mergeCell ref="B88:D88"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B59:D59"/>
-    <mergeCell ref="A60:A69"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="A89:A95"/>
-    <mergeCell ref="B89:C89"/>
-    <mergeCell ref="B90:C90"/>
-    <mergeCell ref="B91:C91"/>
-    <mergeCell ref="B92:C92"/>
-    <mergeCell ref="B93:C93"/>
-    <mergeCell ref="B95:D95"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B69:D69"/>
-    <mergeCell ref="A20:A27"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B81:D81"/>
+    <mergeCell ref="B74:C74"/>
   </mergeCells>
-  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="D6:D11 D13:D14 D16:D18 D20:D23 D25:D26 D60:D66 D68 D70:D72 D74:D76 D79:D80">
     <cfRule type="containsText" dxfId="15" priority="23" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D6)))</formula>
@@ -2481,17 +2497,15 @@
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.47244094488188981" right="0.15748031496062992" top="1.4566929133858268" bottom="0.43307086614173229" header="0.31496062992125984" footer="0.19685039370078741"/>
+  <pageMargins left="0.47244094488188981" right="0.15748031496062989" top="1.4566929133858271" bottom="0.43307086614173229" header="0.31496062992125978" footer="0.19685039370078741"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
-    <oddHeader>&amp;L&amp;"Arial,Gras"&amp;14Informaticien/-ne CFC&amp;"Arial,Normal"&amp;10
-Travail pratique individuel 2026 (TPI)&amp;R&amp;"Arial,Gras"&amp;14&amp;G</oddHeader>
-    <oddFooter>&amp;L&amp;8&amp;F&amp;R&amp;8Page &amp;P/&amp;N</oddFooter>
+    <oddHeader>&amp;L&amp;"Arial,Gras"&amp;14Informaticien/-ne CFC&amp;"Arial,Normal"&amp;10 Travail pratique individuel 2026 (TPI)&amp;R&amp;"Arial,Gras"&amp;14 &amp;G</oddHeader>
+    <oddFooter>&amp;L&amp;8 &amp;F&amp;R&amp;8 Page &amp;P/&amp;N</oddFooter>
   </headerFooter>
   <rowBreaks count="2" manualBreakCount="2">
     <brk id="50" max="16383" man="1"/>
     <brk id="96" max="3" man="1"/>
   </rowBreaks>
-  <legacyDrawingHF r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>